<commit_message>
refactor(doc) update project repport
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -5,10 +5,10 @@
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Downloads\TPI\TPI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E9F140C-37EC-479F-AD0A-A708CB777A4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CFB6D5D-6509-4A32-84AA-BA52B0E82140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$67</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$68</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="42">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -52,9 +52,6 @@
   </si>
   <si>
     <t>Experts </t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
   <si>
     <t>Chef.fe de Projet</t>
@@ -153,6 +150,33 @@
   </si>
   <si>
     <t>TOTAL :</t>
+  </si>
+  <si>
+    <t>90h</t>
+  </si>
+  <si>
+    <t>Nicolas Bordoën, Michael Wyssa</t>
+  </si>
+  <si>
+    <t>Travail pratique individuel (TPI)</t>
+  </si>
+  <si>
+    <t>Agora</t>
+  </si>
+  <si>
+    <t>J'ai rencontré un de mes deux expert avec on a pu discuter des modalité du TPI</t>
+  </si>
+  <si>
+    <t>Rapport</t>
+  </si>
+  <si>
+    <t>J'ai terminé la plannification je vais l'envoyer cet après midi aux experts</t>
+  </si>
+  <si>
+    <t>J'ai déjà commencé la rédaction du rapport</t>
+  </si>
+  <si>
+    <t>https://www.onlinegantt.com/#/gantt</t>
   </si>
 </sst>
 </file>
@@ -479,6 +503,41 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -491,41 +550,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
@@ -842,7 +866,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -858,74 +882,80 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="26"/>
+      <c r="B1" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="36"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="20"/>
+      <c r="E1" s="20" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="2" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="26"/>
+      <c r="B2" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="36"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="36"/>
+      <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="26"/>
-      <c r="D3" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="19"/>
+      <c r="E3" s="19" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="4" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="29"/>
+        <v>6</v>
+      </c>
+      <c r="B4" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="39"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="36">
+        <v>18</v>
+      </c>
+      <c r="B6" s="27">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -936,31 +966,35 @@
     </row>
     <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="31"/>
+        <v>19</v>
+      </c>
+      <c r="B7" s="28"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
-      <c r="D7" s="9"/>
+      <c r="D7" s="9" t="s">
+        <v>37</v>
+      </c>
       <c r="E7" s="8"/>
     </row>
     <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="31"/>
+        <v>20</v>
+      </c>
+      <c r="B8" s="28"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
       <c r="D8" s="9"/>
-      <c r="E8" s="8"/>
+      <c r="E8" s="8" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="9" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="31"/>
+        <v>20</v>
+      </c>
+      <c r="B9" s="28"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -969,9 +1003,9 @@
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="31"/>
+        <v>20</v>
+      </c>
+      <c r="B10" s="28"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -980,479 +1014,496 @@
       <c r="F10" s="24"/>
       <c r="G10" s="24"/>
     </row>
-    <row r="11" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="32"/>
+        <v>20</v>
+      </c>
+      <c r="B11" s="28"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
-      <c r="D11" s="11"/>
+      <c r="D11" s="11" t="s">
+        <v>39</v>
+      </c>
       <c r="E11" s="10"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="24"/>
     </row>
     <row r="12" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="33" t="str">
-        <f>INT(SUM(C6:C11)/60)&amp;"h"&amp;MOD(SUM(C6:C11),60)</f>
-        <v>2h10</v>
-      </c>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="35"/>
-    </row>
-    <row r="13" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-      <c r="B13" s="36"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="5"/>
+      <c r="A12" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="29"/>
+      <c r="C12" s="10">
+        <v>60</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="10"/>
+    </row>
+    <row r="13" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="30" t="str">
+        <f>INT(SUM(C6:C12)/60)&amp;"h"&amp;MOD(SUM(C6:C12),60)</f>
+        <v>3h10</v>
+      </c>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="32"/>
     </row>
     <row r="14" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="31"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="8"/>
-    </row>
-    <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="4"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="5"/>
+    </row>
+    <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7"/>
-      <c r="B15" s="31"/>
+      <c r="B15" s="28"/>
       <c r="C15" s="8"/>
       <c r="D15" s="9"/>
       <c r="E15" s="8"/>
-      <c r="G15" s="25"/>
-    </row>
-    <row r="16" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="7"/>
-      <c r="B16" s="31"/>
+      <c r="B16" s="28"/>
       <c r="C16" s="8"/>
       <c r="D16" s="9"/>
       <c r="E16" s="8"/>
-    </row>
-    <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="10"/>
-      <c r="B17" s="32"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="10"/>
+      <c r="G16" s="25"/>
+    </row>
+    <row r="17" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="7"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B18" s="33"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="35"/>
-    </row>
-    <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="4"/>
+      <c r="A18" s="10"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="10"/>
+    </row>
+    <row r="19" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="12" t="s">
+        <v>12</v>
+      </c>
       <c r="B19" s="30"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="5"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="32"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="B20" s="31"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="8"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="35"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="5"/>
     </row>
     <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
-      <c r="B21" s="31"/>
+      <c r="B21" s="28"/>
       <c r="C21" s="8"/>
       <c r="D21" s="9"/>
       <c r="E21" s="8"/>
     </row>
     <row r="22" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
-      <c r="B22" s="31"/>
+      <c r="B22" s="28"/>
       <c r="C22" s="8"/>
       <c r="D22" s="9"/>
       <c r="E22" s="8"/>
     </row>
-    <row r="23" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="10"/>
-      <c r="B23" s="32"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="10"/>
+    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="7"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="8"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B24" s="33"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="34"/>
-      <c r="E24" s="35"/>
-    </row>
-    <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4"/>
+      <c r="A24" s="10"/>
+      <c r="B24" s="29"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="10"/>
+    </row>
+    <row r="25" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="12" t="s">
+        <v>12</v>
+      </c>
       <c r="B25" s="30"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="5"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="32"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="7"/>
-      <c r="B26" s="31"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="8"/>
+      <c r="A26" s="4"/>
+      <c r="B26" s="35"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="5"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7"/>
-      <c r="B27" s="31"/>
+      <c r="B27" s="28"/>
       <c r="C27" s="8"/>
       <c r="D27" s="9"/>
       <c r="E27" s="8"/>
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
-      <c r="B28" s="31"/>
+      <c r="B28" s="28"/>
       <c r="C28" s="8"/>
       <c r="D28" s="9"/>
       <c r="E28" s="8"/>
     </row>
-    <row r="29" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="10"/>
-      <c r="B29" s="32"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="10"/>
+    <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="7"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="8"/>
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B30" s="33"/>
-      <c r="C30" s="34"/>
-      <c r="D30" s="34"/>
-      <c r="E30" s="35"/>
-    </row>
-    <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="13"/>
+      <c r="A30" s="10"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="10"/>
+    </row>
+    <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="12" t="s">
+        <v>12</v>
+      </c>
       <c r="B31" s="30"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="13"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="31"/>
+      <c r="E31" s="32"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="8"/>
-      <c r="B32" s="31"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="8"/>
+      <c r="A32" s="13"/>
+      <c r="B32" s="35"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="13"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8"/>
-      <c r="B33" s="31"/>
+      <c r="B33" s="28"/>
       <c r="C33" s="8"/>
       <c r="D33" s="9"/>
       <c r="E33" s="8"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8"/>
-      <c r="B34" s="31"/>
+      <c r="B34" s="28"/>
       <c r="C34" s="8"/>
       <c r="D34" s="9"/>
       <c r="E34" s="8"/>
     </row>
-    <row r="35" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8"/>
-      <c r="B35" s="32"/>
+      <c r="B35" s="28"/>
       <c r="C35" s="8"/>
       <c r="D35" s="9"/>
       <c r="E35" s="8"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B36" s="33"/>
-      <c r="C36" s="34"/>
-      <c r="D36" s="34"/>
-      <c r="E36" s="35"/>
-    </row>
-    <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="4"/>
-      <c r="B37" s="36"/>
-      <c r="C37" s="5"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="5"/>
+      <c r="A36" s="8"/>
+      <c r="B36" s="29"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="8"/>
+    </row>
+    <row r="37" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B37" s="30"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="31"/>
+      <c r="E37" s="32"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="7"/>
-      <c r="B38" s="31"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="8"/>
+      <c r="A38" s="4"/>
+      <c r="B38" s="27"/>
+      <c r="C38" s="5"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="5"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="7"/>
-      <c r="B39" s="31"/>
+      <c r="B39" s="28"/>
       <c r="C39" s="8"/>
       <c r="D39" s="9"/>
       <c r="E39" s="8"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="7"/>
-      <c r="B40" s="31"/>
+      <c r="B40" s="28"/>
       <c r="C40" s="8"/>
       <c r="D40" s="9"/>
       <c r="E40" s="8"/>
     </row>
-    <row r="41" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="10"/>
-      <c r="B41" s="32"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="11"/>
-      <c r="E41" s="10"/>
+    <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="7"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="8"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B42" s="33"/>
-      <c r="C42" s="34"/>
-      <c r="D42" s="34"/>
-      <c r="E42" s="35"/>
-    </row>
-    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="4"/>
+      <c r="A42" s="10"/>
+      <c r="B42" s="29"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="10"/>
+    </row>
+    <row r="43" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="12" t="s">
+        <v>12</v>
+      </c>
       <c r="B43" s="30"/>
-      <c r="C43" s="5"/>
-      <c r="D43" s="6"/>
-      <c r="E43" s="5"/>
+      <c r="C43" s="31"/>
+      <c r="D43" s="31"/>
+      <c r="E43" s="32"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="7"/>
-      <c r="B44" s="31"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="8"/>
+      <c r="A44" s="4"/>
+      <c r="B44" s="35"/>
+      <c r="C44" s="5"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="5"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="7"/>
-      <c r="B45" s="31"/>
+      <c r="B45" s="28"/>
       <c r="C45" s="8"/>
       <c r="D45" s="9"/>
       <c r="E45" s="8"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="7"/>
-      <c r="B46" s="31"/>
+      <c r="B46" s="28"/>
       <c r="C46" s="8"/>
       <c r="D46" s="9"/>
       <c r="E46" s="8"/>
     </row>
-    <row r="47" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="10"/>
-      <c r="B47" s="32"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="10"/>
+    <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="7"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="8"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B48" s="33"/>
-      <c r="C48" s="34"/>
-      <c r="D48" s="34"/>
-      <c r="E48" s="35"/>
-    </row>
-    <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="4"/>
+      <c r="A48" s="10"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="11"/>
+      <c r="E48" s="10"/>
+    </row>
+    <row r="49" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="12" t="s">
+        <v>12</v>
+      </c>
       <c r="B49" s="30"/>
-      <c r="C49" s="5"/>
-      <c r="D49" s="6"/>
-      <c r="E49" s="5"/>
+      <c r="C49" s="31"/>
+      <c r="D49" s="31"/>
+      <c r="E49" s="32"/>
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="7"/>
-      <c r="B50" s="31"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="8"/>
+      <c r="A50" s="4"/>
+      <c r="B50" s="35"/>
+      <c r="C50" s="5"/>
+      <c r="D50" s="6"/>
+      <c r="E50" s="5"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
-      <c r="B51" s="31"/>
+      <c r="B51" s="28"/>
       <c r="C51" s="8"/>
       <c r="D51" s="9"/>
       <c r="E51" s="8"/>
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="7"/>
-      <c r="B52" s="31"/>
+      <c r="B52" s="28"/>
       <c r="C52" s="8"/>
       <c r="D52" s="9"/>
       <c r="E52" s="8"/>
     </row>
-    <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="10"/>
-      <c r="B53" s="32"/>
-      <c r="C53" s="10"/>
-      <c r="D53" s="11"/>
-      <c r="E53" s="10"/>
+    <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="7"/>
+      <c r="B53" s="28"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="8"/>
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B54" s="33"/>
-      <c r="C54" s="34"/>
-      <c r="D54" s="34"/>
-      <c r="E54" s="35"/>
-    </row>
-    <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="4"/>
+      <c r="A54" s="10"/>
+      <c r="B54" s="29"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="10"/>
+    </row>
+    <row r="55" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="12" t="s">
+        <v>12</v>
+      </c>
       <c r="B55" s="30"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="6"/>
-      <c r="E55" s="5"/>
+      <c r="C55" s="31"/>
+      <c r="D55" s="31"/>
+      <c r="E55" s="32"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="7"/>
-      <c r="B56" s="31"/>
-      <c r="C56" s="8"/>
-      <c r="D56" s="9"/>
-      <c r="E56" s="8"/>
+      <c r="A56" s="4"/>
+      <c r="B56" s="35"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="5"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="31"/>
+      <c r="B57" s="28"/>
       <c r="C57" s="8"/>
       <c r="D57" s="9"/>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="31"/>
+      <c r="B58" s="28"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
-    <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="10"/>
-      <c r="B59" s="32"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="11"/>
-      <c r="E59" s="10"/>
+    <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="7"/>
+      <c r="B59" s="28"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="8"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B60" s="33"/>
-      <c r="C60" s="34"/>
-      <c r="D60" s="34"/>
-      <c r="E60" s="35"/>
-    </row>
-    <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="13"/>
+      <c r="A60" s="10"/>
+      <c r="B60" s="29"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="11"/>
+      <c r="E60" s="10"/>
+    </row>
+    <row r="61" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="12" t="s">
+        <v>12</v>
+      </c>
       <c r="B61" s="30"/>
-      <c r="C61" s="13"/>
-      <c r="D61" s="14"/>
-      <c r="E61" s="13"/>
+      <c r="C61" s="31"/>
+      <c r="D61" s="31"/>
+      <c r="E61" s="32"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="8"/>
-      <c r="B62" s="31"/>
-      <c r="C62" s="8"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="8"/>
+      <c r="A62" s="13"/>
+      <c r="B62" s="35"/>
+      <c r="C62" s="13"/>
+      <c r="D62" s="14"/>
+      <c r="E62" s="13"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="8"/>
-      <c r="B63" s="31"/>
+      <c r="B63" s="28"/>
       <c r="C63" s="8"/>
       <c r="D63" s="9"/>
       <c r="E63" s="8"/>
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="8"/>
-      <c r="B64" s="31"/>
+      <c r="B64" s="28"/>
       <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
-    <row r="65" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="8"/>
-      <c r="B65" s="32"/>
+      <c r="B65" s="28"/>
       <c r="C65" s="8"/>
       <c r="D65" s="9"/>
       <c r="E65" s="8"/>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="12" t="s">
+      <c r="A66" s="8"/>
+      <c r="B66" s="29"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="9"/>
+      <c r="E66" s="8"/>
+    </row>
+    <row r="67" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B67" s="30"/>
+      <c r="C67" s="31"/>
+      <c r="D67" s="31"/>
+      <c r="E67" s="32"/>
+    </row>
+    <row r="68" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="B66" s="33"/>
-      <c r="C66" s="34"/>
-      <c r="D66" s="34"/>
-      <c r="E66" s="35"/>
-    </row>
-    <row r="67" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="37" t="s">
+      <c r="B68" s="34"/>
+      <c r="C68" s="15">
+        <f>MROUND(SUM(C6:C67) /60,0.2)</f>
+        <v>3.2</v>
+      </c>
+      <c r="D68" s="16"/>
+      <c r="E68" s="17"/>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B67" s="38"/>
-      <c r="C67" s="15">
-        <f>MROUND(SUM(C6:C66) /60,0.2)</f>
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="D67" s="16"/>
-      <c r="E67" s="17"/>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="18" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="18"/>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B66:E66"/>
-    <mergeCell ref="A67:B67"/>
-    <mergeCell ref="B43:B47"/>
-    <mergeCell ref="B48:E48"/>
-    <mergeCell ref="B49:B53"/>
-    <mergeCell ref="B54:E54"/>
-    <mergeCell ref="B55:B59"/>
-    <mergeCell ref="B60:E60"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B61:B65"/>
-    <mergeCell ref="B42:E42"/>
-    <mergeCell ref="B6:B11"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B13:B17"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B19:B23"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B25:B29"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B31:B35"/>
-    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="B6:B12"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B20:B24"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B26:B30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B38:B42"/>
+    <mergeCell ref="B67:E67"/>
+    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="B44:B48"/>
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="B56:B60"/>
+    <mergeCell ref="B61:E61"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C55:C59 C49:C53 C37:C41 C43:C47 C19:C23 B6 C13:C17 C25:C29 C31:C35 C61:C65 C6:C11" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C56:C60 C50:C54 C38:C42 C44:C48 C20:C24 B6 C14:C18 C26:C30 C32:C36 C62:C66 C6:C12" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B13:B17 B19:B23 B25:B29 B31:B35 B37:B41 B43:B47 B49:B53 B55:B59 B61:B65" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B14:B18 B20:B24 B26:B30 B32:B36 B38:B42 B44:B48 B50:B54 B56:B60 B62:B66" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -1478,149 +1529,149 @@
   <sheetData>
     <row r="5" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
         <v>22</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>23</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>24</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>25</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>26</v>
-      </c>
-      <c r="I5" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="6" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="39">
+        <v>27</v>
+      </c>
+      <c r="D6" s="26">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E6" s="39">
+      <c r="E6" s="26">
         <v>0.47569444444444442</v>
       </c>
-      <c r="F6" s="39">
+      <c r="F6" s="26">
         <v>0.51388888888888884</v>
       </c>
-      <c r="G6" s="39">
+      <c r="G6" s="26">
         <v>0.61458333333333337</v>
       </c>
-      <c r="H6" s="39">
+      <c r="H6" s="26">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="I6" s="39">
+      <c r="I6" s="26">
         <v>0.22222222222222221</v>
       </c>
     </row>
     <row r="7" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" s="39">
+        <v>28</v>
+      </c>
+      <c r="D7" s="26">
         <v>0</v>
       </c>
-      <c r="E7" s="39">
+      <c r="E7" s="26">
         <v>0</v>
       </c>
-      <c r="F7" s="39">
+      <c r="F7" s="26">
         <v>0</v>
       </c>
-      <c r="G7" s="39">
+      <c r="G7" s="26">
         <v>0</v>
       </c>
-      <c r="H7" s="39">
+      <c r="H7" s="26">
         <v>0</v>
       </c>
-      <c r="I7" s="39">
+      <c r="I7" s="26">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" s="39">
+        <v>29</v>
+      </c>
+      <c r="D8" s="26">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E8" s="39">
+      <c r="E8" s="26">
         <v>0.51041666666666663</v>
       </c>
-      <c r="F8" s="39">
+      <c r="F8" s="26">
         <v>0.54861111111111116</v>
       </c>
-      <c r="G8" s="39">
+      <c r="G8" s="26">
         <v>0.69097222222222221</v>
       </c>
-      <c r="H8" s="39">
+      <c r="H8" s="26">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="I8" s="39">
+      <c r="I8" s="26">
         <v>0.2986111111111111</v>
       </c>
     </row>
     <row r="9" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D9" s="39">
+        <v>30</v>
+      </c>
+      <c r="D9" s="26">
         <v>0</v>
       </c>
-      <c r="E9" s="39">
+      <c r="E9" s="26">
         <v>0</v>
       </c>
-      <c r="F9" s="39">
+      <c r="F9" s="26">
         <v>0.54861111111111116</v>
       </c>
-      <c r="G9" s="39">
+      <c r="G9" s="26">
         <v>0.69097222222222221</v>
       </c>
-      <c r="H9" s="39">
+      <c r="H9" s="26">
         <v>1.0416666666666666E-2</v>
       </c>
-      <c r="I9" s="39">
+      <c r="I9" s="26">
         <v>0.13194444444444445</v>
       </c>
     </row>
     <row r="10" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" s="39">
+        <v>31</v>
+      </c>
+      <c r="D10" s="26">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E10" s="39">
+      <c r="E10" s="26">
         <v>0.51041666666666663</v>
       </c>
-      <c r="F10" s="39">
+      <c r="F10" s="26">
         <v>0.54861111111111116</v>
       </c>
-      <c r="G10" s="39">
+      <c r="G10" s="26">
         <v>0.69097222222222221</v>
       </c>
-      <c r="H10" s="39">
+      <c r="H10" s="26">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="I10" s="39">
+      <c r="I10" s="26">
         <v>0.2986111111111111</v>
       </c>
     </row>
     <row r="12" spans="3:9" x14ac:dyDescent="0.25">
       <c r="H12" t="s">
-        <v>33</v>
-      </c>
-      <c r="I12" s="39">
+        <v>32</v>
+      </c>
+      <c r="I12" s="26">
         <v>0.95138888888888884</v>
       </c>
     </row>
     <row r="19" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E19" s="39">
+      <c r="E19" s="26">
         <f>E6-D6-H6/2</f>
         <v>0.13194444444444445</v>
       </c>
@@ -1631,6 +1682,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -1792,22 +1858,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1823,21 +1891,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(app): create next project with prisma
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CFB6D5D-6509-4A32-84AA-BA52B0E82140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65E7DCF2-6A9B-461B-848F-084F43F32DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$68</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$69</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="43">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -177,6 +177,9 @@
   </si>
   <si>
     <t>https://www.onlinegantt.com/#/gantt</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> J'ai un peu avancé sur la rédaction du rapport où j'ai notament fait le contexte ma méthode de travail et les risques j'ai utilisé l'IA afin de corrigé les fautes reformuler des tournure de phrase </t>
   </si>
 </sst>
 </file>
@@ -504,51 +507,51 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -866,7 +869,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -882,10 +885,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="36"/>
+      <c r="C1" s="27"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -897,10 +900,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="36"/>
+      <c r="C2" s="27"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -912,10 +915,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="36"/>
+      <c r="C3" s="27"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -927,12 +930,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="39"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -955,7 +958,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="27">
+      <c r="B6" s="37">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -968,7 +971,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="28"/>
+      <c r="B7" s="32"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -981,7 +984,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="28"/>
+      <c r="B8" s="32"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -994,7 +997,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="28"/>
+      <c r="B9" s="32"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1005,7 +1008,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="28"/>
+      <c r="B10" s="32"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1018,7 +1021,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="28"/>
+      <c r="B11" s="32"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1029,11 +1032,11 @@
       <c r="F11" s="24"/>
       <c r="G11" s="24"/>
     </row>
-    <row r="12" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="29"/>
+      <c r="B12" s="32"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1041,469 +1044,484 @@
         <v>40</v>
       </c>
       <c r="E12" s="10"/>
-    </row>
-    <row r="13" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="12" t="s">
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+    </row>
+    <row r="13" spans="1:7" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="33"/>
+      <c r="C13" s="10">
+        <v>40</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="10"/>
+    </row>
+    <row r="14" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="30" t="str">
-        <f>INT(SUM(C6:C12)/60)&amp;"h"&amp;MOD(SUM(C6:C12),60)</f>
-        <v>3h10</v>
-      </c>
-      <c r="C13" s="31"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="32"/>
-    </row>
-    <row r="14" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
-      <c r="B14" s="27"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="5"/>
+      <c r="B14" s="34" t="str">
+        <f>INT(SUM(C6:C13)/60)&amp;"h"&amp;MOD(SUM(C6:C13),60)</f>
+        <v>3h50</v>
+      </c>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="36"/>
     </row>
     <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="B15" s="28"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="8"/>
-    </row>
-    <row r="16" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="4"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="5"/>
+    </row>
+    <row r="16" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
-      <c r="B16" s="28"/>
+      <c r="B16" s="32"/>
       <c r="C16" s="8"/>
       <c r="D16" s="9"/>
       <c r="E16" s="8"/>
-      <c r="G16" s="25"/>
-    </row>
-    <row r="17" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="7"/>
-      <c r="B17" s="28"/>
+      <c r="B17" s="32"/>
       <c r="C17" s="8"/>
       <c r="D17" s="9"/>
       <c r="E17" s="8"/>
-    </row>
-    <row r="18" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="10"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="10"/>
-    </row>
-    <row r="19" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="12" t="s">
+      <c r="G17" s="25"/>
+    </row>
+    <row r="18" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="7"/>
+      <c r="B18" s="32"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="8"/>
+    </row>
+    <row r="19" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="10"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="10"/>
+    </row>
+    <row r="20" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="30"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="32"/>
-    </row>
-    <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="4"/>
-      <c r="B20" s="35"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="5"/>
-    </row>
-    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="28"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="8"/>
-    </row>
-    <row r="22" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="34"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="36"/>
+    </row>
+    <row r="21" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="4"/>
+      <c r="B21" s="31"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="5"/>
+    </row>
+    <row r="22" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
-      <c r="B22" s="28"/>
+      <c r="B22" s="32"/>
       <c r="C22" s="8"/>
       <c r="D22" s="9"/>
       <c r="E22" s="8"/>
     </row>
-    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
-      <c r="B23" s="28"/>
+      <c r="B23" s="32"/>
       <c r="C23" s="8"/>
       <c r="D23" s="9"/>
       <c r="E23" s="8"/>
     </row>
-    <row r="24" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="10"/>
-      <c r="B24" s="29"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="10"/>
-    </row>
-    <row r="25" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
+    <row r="24" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="7"/>
+      <c r="B24" s="32"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="8"/>
+    </row>
+    <row r="25" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="10"/>
+      <c r="B25" s="33"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="10"/>
+    </row>
+    <row r="26" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="30"/>
-      <c r="C25" s="31"/>
-      <c r="D25" s="31"/>
-      <c r="E25" s="32"/>
-    </row>
-    <row r="26" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="4"/>
-      <c r="B26" s="35"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="5"/>
-    </row>
-    <row r="27" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="7"/>
-      <c r="B27" s="28"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="8"/>
-    </row>
-    <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="34"/>
+      <c r="C26" s="35"/>
+      <c r="D26" s="35"/>
+      <c r="E26" s="36"/>
+    </row>
+    <row r="27" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="4"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="5"/>
+    </row>
+    <row r="28" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
-      <c r="B28" s="28"/>
+      <c r="B28" s="32"/>
       <c r="C28" s="8"/>
       <c r="D28" s="9"/>
       <c r="E28" s="8"/>
     </row>
-    <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
-      <c r="B29" s="28"/>
+      <c r="B29" s="32"/>
       <c r="C29" s="8"/>
       <c r="D29" s="9"/>
       <c r="E29" s="8"/>
     </row>
-    <row r="30" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="10"/>
-      <c r="B30" s="29"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="10"/>
-    </row>
-    <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="12" t="s">
+    <row r="30" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="7"/>
+      <c r="B30" s="32"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="8"/>
+    </row>
+    <row r="31" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="10"/>
+      <c r="B31" s="33"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="10"/>
+    </row>
+    <row r="32" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B31" s="30"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
-      <c r="E31" s="32"/>
-    </row>
-    <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="13"/>
-      <c r="B32" s="35"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="13"/>
+      <c r="B32" s="34"/>
+      <c r="C32" s="35"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="36"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="8"/>
-      <c r="B33" s="28"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="8"/>
+      <c r="A33" s="13"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="13"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8"/>
-      <c r="B34" s="28"/>
+      <c r="B34" s="32"/>
       <c r="C34" s="8"/>
       <c r="D34" s="9"/>
       <c r="E34" s="8"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8"/>
-      <c r="B35" s="28"/>
+      <c r="B35" s="32"/>
       <c r="C35" s="8"/>
       <c r="D35" s="9"/>
       <c r="E35" s="8"/>
     </row>
-    <row r="36" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8"/>
-      <c r="B36" s="29"/>
+      <c r="B36" s="32"/>
       <c r="C36" s="8"/>
       <c r="D36" s="9"/>
       <c r="E36" s="8"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="12" t="s">
+      <c r="A37" s="8"/>
+      <c r="B37" s="33"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="8"/>
+    </row>
+    <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B37" s="30"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="31"/>
-      <c r="E37" s="32"/>
-    </row>
-    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="4"/>
-      <c r="B38" s="27"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="6"/>
-      <c r="E38" s="5"/>
+      <c r="B38" s="34"/>
+      <c r="C38" s="35"/>
+      <c r="D38" s="35"/>
+      <c r="E38" s="36"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="7"/>
-      <c r="B39" s="28"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="8"/>
+      <c r="A39" s="4"/>
+      <c r="B39" s="37"/>
+      <c r="C39" s="5"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="5"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="7"/>
-      <c r="B40" s="28"/>
+      <c r="B40" s="32"/>
       <c r="C40" s="8"/>
       <c r="D40" s="9"/>
       <c r="E40" s="8"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="7"/>
-      <c r="B41" s="28"/>
+      <c r="B41" s="32"/>
       <c r="C41" s="8"/>
       <c r="D41" s="9"/>
       <c r="E41" s="8"/>
     </row>
-    <row r="42" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="10"/>
-      <c r="B42" s="29"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="10"/>
+    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="7"/>
+      <c r="B42" s="32"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="8"/>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="12" t="s">
+      <c r="A43" s="10"/>
+      <c r="B43" s="33"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="10"/>
+    </row>
+    <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B43" s="30"/>
-      <c r="C43" s="31"/>
-      <c r="D43" s="31"/>
-      <c r="E43" s="32"/>
-    </row>
-    <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="4"/>
-      <c r="B44" s="35"/>
-      <c r="C44" s="5"/>
-      <c r="D44" s="6"/>
-      <c r="E44" s="5"/>
+      <c r="B44" s="34"/>
+      <c r="C44" s="35"/>
+      <c r="D44" s="35"/>
+      <c r="E44" s="36"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="7"/>
-      <c r="B45" s="28"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="8"/>
+      <c r="A45" s="4"/>
+      <c r="B45" s="31"/>
+      <c r="C45" s="5"/>
+      <c r="D45" s="6"/>
+      <c r="E45" s="5"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="7"/>
-      <c r="B46" s="28"/>
+      <c r="B46" s="32"/>
       <c r="C46" s="8"/>
       <c r="D46" s="9"/>
       <c r="E46" s="8"/>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7"/>
-      <c r="B47" s="28"/>
+      <c r="B47" s="32"/>
       <c r="C47" s="8"/>
       <c r="D47" s="9"/>
       <c r="E47" s="8"/>
     </row>
-    <row r="48" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="10"/>
-      <c r="B48" s="29"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="10"/>
+    <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="7"/>
+      <c r="B48" s="32"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="8"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="12" t="s">
+      <c r="A49" s="10"/>
+      <c r="B49" s="33"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="10"/>
+    </row>
+    <row r="50" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B49" s="30"/>
-      <c r="C49" s="31"/>
-      <c r="D49" s="31"/>
-      <c r="E49" s="32"/>
-    </row>
-    <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="4"/>
-      <c r="B50" s="35"/>
-      <c r="C50" s="5"/>
-      <c r="D50" s="6"/>
-      <c r="E50" s="5"/>
+      <c r="B50" s="34"/>
+      <c r="C50" s="35"/>
+      <c r="D50" s="35"/>
+      <c r="E50" s="36"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="7"/>
-      <c r="B51" s="28"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="9"/>
-      <c r="E51" s="8"/>
+      <c r="A51" s="4"/>
+      <c r="B51" s="31"/>
+      <c r="C51" s="5"/>
+      <c r="D51" s="6"/>
+      <c r="E51" s="5"/>
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="7"/>
-      <c r="B52" s="28"/>
+      <c r="B52" s="32"/>
       <c r="C52" s="8"/>
       <c r="D52" s="9"/>
       <c r="E52" s="8"/>
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="7"/>
-      <c r="B53" s="28"/>
+      <c r="B53" s="32"/>
       <c r="C53" s="8"/>
       <c r="D53" s="9"/>
       <c r="E53" s="8"/>
     </row>
-    <row r="54" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="10"/>
-      <c r="B54" s="29"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="10"/>
+    <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="7"/>
+      <c r="B54" s="32"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="8"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="12" t="s">
+      <c r="A55" s="10"/>
+      <c r="B55" s="33"/>
+      <c r="C55" s="10"/>
+      <c r="D55" s="11"/>
+      <c r="E55" s="10"/>
+    </row>
+    <row r="56" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B55" s="30"/>
-      <c r="C55" s="31"/>
-      <c r="D55" s="31"/>
-      <c r="E55" s="32"/>
-    </row>
-    <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="4"/>
-      <c r="B56" s="35"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="6"/>
-      <c r="E56" s="5"/>
+      <c r="B56" s="34"/>
+      <c r="C56" s="35"/>
+      <c r="D56" s="35"/>
+      <c r="E56" s="36"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="7"/>
-      <c r="B57" s="28"/>
-      <c r="C57" s="8"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="8"/>
+      <c r="A57" s="4"/>
+      <c r="B57" s="31"/>
+      <c r="C57" s="5"/>
+      <c r="D57" s="6"/>
+      <c r="E57" s="5"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="28"/>
+      <c r="B58" s="32"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="7"/>
-      <c r="B59" s="28"/>
+      <c r="B59" s="32"/>
       <c r="C59" s="8"/>
       <c r="D59" s="9"/>
       <c r="E59" s="8"/>
     </row>
-    <row r="60" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="10"/>
-      <c r="B60" s="29"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="11"/>
-      <c r="E60" s="10"/>
+    <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="7"/>
+      <c r="B60" s="32"/>
+      <c r="C60" s="8"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="8"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="12" t="s">
+      <c r="A61" s="10"/>
+      <c r="B61" s="33"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="11"/>
+      <c r="E61" s="10"/>
+    </row>
+    <row r="62" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B61" s="30"/>
-      <c r="C61" s="31"/>
-      <c r="D61" s="31"/>
-      <c r="E61" s="32"/>
-    </row>
-    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="13"/>
-      <c r="B62" s="35"/>
-      <c r="C62" s="13"/>
-      <c r="D62" s="14"/>
-      <c r="E62" s="13"/>
+      <c r="B62" s="34"/>
+      <c r="C62" s="35"/>
+      <c r="D62" s="35"/>
+      <c r="E62" s="36"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="8"/>
-      <c r="B63" s="28"/>
-      <c r="C63" s="8"/>
-      <c r="D63" s="9"/>
-      <c r="E63" s="8"/>
+      <c r="A63" s="13"/>
+      <c r="B63" s="31"/>
+      <c r="C63" s="13"/>
+      <c r="D63" s="14"/>
+      <c r="E63" s="13"/>
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="8"/>
-      <c r="B64" s="28"/>
+      <c r="B64" s="32"/>
       <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="8"/>
-      <c r="B65" s="28"/>
+      <c r="B65" s="32"/>
       <c r="C65" s="8"/>
       <c r="D65" s="9"/>
       <c r="E65" s="8"/>
     </row>
-    <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="8"/>
-      <c r="B66" s="29"/>
+      <c r="B66" s="32"/>
       <c r="C66" s="8"/>
       <c r="D66" s="9"/>
       <c r="E66" s="8"/>
     </row>
     <row r="67" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="12" t="s">
+      <c r="A67" s="8"/>
+      <c r="B67" s="33"/>
+      <c r="C67" s="8"/>
+      <c r="D67" s="9"/>
+      <c r="E67" s="8"/>
+    </row>
+    <row r="68" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B67" s="30"/>
-      <c r="C67" s="31"/>
-      <c r="D67" s="31"/>
-      <c r="E67" s="32"/>
-    </row>
-    <row r="68" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="33" t="s">
+      <c r="B68" s="34"/>
+      <c r="C68" s="35"/>
+      <c r="D68" s="35"/>
+      <c r="E68" s="36"/>
+    </row>
+    <row r="69" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="B68" s="34"/>
-      <c r="C68" s="15">
-        <f>MROUND(SUM(C6:C67) /60,0.2)</f>
-        <v>3.2</v>
-      </c>
-      <c r="D68" s="16"/>
-      <c r="E68" s="17"/>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="18" t="s">
+      <c r="B69" s="39"/>
+      <c r="C69" s="15">
+        <f>MROUND(SUM(C6:C68) /60,0.2)</f>
+        <v>3.8000000000000003</v>
+      </c>
+      <c r="D69" s="16"/>
+      <c r="E69" s="17"/>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="18"/>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B39:B43"/>
+    <mergeCell ref="B68:E68"/>
+    <mergeCell ref="A69:B69"/>
+    <mergeCell ref="B45:B49"/>
+    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B51:B55"/>
+    <mergeCell ref="B56:E56"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="B62:E62"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="B43:E43"/>
-    <mergeCell ref="B6:B12"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="B20:B24"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B26:B30"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="B38:B42"/>
-    <mergeCell ref="B67:E67"/>
-    <mergeCell ref="A68:B68"/>
-    <mergeCell ref="B44:B48"/>
-    <mergeCell ref="B49:E49"/>
-    <mergeCell ref="B50:B54"/>
-    <mergeCell ref="B55:E55"/>
-    <mergeCell ref="B56:B60"/>
-    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="B63:B67"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="B6:B13"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B15:B19"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="B21:B25"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B33:B37"/>
+    <mergeCell ref="B38:E38"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C56:C60 C50:C54 C38:C42 C44:C48 C20:C24 B6 C14:C18 C26:C30 C32:C36 C62:C66 C6:C12" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C57:C61 C51:C55 C39:C43 C45:C49 C21:C25 B6 C15:C19 C27:C31 C33:C37 C63:C67 C6:C13" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B14:B18 B20:B24 B26:B30 B32:B36 B38:B42 B44:B48 B50:B54 B56:B60 B62:B66" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B15:B19 B21:B25 B27:B31 B33:B37 B39:B43 B45:B49 B51:B55 B57:B61 B63:B67" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -1682,18 +1700,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1859,18 +1877,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
refactor, feat(doc): update JDT and add maquettes basse
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65E7DCF2-6A9B-461B-848F-084F43F32DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D631A27-029D-4D9E-84B3-803093B451FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$69</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$73</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="48">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -180,6 +180,21 @@
   </si>
   <si>
     <t xml:space="preserve"> J'ai un peu avancé sur la rédaction du rapport où j'ai notament fait le contexte ma méthode de travail et les risques j'ai utilisé l'IA afin de corrigé les fautes reformuler des tournure de phrase </t>
+  </si>
+  <si>
+    <t>Discussion</t>
+  </si>
+  <si>
+    <t>J'avais quelques question concernant le CRON j'en ai donc discuté avec M. Melly et on a aussi discuté si le stattus En cours, Terminé/ Echouée concernait la campagne ou juste le mail et on a décidé que ca touchais uniquement la campagne</t>
+  </si>
+  <si>
+    <t>Maquettes</t>
+  </si>
+  <si>
+    <t>J'ai commencé les maquettes basse fidélité en me basant sur une ancienne app que j'ai faite afin de gagner du temps</t>
+  </si>
+  <si>
+    <t>J'ai continué mes maquettes</t>
   </si>
 </sst>
 </file>
@@ -507,51 +522,51 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -869,7 +884,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -885,10 +900,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="27"/>
+      <c r="C1" s="36"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -900,10 +915,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="27"/>
+      <c r="C2" s="36"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -915,10 +930,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="27"/>
+      <c r="C3" s="36"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -930,12 +945,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="30"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="39"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -958,7 +973,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="37">
+      <c r="B6" s="27">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -971,7 +986,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="32"/>
+      <c r="B7" s="28"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -984,7 +999,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="32"/>
+      <c r="B8" s="28"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -997,7 +1012,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="32"/>
+      <c r="B9" s="28"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1008,7 +1023,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="32"/>
+      <c r="B10" s="28"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1021,7 +1036,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="32"/>
+      <c r="B11" s="28"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1036,7 +1051,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="32"/>
+      <c r="B12" s="28"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1047,481 +1062,535 @@
       <c r="F12" s="24"/>
       <c r="G12" s="24"/>
     </row>
-    <row r="13" spans="1:7" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="28"/>
+      <c r="C13" s="10">
+        <v>10</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="10"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+    </row>
+    <row r="14" spans="1:7" ht="27" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="28"/>
+      <c r="C14" s="10">
+        <v>60</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E14" s="10"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+    </row>
+    <row r="15" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="33"/>
-      <c r="C13" s="10">
+      <c r="B15" s="28"/>
+      <c r="C15" s="10">
         <v>40</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D15" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="E13" s="10"/>
-    </row>
-    <row r="14" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="12" t="s">
+      <c r="E15" s="10"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="28"/>
+      <c r="C16" s="10">
+        <v>20</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E16" s="10"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+    </row>
+    <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="7"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="10"/>
+    </row>
+    <row r="18" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="34" t="str">
-        <f>INT(SUM(C6:C13)/60)&amp;"h"&amp;MOD(SUM(C6:C13),60)</f>
-        <v>3h50</v>
-      </c>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="36"/>
-    </row>
-    <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4"/>
-      <c r="B15" s="37"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="5"/>
-    </row>
-    <row r="16" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="32"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="8"/>
-    </row>
-    <row r="17" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="7"/>
-      <c r="B17" s="32"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="8"/>
-      <c r="G17" s="25"/>
-    </row>
-    <row r="18" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="32"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="8"/>
-    </row>
-    <row r="19" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="10"/>
-      <c r="B19" s="33"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="10"/>
-    </row>
-    <row r="20" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B20" s="34"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="35"/>
-      <c r="E20" s="36"/>
-    </row>
-    <row r="21" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="4"/>
-      <c r="B21" s="31"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="5"/>
+      <c r="B18" s="30" t="str">
+        <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
+        <v>5h20</v>
+      </c>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="32"/>
+    </row>
+    <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="5"/>
+    </row>
+    <row r="20" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="7"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="8"/>
+    </row>
+    <row r="21" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="7"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="8"/>
+      <c r="G21" s="25"/>
     </row>
     <row r="22" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
-      <c r="B22" s="32"/>
+      <c r="B22" s="28"/>
       <c r="C22" s="8"/>
       <c r="D22" s="9"/>
       <c r="E22" s="8"/>
     </row>
-    <row r="23" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="B23" s="32"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="8"/>
-    </row>
-    <row r="24" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="7"/>
-      <c r="B24" s="32"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="8"/>
-    </row>
-    <row r="25" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="10"/>
-      <c r="B25" s="33"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="10"/>
-    </row>
-    <row r="26" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="12" t="s">
+    <row r="23" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="10"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="10"/>
+    </row>
+    <row r="24" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B26" s="34"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="35"/>
-      <c r="E26" s="36"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="32"/>
+    </row>
+    <row r="25" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="4"/>
+      <c r="B25" s="35"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="5"/>
+    </row>
+    <row r="26" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="7"/>
+      <c r="B26" s="28"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="8"/>
     </row>
     <row r="27" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="4"/>
-      <c r="B27" s="31"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="5"/>
+      <c r="A27" s="7"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="8"/>
     </row>
     <row r="28" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
-      <c r="B28" s="32"/>
+      <c r="B28" s="28"/>
       <c r="C28" s="8"/>
       <c r="D28" s="9"/>
       <c r="E28" s="8"/>
     </row>
-    <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="7"/>
-      <c r="B29" s="32"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="8"/>
-    </row>
-    <row r="30" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="7"/>
-      <c r="B30" s="32"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="8"/>
-    </row>
-    <row r="31" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="10"/>
-      <c r="B31" s="33"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="10"/>
-    </row>
-    <row r="32" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="12" t="s">
+    <row r="29" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="10"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="10"/>
+    </row>
+    <row r="30" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B32" s="34"/>
-      <c r="C32" s="35"/>
-      <c r="D32" s="35"/>
-      <c r="E32" s="36"/>
+      <c r="B30" s="30"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="32"/>
+    </row>
+    <row r="31" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="4"/>
+      <c r="B31" s="35"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="5"/>
+    </row>
+    <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="7"/>
+      <c r="B32" s="28"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="13"/>
-      <c r="B33" s="31"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="13"/>
+      <c r="A33" s="7"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="8"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="8"/>
-      <c r="B34" s="32"/>
+      <c r="A34" s="7"/>
+      <c r="B34" s="28"/>
       <c r="C34" s="8"/>
       <c r="D34" s="9"/>
       <c r="E34" s="8"/>
     </row>
-    <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="8"/>
-      <c r="B35" s="32"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="8"/>
-    </row>
-    <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="8"/>
-      <c r="B36" s="32"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="8"/>
-    </row>
-    <row r="37" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="8"/>
-      <c r="B37" s="33"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="8"/>
-    </row>
-    <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="12" t="s">
+    <row r="35" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="10"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="10"/>
+    </row>
+    <row r="36" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="34"/>
-      <c r="C38" s="35"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="36"/>
+      <c r="B36" s="30"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="31"/>
+      <c r="E36" s="32"/>
+    </row>
+    <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="13"/>
+      <c r="B37" s="35"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="13"/>
+    </row>
+    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="8"/>
+      <c r="B38" s="28"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="8"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="4"/>
-      <c r="B39" s="37"/>
-      <c r="C39" s="5"/>
-      <c r="D39" s="6"/>
-      <c r="E39" s="5"/>
+      <c r="A39" s="8"/>
+      <c r="B39" s="28"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="8"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="7"/>
-      <c r="B40" s="32"/>
+      <c r="A40" s="8"/>
+      <c r="B40" s="28"/>
       <c r="C40" s="8"/>
       <c r="D40" s="9"/>
       <c r="E40" s="8"/>
     </row>
-    <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="7"/>
-      <c r="B41" s="32"/>
+    <row r="41" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="8"/>
+      <c r="B41" s="29"/>
       <c r="C41" s="8"/>
       <c r="D41" s="9"/>
       <c r="E41" s="8"/>
     </row>
-    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="7"/>
-      <c r="B42" s="32"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="8"/>
-    </row>
-    <row r="43" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="10"/>
-      <c r="B43" s="33"/>
-      <c r="C43" s="10"/>
-      <c r="D43" s="11"/>
-      <c r="E43" s="10"/>
-    </row>
-    <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="12" t="s">
+    <row r="42" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B44" s="34"/>
-      <c r="C44" s="35"/>
-      <c r="D44" s="35"/>
-      <c r="E44" s="36"/>
+      <c r="B42" s="30"/>
+      <c r="C42" s="31"/>
+      <c r="D42" s="31"/>
+      <c r="E42" s="32"/>
+    </row>
+    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="4"/>
+      <c r="B43" s="27"/>
+      <c r="C43" s="5"/>
+      <c r="D43" s="6"/>
+      <c r="E43" s="5"/>
+    </row>
+    <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="7"/>
+      <c r="B44" s="28"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="4"/>
-      <c r="B45" s="31"/>
-      <c r="C45" s="5"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="5"/>
+      <c r="A45" s="7"/>
+      <c r="B45" s="28"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="8"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="7"/>
-      <c r="B46" s="32"/>
+      <c r="B46" s="28"/>
       <c r="C46" s="8"/>
       <c r="D46" s="9"/>
       <c r="E46" s="8"/>
     </row>
-    <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="7"/>
-      <c r="B47" s="32"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="9"/>
-      <c r="E47" s="8"/>
-    </row>
-    <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="7"/>
-      <c r="B48" s="32"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="9"/>
-      <c r="E48" s="8"/>
-    </row>
-    <row r="49" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="10"/>
-      <c r="B49" s="33"/>
-      <c r="C49" s="10"/>
-      <c r="D49" s="11"/>
-      <c r="E49" s="10"/>
-    </row>
-    <row r="50" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="12" t="s">
+    <row r="47" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="10"/>
+      <c r="B47" s="29"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="10"/>
+    </row>
+    <row r="48" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B50" s="34"/>
-      <c r="C50" s="35"/>
-      <c r="D50" s="35"/>
-      <c r="E50" s="36"/>
+      <c r="B48" s="30"/>
+      <c r="C48" s="31"/>
+      <c r="D48" s="31"/>
+      <c r="E48" s="32"/>
+    </row>
+    <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="4"/>
+      <c r="B49" s="35"/>
+      <c r="C49" s="5"/>
+      <c r="D49" s="6"/>
+      <c r="E49" s="5"/>
+    </row>
+    <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="7"/>
+      <c r="B50" s="28"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="4"/>
-      <c r="B51" s="31"/>
-      <c r="C51" s="5"/>
-      <c r="D51" s="6"/>
-      <c r="E51" s="5"/>
+      <c r="A51" s="7"/>
+      <c r="B51" s="28"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="8"/>
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="7"/>
-      <c r="B52" s="32"/>
+      <c r="B52" s="28"/>
       <c r="C52" s="8"/>
       <c r="D52" s="9"/>
       <c r="E52" s="8"/>
     </row>
-    <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="7"/>
-      <c r="B53" s="32"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="8"/>
-    </row>
-    <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="7"/>
-      <c r="B54" s="32"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="8"/>
-    </row>
-    <row r="55" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="10"/>
-      <c r="B55" s="33"/>
-      <c r="C55" s="10"/>
-      <c r="D55" s="11"/>
-      <c r="E55" s="10"/>
-    </row>
-    <row r="56" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="12" t="s">
+    <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="10"/>
+      <c r="B53" s="29"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="11"/>
+      <c r="E53" s="10"/>
+    </row>
+    <row r="54" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B56" s="34"/>
-      <c r="C56" s="35"/>
-      <c r="D56" s="35"/>
-      <c r="E56" s="36"/>
+      <c r="B54" s="30"/>
+      <c r="C54" s="31"/>
+      <c r="D54" s="31"/>
+      <c r="E54" s="32"/>
+    </row>
+    <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="4"/>
+      <c r="B55" s="35"/>
+      <c r="C55" s="5"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="5"/>
+    </row>
+    <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="7"/>
+      <c r="B56" s="28"/>
+      <c r="C56" s="8"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="4"/>
-      <c r="B57" s="31"/>
-      <c r="C57" s="5"/>
-      <c r="D57" s="6"/>
-      <c r="E57" s="5"/>
+      <c r="A57" s="7"/>
+      <c r="B57" s="28"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="9"/>
+      <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="32"/>
+      <c r="B58" s="28"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
-    <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="7"/>
-      <c r="B59" s="32"/>
-      <c r="C59" s="8"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="8"/>
-    </row>
-    <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="7"/>
-      <c r="B60" s="32"/>
-      <c r="C60" s="8"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="8"/>
-    </row>
-    <row r="61" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="10"/>
-      <c r="B61" s="33"/>
-      <c r="C61" s="10"/>
-      <c r="D61" s="11"/>
-      <c r="E61" s="10"/>
-    </row>
-    <row r="62" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="12" t="s">
+    <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="10"/>
+      <c r="B59" s="29"/>
+      <c r="C59" s="10"/>
+      <c r="D59" s="11"/>
+      <c r="E59" s="10"/>
+    </row>
+    <row r="60" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B62" s="34"/>
-      <c r="C62" s="35"/>
-      <c r="D62" s="35"/>
-      <c r="E62" s="36"/>
+      <c r="B60" s="30"/>
+      <c r="C60" s="31"/>
+      <c r="D60" s="31"/>
+      <c r="E60" s="32"/>
+    </row>
+    <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="4"/>
+      <c r="B61" s="35"/>
+      <c r="C61" s="5"/>
+      <c r="D61" s="6"/>
+      <c r="E61" s="5"/>
+    </row>
+    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="7"/>
+      <c r="B62" s="28"/>
+      <c r="C62" s="8"/>
+      <c r="D62" s="9"/>
+      <c r="E62" s="8"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="13"/>
-      <c r="B63" s="31"/>
-      <c r="C63" s="13"/>
-      <c r="D63" s="14"/>
-      <c r="E63" s="13"/>
+      <c r="A63" s="7"/>
+      <c r="B63" s="28"/>
+      <c r="C63" s="8"/>
+      <c r="D63" s="9"/>
+      <c r="E63" s="8"/>
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="8"/>
-      <c r="B64" s="32"/>
+      <c r="A64" s="7"/>
+      <c r="B64" s="28"/>
       <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
-    <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="8"/>
-      <c r="B65" s="32"/>
-      <c r="C65" s="8"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="8"/>
-    </row>
-    <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="8"/>
-      <c r="B66" s="32"/>
-      <c r="C66" s="8"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="8"/>
-    </row>
-    <row r="67" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="8"/>
-      <c r="B67" s="33"/>
-      <c r="C67" s="8"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="8"/>
-    </row>
-    <row r="68" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="12" t="s">
+    <row r="65" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="10"/>
+      <c r="B65" s="29"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="11"/>
+      <c r="E65" s="10"/>
+    </row>
+    <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B68" s="34"/>
-      <c r="C68" s="35"/>
-      <c r="D68" s="35"/>
-      <c r="E68" s="36"/>
-    </row>
-    <row r="69" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="38" t="s">
+      <c r="B66" s="30"/>
+      <c r="C66" s="31"/>
+      <c r="D66" s="31"/>
+      <c r="E66" s="32"/>
+    </row>
+    <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="13"/>
+      <c r="B67" s="35"/>
+      <c r="C67" s="13"/>
+      <c r="D67" s="14"/>
+      <c r="E67" s="13"/>
+    </row>
+    <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="8"/>
+      <c r="B68" s="28"/>
+      <c r="C68" s="8"/>
+      <c r="D68" s="9"/>
+      <c r="E68" s="8"/>
+    </row>
+    <row r="69" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="8"/>
+      <c r="B69" s="28"/>
+      <c r="C69" s="8"/>
+      <c r="D69" s="9"/>
+      <c r="E69" s="8"/>
+    </row>
+    <row r="70" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="8"/>
+      <c r="B70" s="28"/>
+      <c r="C70" s="8"/>
+      <c r="D70" s="9"/>
+      <c r="E70" s="8"/>
+    </row>
+    <row r="71" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="8"/>
+      <c r="B71" s="29"/>
+      <c r="C71" s="8"/>
+      <c r="D71" s="9"/>
+      <c r="E71" s="8"/>
+    </row>
+    <row r="72" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B72" s="30"/>
+      <c r="C72" s="31"/>
+      <c r="D72" s="31"/>
+      <c r="E72" s="32"/>
+    </row>
+    <row r="73" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="B69" s="39"/>
-      <c r="C69" s="15">
-        <f>MROUND(SUM(C6:C68) /60,0.2)</f>
-        <v>3.8000000000000003</v>
-      </c>
-      <c r="D69" s="16"/>
-      <c r="E69" s="17"/>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="18" t="s">
+      <c r="B73" s="34"/>
+      <c r="C73" s="15">
+        <f>MROUND(SUM(C6:C72) /60,0.2)</f>
+        <v>5.4</v>
+      </c>
+      <c r="D73" s="16"/>
+      <c r="E73" s="17"/>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="18"/>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B39:B43"/>
-    <mergeCell ref="B68:E68"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="B45:B49"/>
-    <mergeCell ref="B50:E50"/>
-    <mergeCell ref="B51:B55"/>
-    <mergeCell ref="B56:E56"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="B62:E62"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B63:B67"/>
-    <mergeCell ref="B44:E44"/>
-    <mergeCell ref="B6:B13"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="B15:B19"/>
-    <mergeCell ref="B20:E20"/>
-    <mergeCell ref="B21:B25"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B27:B31"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B33:B37"/>
-    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B67:B71"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B6:B17"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="B19:B23"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B25:B29"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B31:B35"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B43:B47"/>
+    <mergeCell ref="B72:E72"/>
+    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="B49:B53"/>
+    <mergeCell ref="B54:E54"/>
+    <mergeCell ref="B55:B59"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="B61:B65"/>
+    <mergeCell ref="B66:E66"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C57:C61 C51:C55 C39:C43 C45:C49 C21:C25 B6 C15:C19 C27:C31 C33:C37 C63:C67 C6:C13" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C61:C65 C55:C59 C43:C47 C49:C53 C25:C29 B6 C19:C23 C31:C35 C37:C41 C67:C71 C6:C17" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B15:B19 B21:B25 B27:B31 B33:B37 B39:B43 B45:B49 B51:B55 B57:B61 B63:B67" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B23 B25:B29 B31:B35 B37:B41 B43:B47 B49:B53 B55:B59 B61:B65 B67:B71" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -1700,18 +1769,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1877,18 +1946,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat(doc): add high fidelity model
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D631A27-029D-4D9E-84B3-803093B451FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{458EF6D6-EE96-428C-9979-08C15E5B0C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="53">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -195,6 +195,21 @@
   </si>
   <si>
     <t>J'ai continué mes maquettes</t>
+  </si>
+  <si>
+    <t>Suite au mail de M. Borboën j'ai modifié ma planification</t>
+  </si>
+  <si>
+    <t>J'ai commencé les maquettes hautes fidélité et en cours j'ai remarqué que j'avais oublié de faire la page de vue d'une campagne dans les maquette basse fidélité</t>
+  </si>
+  <si>
+    <t>J'ai finis les maquette HF pour la page d'accueil</t>
+  </si>
+  <si>
+    <t>J'ai terminé mes maquettes HF et j'ai aussi corrigé les maquette BF</t>
+  </si>
+  <si>
+    <t>11h15</t>
   </si>
 </sst>
 </file>
@@ -1142,33 +1157,61 @@
       <c r="E18" s="32"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="4"/>
-      <c r="B19" s="27"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="6"/>
+      <c r="A19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="27">
+        <v>46139</v>
+      </c>
+      <c r="C19" s="5">
+        <v>30</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>48</v>
+      </c>
       <c r="E19" s="5"/>
     </row>
-    <row r="20" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
+    <row r="20" spans="1:7" ht="27" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>45</v>
+      </c>
       <c r="B20" s="28"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="9"/>
+      <c r="C20" s="8">
+        <v>55</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>49</v>
+      </c>
       <c r="E20" s="8"/>
     </row>
     <row r="21" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="7"/>
+      <c r="A21" s="7" t="s">
+        <v>45</v>
+      </c>
       <c r="B21" s="28"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="9"/>
+      <c r="C21" s="8">
+        <v>40</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>50</v>
+      </c>
       <c r="E21" s="8"/>
       <c r="G21" s="25"/>
     </row>
     <row r="22" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
+      <c r="A22" s="7" t="s">
+        <v>45</v>
+      </c>
       <c r="B22" s="28"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="8"/>
+      <c r="C22" s="8">
+        <v>45</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="23" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="10"/>
@@ -1181,7 +1224,10 @@
       <c r="A24" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="30"/>
+      <c r="B24" s="30" t="str">
+        <f>INT(SUM(C19:C23)/60)&amp;"h"&amp;MOD(SUM(C19:C23),60)</f>
+        <v>2h50</v>
+      </c>
       <c r="C24" s="31"/>
       <c r="D24" s="31"/>
       <c r="E24" s="32"/>
@@ -1545,7 +1591,7 @@
       <c r="B73" s="34"/>
       <c r="C73" s="15">
         <f>MROUND(SUM(C6:C72) /60,0.2)</f>
-        <v>5.4</v>
+        <v>8.2000000000000011</v>
       </c>
       <c r="D73" s="16"/>
       <c r="E73" s="17"/>

</xml_diff>

<commit_message>
feat(db) add database and create login endpoint
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{458EF6D6-EE96-428C-9979-08C15E5B0C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA66601-AE3F-4853-AF87-82C169D9B25A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$73</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$74</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="54">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -209,7 +209,10 @@
     <t>J'ai terminé mes maquettes HF et j'ai aussi corrigé les maquette BF</t>
   </si>
   <si>
-    <t>11h15</t>
+    <t>Base de donnée</t>
+  </si>
+  <si>
+    <t>J'ai fais la modélisation de ma base de donnée et j'ai aussi profité pour créer la route de login</t>
   </si>
 </sst>
 </file>
@@ -537,51 +540,51 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -899,7 +902,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -915,10 +918,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="36"/>
+      <c r="C1" s="27"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -930,10 +933,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="36"/>
+      <c r="C2" s="27"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -945,10 +948,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="36"/>
+      <c r="C3" s="27"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -960,12 +963,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="39"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -988,7 +991,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="27">
+      <c r="B6" s="37">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1001,7 +1004,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="28"/>
+      <c r="B7" s="32"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1014,7 +1017,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="28"/>
+      <c r="B8" s="32"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1027,7 +1030,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="28"/>
+      <c r="B9" s="32"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1038,7 +1041,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="28"/>
+      <c r="B10" s="32"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1051,7 +1054,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="28"/>
+      <c r="B11" s="32"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1066,7 +1069,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="28"/>
+      <c r="B12" s="32"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1081,7 +1084,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="28"/>
+      <c r="B13" s="32"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1096,7 +1099,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="28"/>
+      <c r="B14" s="32"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1111,7 +1114,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="28"/>
+      <c r="B15" s="32"/>
       <c r="C15" s="10">
         <v>40</v>
       </c>
@@ -1126,7 +1129,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="28"/>
+      <c r="B16" s="32"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1139,7 +1142,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="29"/>
+      <c r="B17" s="33"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1148,23 +1151,23 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="30" t="str">
+      <c r="B18" s="34" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="32"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="36"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="27">
+      <c r="B19" s="37">
         <v>46139</v>
       </c>
       <c r="C19" s="5">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>48</v>
@@ -1175,7 +1178,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="28"/>
+      <c r="B20" s="32"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1188,7 +1191,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="28"/>
+      <c r="B21" s="32"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1202,441 +1205,452 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="28"/>
+      <c r="B22" s="32"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="8"/>
+    </row>
+    <row r="23" spans="1:7" ht="27" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="10"/>
-      <c r="B23" s="29"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="11"/>
+      <c r="B23" s="32"/>
+      <c r="C23" s="10">
+        <v>60</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>53</v>
+      </c>
       <c r="E23" s="10"/>
     </row>
     <row r="24" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="10"/>
+      <c r="B24" s="33"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="10"/>
+    </row>
+    <row r="25" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="30" t="str">
-        <f>INT(SUM(C19:C23)/60)&amp;"h"&amp;MOD(SUM(C19:C23),60)</f>
-        <v>2h50</v>
-      </c>
-      <c r="C24" s="31"/>
-      <c r="D24" s="31"/>
-      <c r="E24" s="32"/>
-    </row>
-    <row r="25" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4"/>
-      <c r="B25" s="35"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="5"/>
+      <c r="B25" s="34" t="str">
+        <f>INT(SUM(C19:C24)/60)&amp;"h"&amp;MOD(SUM(C19:C24),60)</f>
+        <v>4h0</v>
+      </c>
+      <c r="C25" s="35"/>
+      <c r="D25" s="35"/>
+      <c r="E25" s="36"/>
     </row>
     <row r="26" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="7"/>
-      <c r="B26" s="28"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="8"/>
+      <c r="A26" s="4"/>
+      <c r="B26" s="31"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="5"/>
     </row>
     <row r="27" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7"/>
-      <c r="B27" s="28"/>
+      <c r="B27" s="32"/>
       <c r="C27" s="8"/>
       <c r="D27" s="9"/>
       <c r="E27" s="8"/>
     </row>
     <row r="28" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
-      <c r="B28" s="28"/>
+      <c r="B28" s="32"/>
       <c r="C28" s="8"/>
       <c r="D28" s="9"/>
       <c r="E28" s="8"/>
     </row>
-    <row r="29" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="10"/>
-      <c r="B29" s="29"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="10"/>
+    <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="7"/>
+      <c r="B29" s="32"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="8"/>
     </row>
     <row r="30" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="10"/>
+      <c r="B30" s="33"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B30" s="30"/>
-      <c r="C30" s="31"/>
-      <c r="D30" s="31"/>
-      <c r="E30" s="32"/>
-    </row>
-    <row r="31" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="4"/>
-      <c r="B31" s="35"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="5"/>
+      <c r="B31" s="34"/>
+      <c r="C31" s="35"/>
+      <c r="D31" s="35"/>
+      <c r="E31" s="36"/>
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="7"/>
-      <c r="B32" s="28"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="8"/>
+      <c r="A32" s="4"/>
+      <c r="B32" s="31"/>
+      <c r="C32" s="5"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="5"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7"/>
-      <c r="B33" s="28"/>
+      <c r="B33" s="32"/>
       <c r="C33" s="8"/>
       <c r="D33" s="9"/>
       <c r="E33" s="8"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7"/>
-      <c r="B34" s="28"/>
+      <c r="B34" s="32"/>
       <c r="C34" s="8"/>
       <c r="D34" s="9"/>
       <c r="E34" s="8"/>
     </row>
-    <row r="35" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="10"/>
-      <c r="B35" s="29"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="10"/>
+    <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="7"/>
+      <c r="B35" s="32"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="8"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="12" t="s">
+      <c r="A36" s="10"/>
+      <c r="B36" s="33"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="10"/>
+    </row>
+    <row r="37" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B36" s="30"/>
-      <c r="C36" s="31"/>
-      <c r="D36" s="31"/>
-      <c r="E36" s="32"/>
-    </row>
-    <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="13"/>
-      <c r="B37" s="35"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="13"/>
+      <c r="B37" s="34"/>
+      <c r="C37" s="35"/>
+      <c r="D37" s="35"/>
+      <c r="E37" s="36"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="8"/>
-      <c r="B38" s="28"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="8"/>
+      <c r="A38" s="13"/>
+      <c r="B38" s="31"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="13"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8"/>
-      <c r="B39" s="28"/>
+      <c r="B39" s="32"/>
       <c r="C39" s="8"/>
       <c r="D39" s="9"/>
       <c r="E39" s="8"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8"/>
-      <c r="B40" s="28"/>
+      <c r="B40" s="32"/>
       <c r="C40" s="8"/>
       <c r="D40" s="9"/>
       <c r="E40" s="8"/>
     </row>
-    <row r="41" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8"/>
-      <c r="B41" s="29"/>
+      <c r="B41" s="32"/>
       <c r="C41" s="8"/>
       <c r="D41" s="9"/>
       <c r="E41" s="8"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="12" t="s">
+      <c r="A42" s="8"/>
+      <c r="B42" s="33"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="8"/>
+    </row>
+    <row r="43" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B42" s="30"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="31"/>
-      <c r="E42" s="32"/>
-    </row>
-    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="4"/>
-      <c r="B43" s="27"/>
-      <c r="C43" s="5"/>
-      <c r="D43" s="6"/>
-      <c r="E43" s="5"/>
+      <c r="B43" s="34"/>
+      <c r="C43" s="35"/>
+      <c r="D43" s="35"/>
+      <c r="E43" s="36"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="7"/>
-      <c r="B44" s="28"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="8"/>
+      <c r="A44" s="4"/>
+      <c r="B44" s="37"/>
+      <c r="C44" s="5"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="5"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="7"/>
-      <c r="B45" s="28"/>
+      <c r="B45" s="32"/>
       <c r="C45" s="8"/>
       <c r="D45" s="9"/>
       <c r="E45" s="8"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="7"/>
-      <c r="B46" s="28"/>
+      <c r="B46" s="32"/>
       <c r="C46" s="8"/>
       <c r="D46" s="9"/>
       <c r="E46" s="8"/>
     </row>
-    <row r="47" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="10"/>
-      <c r="B47" s="29"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="10"/>
+    <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="7"/>
+      <c r="B47" s="32"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="8"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="12" t="s">
+      <c r="A48" s="10"/>
+      <c r="B48" s="33"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="11"/>
+      <c r="E48" s="10"/>
+    </row>
+    <row r="49" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="30"/>
-      <c r="C48" s="31"/>
-      <c r="D48" s="31"/>
-      <c r="E48" s="32"/>
-    </row>
-    <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="4"/>
-      <c r="B49" s="35"/>
-      <c r="C49" s="5"/>
-      <c r="D49" s="6"/>
-      <c r="E49" s="5"/>
+      <c r="B49" s="34"/>
+      <c r="C49" s="35"/>
+      <c r="D49" s="35"/>
+      <c r="E49" s="36"/>
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="7"/>
-      <c r="B50" s="28"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="8"/>
+      <c r="A50" s="4"/>
+      <c r="B50" s="31"/>
+      <c r="C50" s="5"/>
+      <c r="D50" s="6"/>
+      <c r="E50" s="5"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
-      <c r="B51" s="28"/>
+      <c r="B51" s="32"/>
       <c r="C51" s="8"/>
       <c r="D51" s="9"/>
       <c r="E51" s="8"/>
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="7"/>
-      <c r="B52" s="28"/>
+      <c r="B52" s="32"/>
       <c r="C52" s="8"/>
       <c r="D52" s="9"/>
       <c r="E52" s="8"/>
     </row>
-    <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="10"/>
-      <c r="B53" s="29"/>
-      <c r="C53" s="10"/>
-      <c r="D53" s="11"/>
-      <c r="E53" s="10"/>
+    <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="7"/>
+      <c r="B53" s="32"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="8"/>
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="12" t="s">
+      <c r="A54" s="10"/>
+      <c r="B54" s="33"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="10"/>
+    </row>
+    <row r="55" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B54" s="30"/>
-      <c r="C54" s="31"/>
-      <c r="D54" s="31"/>
-      <c r="E54" s="32"/>
-    </row>
-    <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="4"/>
-      <c r="B55" s="35"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="6"/>
-      <c r="E55" s="5"/>
+      <c r="B55" s="34"/>
+      <c r="C55" s="35"/>
+      <c r="D55" s="35"/>
+      <c r="E55" s="36"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="7"/>
-      <c r="B56" s="28"/>
-      <c r="C56" s="8"/>
-      <c r="D56" s="9"/>
-      <c r="E56" s="8"/>
+      <c r="A56" s="4"/>
+      <c r="B56" s="31"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="5"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="28"/>
+      <c r="B57" s="32"/>
       <c r="C57" s="8"/>
       <c r="D57" s="9"/>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="28"/>
+      <c r="B58" s="32"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
-    <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="10"/>
-      <c r="B59" s="29"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="11"/>
-      <c r="E59" s="10"/>
+    <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="7"/>
+      <c r="B59" s="32"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="8"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="12" t="s">
+      <c r="A60" s="10"/>
+      <c r="B60" s="33"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="11"/>
+      <c r="E60" s="10"/>
+    </row>
+    <row r="61" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B60" s="30"/>
-      <c r="C60" s="31"/>
-      <c r="D60" s="31"/>
-      <c r="E60" s="32"/>
-    </row>
-    <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="4"/>
-      <c r="B61" s="35"/>
-      <c r="C61" s="5"/>
-      <c r="D61" s="6"/>
-      <c r="E61" s="5"/>
+      <c r="B61" s="34"/>
+      <c r="C61" s="35"/>
+      <c r="D61" s="35"/>
+      <c r="E61" s="36"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="7"/>
-      <c r="B62" s="28"/>
-      <c r="C62" s="8"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="8"/>
+      <c r="A62" s="4"/>
+      <c r="B62" s="31"/>
+      <c r="C62" s="5"/>
+      <c r="D62" s="6"/>
+      <c r="E62" s="5"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="28"/>
+      <c r="B63" s="32"/>
       <c r="C63" s="8"/>
       <c r="D63" s="9"/>
       <c r="E63" s="8"/>
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="28"/>
+      <c r="B64" s="32"/>
       <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
-    <row r="65" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="10"/>
-      <c r="B65" s="29"/>
-      <c r="C65" s="10"/>
-      <c r="D65" s="11"/>
-      <c r="E65" s="10"/>
+    <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="7"/>
+      <c r="B65" s="32"/>
+      <c r="C65" s="8"/>
+      <c r="D65" s="9"/>
+      <c r="E65" s="8"/>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="12" t="s">
+      <c r="A66" s="10"/>
+      <c r="B66" s="33"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="11"/>
+      <c r="E66" s="10"/>
+    </row>
+    <row r="67" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B66" s="30"/>
-      <c r="C66" s="31"/>
-      <c r="D66" s="31"/>
-      <c r="E66" s="32"/>
-    </row>
-    <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="13"/>
-      <c r="B67" s="35"/>
-      <c r="C67" s="13"/>
-      <c r="D67" s="14"/>
-      <c r="E67" s="13"/>
+      <c r="B67" s="34"/>
+      <c r="C67" s="35"/>
+      <c r="D67" s="35"/>
+      <c r="E67" s="36"/>
     </row>
     <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="8"/>
-      <c r="B68" s="28"/>
-      <c r="C68" s="8"/>
-      <c r="D68" s="9"/>
-      <c r="E68" s="8"/>
+      <c r="A68" s="13"/>
+      <c r="B68" s="31"/>
+      <c r="C68" s="13"/>
+      <c r="D68" s="14"/>
+      <c r="E68" s="13"/>
     </row>
     <row r="69" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="8"/>
-      <c r="B69" s="28"/>
+      <c r="B69" s="32"/>
       <c r="C69" s="8"/>
       <c r="D69" s="9"/>
       <c r="E69" s="8"/>
     </row>
     <row r="70" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="8"/>
-      <c r="B70" s="28"/>
+      <c r="B70" s="32"/>
       <c r="C70" s="8"/>
       <c r="D70" s="9"/>
       <c r="E70" s="8"/>
     </row>
-    <row r="71" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="8"/>
-      <c r="B71" s="29"/>
+      <c r="B71" s="32"/>
       <c r="C71" s="8"/>
       <c r="D71" s="9"/>
       <c r="E71" s="8"/>
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="12" t="s">
+      <c r="A72" s="8"/>
+      <c r="B72" s="33"/>
+      <c r="C72" s="8"/>
+      <c r="D72" s="9"/>
+      <c r="E72" s="8"/>
+    </row>
+    <row r="73" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B72" s="30"/>
-      <c r="C72" s="31"/>
-      <c r="D72" s="31"/>
-      <c r="E72" s="32"/>
-    </row>
-    <row r="73" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="33" t="s">
+      <c r="B73" s="34"/>
+      <c r="C73" s="35"/>
+      <c r="D73" s="35"/>
+      <c r="E73" s="36"/>
+    </row>
+    <row r="74" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="B73" s="34"/>
-      <c r="C73" s="15">
-        <f>MROUND(SUM(C6:C72) /60,0.2)</f>
-        <v>8.2000000000000011</v>
-      </c>
-      <c r="D73" s="16"/>
-      <c r="E73" s="17"/>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" s="18" t="s">
+      <c r="B74" s="39"/>
+      <c r="C74" s="15">
+        <f>MROUND(SUM(C6:C73) /60,0.2)</f>
+        <v>9.4</v>
+      </c>
+      <c r="D74" s="16"/>
+      <c r="E74" s="17"/>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" s="18"/>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B44:B48"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="B56:B60"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="B67:E67"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B67:B71"/>
-    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B49:E49"/>
     <mergeCell ref="B6:B17"/>
     <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B19:B23"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B25:B29"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B31:B35"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B42:E42"/>
-    <mergeCell ref="B43:B47"/>
-    <mergeCell ref="B72:E72"/>
-    <mergeCell ref="A73:B73"/>
-    <mergeCell ref="B49:B53"/>
-    <mergeCell ref="B54:E54"/>
-    <mergeCell ref="B55:B59"/>
-    <mergeCell ref="B60:E60"/>
-    <mergeCell ref="B61:B65"/>
-    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="B19:B24"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B26:B30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B38:B42"/>
+    <mergeCell ref="B43:E43"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C61:C65 C55:C59 C43:C47 C49:C53 C25:C29 B6 C19:C23 C31:C35 C37:C41 C67:C71 C6:C17" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C62:C66 C56:C60 C44:C48 C50:C54 C26:C30 B6 C6:C17 C32:C36 C38:C42 C68:C72 C19:C24" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B23 B25:B29 B31:B35 B37:B41 B43:B47 B49:B53 B55:B59 B61:B65 B67:B71" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B24 B26:B30 B32:B36 B38:B42 B44:B48 B50:B54 B56:B60 B62:B66 B68:B72" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -1653,7 +1667,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E348320A-3DEF-4FFB-92B3-3073BCAD0028}">
-  <dimension ref="C5:I19"/>
+  <dimension ref="C5:I20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
@@ -1809,24 +1823,30 @@
         <v>0.13194444444444445</v>
       </c>
     </row>
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E20" s="26">
+        <f>E8-D8-(H8/2)</f>
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1992,18 +2012,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat(db): add connection to DB
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA66601-AE3F-4853-AF87-82C169D9B25A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F2F1A60-635B-4CA1-98B1-04EFAB3F2EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$74</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$76</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="56">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -213,6 +213,12 @@
   </si>
   <si>
     <t>J'ai fais la modélisation de ma base de donnée et j'ai aussi profité pour créer la route de login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai des problème pour pouvoir utilisé ma base de donnée </t>
+  </si>
+  <si>
+    <t>J'ai enfin regle le sproblème avec ma base donnée le problème était du à la verison de prisma je suis donc retourné dans une version antiérieur (celle utilisée dans le P-APPRO2)</t>
   </si>
 </sst>
 </file>
@@ -540,51 +546,51 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -902,7 +908,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -918,10 +924,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="27"/>
+      <c r="C1" s="36"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -933,10 +939,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="27"/>
+      <c r="C2" s="36"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -948,10 +954,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="27"/>
+      <c r="C3" s="36"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -963,12 +969,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="30"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="39"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -991,7 +997,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="37">
+      <c r="B6" s="27">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1004,7 +1010,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="32"/>
+      <c r="B7" s="28"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1017,7 +1023,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="32"/>
+      <c r="B8" s="28"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1030,7 +1036,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="32"/>
+      <c r="B9" s="28"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1041,7 +1047,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="32"/>
+      <c r="B10" s="28"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1054,7 +1060,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="32"/>
+      <c r="B11" s="28"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1069,7 +1075,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="32"/>
+      <c r="B12" s="28"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1084,7 +1090,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="32"/>
+      <c r="B13" s="28"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1099,7 +1105,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="32"/>
+      <c r="B14" s="28"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1114,7 +1120,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="32"/>
+      <c r="B15" s="28"/>
       <c r="C15" s="10">
         <v>40</v>
       </c>
@@ -1129,7 +1135,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="32"/>
+      <c r="B16" s="28"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1142,7 +1148,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="33"/>
+      <c r="B17" s="29"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1151,19 +1157,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="34" t="str">
+      <c r="B18" s="30" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="36"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="32"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="37">
+      <c r="B19" s="27">
         <v>46139</v>
       </c>
       <c r="C19" s="5">
@@ -1178,7 +1184,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="32"/>
+      <c r="B20" s="28"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1191,7 +1197,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="32"/>
+      <c r="B21" s="28"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1205,7 +1211,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="32"/>
+      <c r="B22" s="28"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1218,7 +1224,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="32"/>
+      <c r="B23" s="28"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1227,430 +1233,456 @@
       </c>
       <c r="E23" s="10"/>
     </row>
-    <row r="24" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="10"/>
-      <c r="B24" s="33"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="11"/>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" s="28"/>
+      <c r="C24" s="10">
+        <v>60</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>54</v>
+      </c>
       <c r="E24" s="10"/>
     </row>
-    <row r="25" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
+    <row r="25" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="28"/>
+      <c r="C25" s="10">
+        <v>30</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="E25" s="10"/>
+    </row>
+    <row r="26" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="10"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="34" t="str">
-        <f>INT(SUM(C19:C24)/60)&amp;"h"&amp;MOD(SUM(C19:C24),60)</f>
-        <v>4h0</v>
-      </c>
-      <c r="C25" s="35"/>
-      <c r="D25" s="35"/>
-      <c r="E25" s="36"/>
-    </row>
-    <row r="26" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="4"/>
-      <c r="B26" s="31"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="5"/>
-    </row>
-    <row r="27" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="7"/>
-      <c r="B27" s="32"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="8"/>
+      <c r="B27" s="30" t="str">
+        <f>INT(SUM(C19:C26)/60)&amp;"h"&amp;MOD(SUM(C19:C26),60)</f>
+        <v>5h30</v>
+      </c>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="32"/>
     </row>
     <row r="28" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="7"/>
-      <c r="B28" s="32"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="8"/>
+      <c r="A28" s="4"/>
+      <c r="B28" s="35"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="5"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
-      <c r="B29" s="32"/>
+      <c r="B29" s="28"/>
       <c r="C29" s="8"/>
       <c r="D29" s="9"/>
       <c r="E29" s="8"/>
     </row>
-    <row r="30" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="10"/>
-      <c r="B30" s="33"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="10"/>
-    </row>
-    <row r="31" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="12" t="s">
+    <row r="30" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="7"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="8"/>
+    </row>
+    <row r="31" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="7"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="8"/>
+    </row>
+    <row r="32" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="10"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="10"/>
+    </row>
+    <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B31" s="34"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="35"/>
-      <c r="E31" s="36"/>
-    </row>
-    <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="4"/>
-      <c r="B32" s="31"/>
-      <c r="C32" s="5"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="5"/>
-    </row>
-    <row r="33" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="7"/>
-      <c r="B33" s="32"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="8"/>
+      <c r="B33" s="30"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="31"/>
+      <c r="E33" s="32"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="7"/>
-      <c r="B34" s="32"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="8"/>
+      <c r="A34" s="4"/>
+      <c r="B34" s="35"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="5"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7"/>
-      <c r="B35" s="32"/>
+      <c r="B35" s="28"/>
       <c r="C35" s="8"/>
       <c r="D35" s="9"/>
       <c r="E35" s="8"/>
     </row>
-    <row r="36" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="10"/>
-      <c r="B36" s="33"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="10"/>
-    </row>
-    <row r="37" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="12" t="s">
+    <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="7"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="8"/>
+    </row>
+    <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="7"/>
+      <c r="B37" s="28"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="8"/>
+    </row>
+    <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="10"/>
+      <c r="B38" s="29"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="11"/>
+      <c r="E38" s="10"/>
+    </row>
+    <row r="39" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B37" s="34"/>
-      <c r="C37" s="35"/>
-      <c r="D37" s="35"/>
-      <c r="E37" s="36"/>
-    </row>
-    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="13"/>
-      <c r="B38" s="31"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="13"/>
-    </row>
-    <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="8"/>
-      <c r="B39" s="32"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="8"/>
+      <c r="B39" s="30"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="31"/>
+      <c r="E39" s="32"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="8"/>
-      <c r="B40" s="32"/>
-      <c r="C40" s="8"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="8"/>
+      <c r="A40" s="13"/>
+      <c r="B40" s="35"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="13"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8"/>
-      <c r="B41" s="32"/>
+      <c r="B41" s="28"/>
       <c r="C41" s="8"/>
       <c r="D41" s="9"/>
       <c r="E41" s="8"/>
     </row>
-    <row r="42" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8"/>
-      <c r="B42" s="33"/>
+      <c r="B42" s="28"/>
       <c r="C42" s="8"/>
       <c r="D42" s="9"/>
       <c r="E42" s="8"/>
     </row>
-    <row r="43" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="12" t="s">
+    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="8"/>
+      <c r="B43" s="28"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="8"/>
+    </row>
+    <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="8"/>
+      <c r="B44" s="29"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="8"/>
+    </row>
+    <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B43" s="34"/>
-      <c r="C43" s="35"/>
-      <c r="D43" s="35"/>
-      <c r="E43" s="36"/>
-    </row>
-    <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="4"/>
-      <c r="B44" s="37"/>
-      <c r="C44" s="5"/>
-      <c r="D44" s="6"/>
-      <c r="E44" s="5"/>
-    </row>
-    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="7"/>
-      <c r="B45" s="32"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="8"/>
+      <c r="B45" s="30"/>
+      <c r="C45" s="31"/>
+      <c r="D45" s="31"/>
+      <c r="E45" s="32"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="7"/>
-      <c r="B46" s="32"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="8"/>
+      <c r="A46" s="4"/>
+      <c r="B46" s="27"/>
+      <c r="C46" s="5"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="5"/>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7"/>
-      <c r="B47" s="32"/>
+      <c r="B47" s="28"/>
       <c r="C47" s="8"/>
       <c r="D47" s="9"/>
       <c r="E47" s="8"/>
     </row>
-    <row r="48" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="10"/>
-      <c r="B48" s="33"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="10"/>
-    </row>
-    <row r="49" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="12" t="s">
+    <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="7"/>
+      <c r="B48" s="28"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="8"/>
+    </row>
+    <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="7"/>
+      <c r="B49" s="28"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="8"/>
+    </row>
+    <row r="50" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="10"/>
+      <c r="B50" s="29"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="10"/>
+    </row>
+    <row r="51" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B49" s="34"/>
-      <c r="C49" s="35"/>
-      <c r="D49" s="35"/>
-      <c r="E49" s="36"/>
-    </row>
-    <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="4"/>
-      <c r="B50" s="31"/>
-      <c r="C50" s="5"/>
-      <c r="D50" s="6"/>
-      <c r="E50" s="5"/>
-    </row>
-    <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="7"/>
-      <c r="B51" s="32"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="9"/>
-      <c r="E51" s="8"/>
+      <c r="B51" s="30"/>
+      <c r="C51" s="31"/>
+      <c r="D51" s="31"/>
+      <c r="E51" s="32"/>
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="7"/>
-      <c r="B52" s="32"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="8"/>
+      <c r="A52" s="4"/>
+      <c r="B52" s="35"/>
+      <c r="C52" s="5"/>
+      <c r="D52" s="6"/>
+      <c r="E52" s="5"/>
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="7"/>
-      <c r="B53" s="32"/>
+      <c r="B53" s="28"/>
       <c r="C53" s="8"/>
       <c r="D53" s="9"/>
       <c r="E53" s="8"/>
     </row>
-    <row r="54" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="10"/>
-      <c r="B54" s="33"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="10"/>
-    </row>
-    <row r="55" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="12" t="s">
+    <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="7"/>
+      <c r="B54" s="28"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="8"/>
+    </row>
+    <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="7"/>
+      <c r="B55" s="28"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="8"/>
+    </row>
+    <row r="56" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="10"/>
+      <c r="B56" s="29"/>
+      <c r="C56" s="10"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="10"/>
+    </row>
+    <row r="57" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B55" s="34"/>
-      <c r="C55" s="35"/>
-      <c r="D55" s="35"/>
-      <c r="E55" s="36"/>
-    </row>
-    <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="4"/>
-      <c r="B56" s="31"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="6"/>
-      <c r="E56" s="5"/>
-    </row>
-    <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="7"/>
-      <c r="B57" s="32"/>
-      <c r="C57" s="8"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="8"/>
+      <c r="B57" s="30"/>
+      <c r="C57" s="31"/>
+      <c r="D57" s="31"/>
+      <c r="E57" s="32"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="7"/>
-      <c r="B58" s="32"/>
-      <c r="C58" s="8"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="8"/>
+      <c r="A58" s="4"/>
+      <c r="B58" s="35"/>
+      <c r="C58" s="5"/>
+      <c r="D58" s="6"/>
+      <c r="E58" s="5"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="7"/>
-      <c r="B59" s="32"/>
+      <c r="B59" s="28"/>
       <c r="C59" s="8"/>
       <c r="D59" s="9"/>
       <c r="E59" s="8"/>
     </row>
-    <row r="60" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="10"/>
-      <c r="B60" s="33"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="11"/>
-      <c r="E60" s="10"/>
-    </row>
-    <row r="61" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="12" t="s">
+    <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="7"/>
+      <c r="B60" s="28"/>
+      <c r="C60" s="8"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="8"/>
+    </row>
+    <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="7"/>
+      <c r="B61" s="28"/>
+      <c r="C61" s="8"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="8"/>
+    </row>
+    <row r="62" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="10"/>
+      <c r="B62" s="29"/>
+      <c r="C62" s="10"/>
+      <c r="D62" s="11"/>
+      <c r="E62" s="10"/>
+    </row>
+    <row r="63" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B61" s="34"/>
-      <c r="C61" s="35"/>
-      <c r="D61" s="35"/>
-      <c r="E61" s="36"/>
-    </row>
-    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="4"/>
-      <c r="B62" s="31"/>
-      <c r="C62" s="5"/>
-      <c r="D62" s="6"/>
-      <c r="E62" s="5"/>
-    </row>
-    <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="7"/>
-      <c r="B63" s="32"/>
-      <c r="C63" s="8"/>
-      <c r="D63" s="9"/>
-      <c r="E63" s="8"/>
+      <c r="B63" s="30"/>
+      <c r="C63" s="31"/>
+      <c r="D63" s="31"/>
+      <c r="E63" s="32"/>
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="7"/>
-      <c r="B64" s="32"/>
-      <c r="C64" s="8"/>
-      <c r="D64" s="9"/>
-      <c r="E64" s="8"/>
+      <c r="A64" s="4"/>
+      <c r="B64" s="35"/>
+      <c r="C64" s="5"/>
+      <c r="D64" s="6"/>
+      <c r="E64" s="5"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
-      <c r="B65" s="32"/>
+      <c r="B65" s="28"/>
       <c r="C65" s="8"/>
       <c r="D65" s="9"/>
       <c r="E65" s="8"/>
     </row>
-    <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="10"/>
-      <c r="B66" s="33"/>
-      <c r="C66" s="10"/>
-      <c r="D66" s="11"/>
-      <c r="E66" s="10"/>
-    </row>
-    <row r="67" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="12" t="s">
+    <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="7"/>
+      <c r="B66" s="28"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="9"/>
+      <c r="E66" s="8"/>
+    </row>
+    <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="7"/>
+      <c r="B67" s="28"/>
+      <c r="C67" s="8"/>
+      <c r="D67" s="9"/>
+      <c r="E67" s="8"/>
+    </row>
+    <row r="68" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="10"/>
+      <c r="B68" s="29"/>
+      <c r="C68" s="10"/>
+      <c r="D68" s="11"/>
+      <c r="E68" s="10"/>
+    </row>
+    <row r="69" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B67" s="34"/>
-      <c r="C67" s="35"/>
-      <c r="D67" s="35"/>
-      <c r="E67" s="36"/>
-    </row>
-    <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="13"/>
-      <c r="B68" s="31"/>
-      <c r="C68" s="13"/>
-      <c r="D68" s="14"/>
-      <c r="E68" s="13"/>
-    </row>
-    <row r="69" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="8"/>
-      <c r="B69" s="32"/>
-      <c r="C69" s="8"/>
-      <c r="D69" s="9"/>
-      <c r="E69" s="8"/>
+      <c r="B69" s="30"/>
+      <c r="C69" s="31"/>
+      <c r="D69" s="31"/>
+      <c r="E69" s="32"/>
     </row>
     <row r="70" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="8"/>
-      <c r="B70" s="32"/>
-      <c r="C70" s="8"/>
-      <c r="D70" s="9"/>
-      <c r="E70" s="8"/>
+      <c r="A70" s="13"/>
+      <c r="B70" s="35"/>
+      <c r="C70" s="13"/>
+      <c r="D70" s="14"/>
+      <c r="E70" s="13"/>
     </row>
     <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="8"/>
-      <c r="B71" s="32"/>
+      <c r="B71" s="28"/>
       <c r="C71" s="8"/>
       <c r="D71" s="9"/>
       <c r="E71" s="8"/>
     </row>
-    <row r="72" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8"/>
-      <c r="B72" s="33"/>
+      <c r="B72" s="28"/>
       <c r="C72" s="8"/>
       <c r="D72" s="9"/>
       <c r="E72" s="8"/>
     </row>
-    <row r="73" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="12" t="s">
+    <row r="73" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="8"/>
+      <c r="B73" s="28"/>
+      <c r="C73" s="8"/>
+      <c r="D73" s="9"/>
+      <c r="E73" s="8"/>
+    </row>
+    <row r="74" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="8"/>
+      <c r="B74" s="29"/>
+      <c r="C74" s="8"/>
+      <c r="D74" s="9"/>
+      <c r="E74" s="8"/>
+    </row>
+    <row r="75" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B73" s="34"/>
-      <c r="C73" s="35"/>
-      <c r="D73" s="35"/>
-      <c r="E73" s="36"/>
-    </row>
-    <row r="74" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="38" t="s">
+      <c r="B75" s="30"/>
+      <c r="C75" s="31"/>
+      <c r="D75" s="31"/>
+      <c r="E75" s="32"/>
+    </row>
+    <row r="76" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="B74" s="39"/>
-      <c r="C74" s="15">
-        <f>MROUND(SUM(C6:C73) /60,0.2)</f>
-        <v>9.4</v>
-      </c>
-      <c r="D74" s="16"/>
-      <c r="E74" s="17"/>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" s="18" t="s">
+      <c r="B76" s="34"/>
+      <c r="C76" s="15">
+        <f>MROUND(SUM(C6:C75) /60,0.2)</f>
+        <v>10.8</v>
+      </c>
+      <c r="D76" s="16"/>
+      <c r="E76" s="17"/>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" s="18"/>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B44:B48"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="A74:B74"/>
-    <mergeCell ref="B50:B54"/>
-    <mergeCell ref="B55:E55"/>
-    <mergeCell ref="B56:B60"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="B67:E67"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B70:B74"/>
+    <mergeCell ref="B51:E51"/>
     <mergeCell ref="B6:B17"/>
     <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B19:B24"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B26:B30"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="B38:B42"/>
-    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="B19:B26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B28:B32"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B40:B44"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B46:B50"/>
+    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="A76:B76"/>
+    <mergeCell ref="B52:B56"/>
+    <mergeCell ref="B57:E57"/>
+    <mergeCell ref="B58:B62"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="B69:E69"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C62:C66 C56:C60 C44:C48 C50:C54 C26:C30 B6 C6:C17 C32:C36 C38:C42 C68:C72 C19:C24" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C64:C68 C58:C62 C46:C50 C52:C56 C28:C32 B6 C6:C17 C34:C38 C40:C44 C70:C74 C19:C26" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B24 B26:B30 B32:B36 B38:B42 B44:B48 B50:B54 B56:B60 B62:B66 B68:B72" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B26 B28:B32 B34:B38 B40:B44 B46:B50 B52:B56 B58:B62 B64:B68 B70:B74" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -1835,18 +1867,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2012,18 +2044,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat(app): add subscribe page
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F2F1A60-635B-4CA1-98B1-04EFAB3F2EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11AF9F37-C307-414E-BE54-DA13E59FDD75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$76</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$77</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="60">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -219,6 +219,18 @@
   </si>
   <si>
     <t>J'ai enfin regle le sproblème avec ma base donnée le problème était du à la verison de prisma je suis donc retourné dans une version antiérieur (celle utilisée dans le P-APPRO2)</t>
+  </si>
+  <si>
+    <t>page d'abonnement</t>
+  </si>
+  <si>
+    <t>J'ai fais la page pour s'abonner</t>
+  </si>
+  <si>
+    <t>Ajustement</t>
+  </si>
+  <si>
+    <t>J'ai fait quelque ajustement au niveau de la page et j'ai aussi fait la page de politique de confidentialité (fait par IA)</t>
   </si>
 </sst>
 </file>
@@ -546,51 +558,51 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -908,7 +920,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -924,10 +936,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="36"/>
+      <c r="C1" s="27"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -939,10 +951,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="36"/>
+      <c r="C2" s="27"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -954,10 +966,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="36"/>
+      <c r="C3" s="27"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -969,12 +981,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="39"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -997,7 +1009,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="27">
+      <c r="B6" s="37">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1010,7 +1022,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="28"/>
+      <c r="B7" s="32"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1023,7 +1035,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="28"/>
+      <c r="B8" s="32"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1036,7 +1048,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="28"/>
+      <c r="B9" s="32"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1047,7 +1059,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="28"/>
+      <c r="B10" s="32"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1060,7 +1072,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="28"/>
+      <c r="B11" s="32"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1075,7 +1087,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="28"/>
+      <c r="B12" s="32"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1090,7 +1102,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="28"/>
+      <c r="B13" s="32"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1105,7 +1117,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="28"/>
+      <c r="B14" s="32"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1120,7 +1132,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="28"/>
+      <c r="B15" s="32"/>
       <c r="C15" s="10">
         <v>40</v>
       </c>
@@ -1135,7 +1147,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="28"/>
+      <c r="B16" s="32"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1148,7 +1160,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="29"/>
+      <c r="B17" s="33"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1157,19 +1169,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="30" t="str">
+      <c r="B18" s="34" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="32"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="36"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="27">
+      <c r="B19" s="37">
         <v>46139</v>
       </c>
       <c r="C19" s="5">
@@ -1184,7 +1196,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="28"/>
+      <c r="B20" s="32"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1197,7 +1209,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="28"/>
+      <c r="B21" s="32"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1211,7 +1223,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="28"/>
+      <c r="B22" s="32"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1224,7 +1236,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="28"/>
+      <c r="B23" s="32"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1237,7 +1249,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="28"/>
+      <c r="B24" s="32"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1250,7 +1262,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="28"/>
+      <c r="B25" s="32"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1259,436 +1271,455 @@
       </c>
       <c r="E25" s="10"/>
     </row>
-    <row r="26" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="10"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="11"/>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" s="32"/>
+      <c r="C26" s="10">
+        <v>60</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>57</v>
+      </c>
       <c r="E26" s="10"/>
     </row>
-    <row r="27" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="12" t="s">
+    <row r="27" spans="1:7" ht="27.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B27" s="33"/>
+      <c r="C27" s="10">
+        <v>40</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="E27" s="10"/>
+    </row>
+    <row r="28" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B27" s="30" t="str">
-        <f>INT(SUM(C19:C26)/60)&amp;"h"&amp;MOD(SUM(C19:C26),60)</f>
-        <v>5h30</v>
-      </c>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="32"/>
-    </row>
-    <row r="28" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="4"/>
-      <c r="B28" s="35"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="5"/>
+      <c r="B28" s="34" t="str">
+        <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
+        <v>7h10</v>
+      </c>
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="36"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="7"/>
-      <c r="B29" s="28"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="8"/>
+      <c r="A29" s="4"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="5"/>
     </row>
     <row r="30" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
-      <c r="B30" s="28"/>
+      <c r="B30" s="32"/>
       <c r="C30" s="8"/>
       <c r="D30" s="9"/>
       <c r="E30" s="8"/>
     </row>
     <row r="31" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7"/>
-      <c r="B31" s="28"/>
+      <c r="B31" s="32"/>
       <c r="C31" s="8"/>
       <c r="D31" s="9"/>
       <c r="E31" s="8"/>
     </row>
-    <row r="32" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="10"/>
-      <c r="B32" s="29"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="10"/>
+    <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="7"/>
+      <c r="B32" s="32"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="12" t="s">
+      <c r="A33" s="10"/>
+      <c r="B33" s="33"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="10"/>
+    </row>
+    <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B33" s="30"/>
-      <c r="C33" s="31"/>
-      <c r="D33" s="31"/>
-      <c r="E33" s="32"/>
-    </row>
-    <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="4"/>
-      <c r="B34" s="35"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="5"/>
+      <c r="B34" s="34"/>
+      <c r="C34" s="35"/>
+      <c r="D34" s="35"/>
+      <c r="E34" s="36"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="7"/>
-      <c r="B35" s="28"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="8"/>
+      <c r="A35" s="4"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="5"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="5"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7"/>
-      <c r="B36" s="28"/>
+      <c r="B36" s="32"/>
       <c r="C36" s="8"/>
       <c r="D36" s="9"/>
       <c r="E36" s="8"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="28"/>
+      <c r="B37" s="32"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
-    <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="10"/>
-      <c r="B38" s="29"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="10"/>
+    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="7"/>
+      <c r="B38" s="32"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="8"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="12" t="s">
+      <c r="A39" s="10"/>
+      <c r="B39" s="33"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="11"/>
+      <c r="E39" s="10"/>
+    </row>
+    <row r="40" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B39" s="30"/>
-      <c r="C39" s="31"/>
-      <c r="D39" s="31"/>
-      <c r="E39" s="32"/>
-    </row>
-    <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="13"/>
-      <c r="B40" s="35"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="13"/>
+      <c r="B40" s="34"/>
+      <c r="C40" s="35"/>
+      <c r="D40" s="35"/>
+      <c r="E40" s="36"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="8"/>
-      <c r="B41" s="28"/>
-      <c r="C41" s="8"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="8"/>
+      <c r="A41" s="13"/>
+      <c r="B41" s="31"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="13"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8"/>
-      <c r="B42" s="28"/>
+      <c r="B42" s="32"/>
       <c r="C42" s="8"/>
       <c r="D42" s="9"/>
       <c r="E42" s="8"/>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8"/>
-      <c r="B43" s="28"/>
+      <c r="B43" s="32"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
-    <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8"/>
-      <c r="B44" s="29"/>
+      <c r="B44" s="32"/>
       <c r="C44" s="8"/>
       <c r="D44" s="9"/>
       <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="12" t="s">
+      <c r="A45" s="8"/>
+      <c r="B45" s="33"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="8"/>
+    </row>
+    <row r="46" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="30"/>
-      <c r="C45" s="31"/>
-      <c r="D45" s="31"/>
-      <c r="E45" s="32"/>
-    </row>
-    <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="4"/>
-      <c r="B46" s="27"/>
-      <c r="C46" s="5"/>
-      <c r="D46" s="6"/>
-      <c r="E46" s="5"/>
+      <c r="B46" s="34"/>
+      <c r="C46" s="35"/>
+      <c r="D46" s="35"/>
+      <c r="E46" s="36"/>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="7"/>
-      <c r="B47" s="28"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="9"/>
-      <c r="E47" s="8"/>
+      <c r="A47" s="4"/>
+      <c r="B47" s="37"/>
+      <c r="C47" s="5"/>
+      <c r="D47" s="6"/>
+      <c r="E47" s="5"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="7"/>
-      <c r="B48" s="28"/>
+      <c r="B48" s="32"/>
       <c r="C48" s="8"/>
       <c r="D48" s="9"/>
       <c r="E48" s="8"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="28"/>
+      <c r="B49" s="32"/>
       <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
-    <row r="50" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="10"/>
-      <c r="B50" s="29"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="11"/>
-      <c r="E50" s="10"/>
+    <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="7"/>
+      <c r="B50" s="32"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="12" t="s">
+      <c r="A51" s="10"/>
+      <c r="B51" s="33"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="11"/>
+      <c r="E51" s="10"/>
+    </row>
+    <row r="52" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B51" s="30"/>
-      <c r="C51" s="31"/>
-      <c r="D51" s="31"/>
-      <c r="E51" s="32"/>
-    </row>
-    <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="4"/>
-      <c r="B52" s="35"/>
-      <c r="C52" s="5"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="5"/>
+      <c r="B52" s="34"/>
+      <c r="C52" s="35"/>
+      <c r="D52" s="35"/>
+      <c r="E52" s="36"/>
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="7"/>
-      <c r="B53" s="28"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="8"/>
+      <c r="A53" s="4"/>
+      <c r="B53" s="31"/>
+      <c r="C53" s="5"/>
+      <c r="D53" s="6"/>
+      <c r="E53" s="5"/>
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="7"/>
-      <c r="B54" s="28"/>
+      <c r="B54" s="32"/>
       <c r="C54" s="8"/>
       <c r="D54" s="9"/>
       <c r="E54" s="8"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="7"/>
-      <c r="B55" s="28"/>
+      <c r="B55" s="32"/>
       <c r="C55" s="8"/>
       <c r="D55" s="9"/>
       <c r="E55" s="8"/>
     </row>
-    <row r="56" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="10"/>
-      <c r="B56" s="29"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="10"/>
+    <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="7"/>
+      <c r="B56" s="32"/>
+      <c r="C56" s="8"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="12" t="s">
+      <c r="A57" s="10"/>
+      <c r="B57" s="33"/>
+      <c r="C57" s="10"/>
+      <c r="D57" s="11"/>
+      <c r="E57" s="10"/>
+    </row>
+    <row r="58" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B57" s="30"/>
-      <c r="C57" s="31"/>
-      <c r="D57" s="31"/>
-      <c r="E57" s="32"/>
-    </row>
-    <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="4"/>
-      <c r="B58" s="35"/>
-      <c r="C58" s="5"/>
-      <c r="D58" s="6"/>
-      <c r="E58" s="5"/>
+      <c r="B58" s="34"/>
+      <c r="C58" s="35"/>
+      <c r="D58" s="35"/>
+      <c r="E58" s="36"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="7"/>
-      <c r="B59" s="28"/>
-      <c r="C59" s="8"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="8"/>
+      <c r="A59" s="4"/>
+      <c r="B59" s="31"/>
+      <c r="C59" s="5"/>
+      <c r="D59" s="6"/>
+      <c r="E59" s="5"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="7"/>
-      <c r="B60" s="28"/>
+      <c r="B60" s="32"/>
       <c r="C60" s="8"/>
       <c r="D60" s="9"/>
       <c r="E60" s="8"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="7"/>
-      <c r="B61" s="28"/>
+      <c r="B61" s="32"/>
       <c r="C61" s="8"/>
       <c r="D61" s="9"/>
       <c r="E61" s="8"/>
     </row>
-    <row r="62" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="10"/>
-      <c r="B62" s="29"/>
-      <c r="C62" s="10"/>
-      <c r="D62" s="11"/>
-      <c r="E62" s="10"/>
+    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="7"/>
+      <c r="B62" s="32"/>
+      <c r="C62" s="8"/>
+      <c r="D62" s="9"/>
+      <c r="E62" s="8"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="12" t="s">
+      <c r="A63" s="10"/>
+      <c r="B63" s="33"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="11"/>
+      <c r="E63" s="10"/>
+    </row>
+    <row r="64" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B63" s="30"/>
-      <c r="C63" s="31"/>
-      <c r="D63" s="31"/>
-      <c r="E63" s="32"/>
-    </row>
-    <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="4"/>
-      <c r="B64" s="35"/>
-      <c r="C64" s="5"/>
-      <c r="D64" s="6"/>
-      <c r="E64" s="5"/>
+      <c r="B64" s="34"/>
+      <c r="C64" s="35"/>
+      <c r="D64" s="35"/>
+      <c r="E64" s="36"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="7"/>
-      <c r="B65" s="28"/>
-      <c r="C65" s="8"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="8"/>
+      <c r="A65" s="4"/>
+      <c r="B65" s="31"/>
+      <c r="C65" s="5"/>
+      <c r="D65" s="6"/>
+      <c r="E65" s="5"/>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="7"/>
-      <c r="B66" s="28"/>
+      <c r="B66" s="32"/>
       <c r="C66" s="8"/>
       <c r="D66" s="9"/>
       <c r="E66" s="8"/>
     </row>
     <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="7"/>
-      <c r="B67" s="28"/>
+      <c r="B67" s="32"/>
       <c r="C67" s="8"/>
       <c r="D67" s="9"/>
       <c r="E67" s="8"/>
     </row>
-    <row r="68" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="10"/>
-      <c r="B68" s="29"/>
-      <c r="C68" s="10"/>
-      <c r="D68" s="11"/>
-      <c r="E68" s="10"/>
+    <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="7"/>
+      <c r="B68" s="32"/>
+      <c r="C68" s="8"/>
+      <c r="D68" s="9"/>
+      <c r="E68" s="8"/>
     </row>
     <row r="69" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="12" t="s">
+      <c r="A69" s="10"/>
+      <c r="B69" s="33"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="11"/>
+      <c r="E69" s="10"/>
+    </row>
+    <row r="70" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B69" s="30"/>
-      <c r="C69" s="31"/>
-      <c r="D69" s="31"/>
-      <c r="E69" s="32"/>
-    </row>
-    <row r="70" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="13"/>
-      <c r="B70" s="35"/>
-      <c r="C70" s="13"/>
-      <c r="D70" s="14"/>
-      <c r="E70" s="13"/>
+      <c r="B70" s="34"/>
+      <c r="C70" s="35"/>
+      <c r="D70" s="35"/>
+      <c r="E70" s="36"/>
     </row>
     <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="8"/>
-      <c r="B71" s="28"/>
-      <c r="C71" s="8"/>
-      <c r="D71" s="9"/>
-      <c r="E71" s="8"/>
+      <c r="A71" s="13"/>
+      <c r="B71" s="31"/>
+      <c r="C71" s="13"/>
+      <c r="D71" s="14"/>
+      <c r="E71" s="13"/>
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8"/>
-      <c r="B72" s="28"/>
+      <c r="B72" s="32"/>
       <c r="C72" s="8"/>
       <c r="D72" s="9"/>
       <c r="E72" s="8"/>
     </row>
     <row r="73" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8"/>
-      <c r="B73" s="28"/>
+      <c r="B73" s="32"/>
       <c r="C73" s="8"/>
       <c r="D73" s="9"/>
       <c r="E73" s="8"/>
     </row>
-    <row r="74" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8"/>
-      <c r="B74" s="29"/>
+      <c r="B74" s="32"/>
       <c r="C74" s="8"/>
       <c r="D74" s="9"/>
       <c r="E74" s="8"/>
     </row>
     <row r="75" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="12" t="s">
+      <c r="A75" s="8"/>
+      <c r="B75" s="33"/>
+      <c r="C75" s="8"/>
+      <c r="D75" s="9"/>
+      <c r="E75" s="8"/>
+    </row>
+    <row r="76" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B75" s="30"/>
-      <c r="C75" s="31"/>
-      <c r="D75" s="31"/>
-      <c r="E75" s="32"/>
-    </row>
-    <row r="76" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="33" t="s">
+      <c r="B76" s="34"/>
+      <c r="C76" s="35"/>
+      <c r="D76" s="35"/>
+      <c r="E76" s="36"/>
+    </row>
+    <row r="77" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="B76" s="34"/>
-      <c r="C76" s="15">
-        <f>MROUND(SUM(C6:C75) /60,0.2)</f>
-        <v>10.8</v>
-      </c>
-      <c r="D76" s="16"/>
-      <c r="E76" s="17"/>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" s="18" t="s">
+      <c r="B77" s="39"/>
+      <c r="C77" s="15">
+        <f>MROUND(SUM(C6:C76) /60,0.2)</f>
+        <v>12.600000000000001</v>
+      </c>
+      <c r="D77" s="16"/>
+      <c r="E77" s="17"/>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" s="18"/>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B76:E76"/>
+    <mergeCell ref="A77:B77"/>
+    <mergeCell ref="B53:B57"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="B65:B69"/>
+    <mergeCell ref="B70:E70"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B70:B74"/>
-    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="B71:B75"/>
+    <mergeCell ref="B52:E52"/>
     <mergeCell ref="B6:B17"/>
     <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B19:B26"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="B28:B32"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="B40:B44"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B46:B50"/>
-    <mergeCell ref="B75:E75"/>
-    <mergeCell ref="A76:B76"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B57:E57"/>
-    <mergeCell ref="B58:B62"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="B64:B68"/>
-    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="B19:B27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B29:B33"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B35:B39"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B41:B45"/>
+    <mergeCell ref="B46:E46"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C64:C68 C58:C62 C46:C50 C52:C56 C28:C32 B6 C6:C17 C34:C38 C40:C44 C70:C74 C19:C26" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C65:C69 C59:C63 C47:C51 C53:C57 C29:C33 B6 C6:C17 C35:C39 C41:C45 C71:C75 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B26 B28:B32 B34:B38 B40:B44 B46:B50 B52:B56 B58:B62 B64:B68 B70:B74" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B39 B41:B45 B47:B51 B53:B57 B59:B63 B65:B69 B71:B75" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="50" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="49" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -1863,22 +1894,23 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2044,18 +2076,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat(app): add un/subscribe system
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11AF9F37-C307-414E-BE54-DA13E59FDD75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4228423-44FD-4EFC-BC2A-226399F89347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="65">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -231,6 +231,21 @@
   </si>
   <si>
     <t>J'ai fait quelque ajustement au niveau de la page et j'ai aussi fait la page de politique de confidentialité (fait par IA)</t>
+  </si>
+  <si>
+    <t>Inscription</t>
+  </si>
+  <si>
+    <t>J'ai presque terminé le système d'abonnement il me manque juste un petit detail</t>
+  </si>
+  <si>
+    <t>Désinscription</t>
+  </si>
+  <si>
+    <t>J'ai fais le système de déinscription, si j'ai pris autant de tempsc'est parce que je ne savais pas si au niveau légal je pouvais conserver l'utilisateur et enfaite j'ai appris que effectivement je dois supprimé les données dès lors quelles ne sont plus utiles cependant je peux les anonymisées et c'est ce que j'ai choisi</t>
+  </si>
+  <si>
+    <t>http://weka.ch/themes/ressources-humaines/contrats-de-travail-et-reglements/protection-des-donnees/article/donnees-rh-quels-sont-les-delais-de-conservation-des-donnees-des-collaborateurs/</t>
   </si>
 </sst>
 </file>
@@ -470,7 +485,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -558,51 +573,55 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -936,10 +955,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="27"/>
+      <c r="C1" s="36"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -951,10 +970,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="27"/>
+      <c r="C2" s="36"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -966,10 +985,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="27"/>
+      <c r="C3" s="36"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -981,12 +1000,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="30"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="39"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1009,7 +1028,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="37">
+      <c r="B6" s="27">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1022,7 +1041,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="32"/>
+      <c r="B7" s="28"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1035,7 +1054,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="32"/>
+      <c r="B8" s="28"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1048,7 +1067,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="32"/>
+      <c r="B9" s="28"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1059,7 +1078,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="32"/>
+      <c r="B10" s="28"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1072,7 +1091,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="32"/>
+      <c r="B11" s="28"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1087,7 +1106,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="32"/>
+      <c r="B12" s="28"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1102,7 +1121,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="32"/>
+      <c r="B13" s="28"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1117,7 +1136,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="32"/>
+      <c r="B14" s="28"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1132,7 +1151,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="32"/>
+      <c r="B15" s="28"/>
       <c r="C15" s="10">
         <v>40</v>
       </c>
@@ -1147,7 +1166,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="32"/>
+      <c r="B16" s="28"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1160,7 +1179,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="33"/>
+      <c r="B17" s="29"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1169,20 +1188,20 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="34" t="str">
+      <c r="B18" s="30" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="36"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="32"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="37">
-        <v>46139</v>
+      <c r="B19" s="27">
+        <v>46141</v>
       </c>
       <c r="C19" s="5">
         <v>40</v>
@@ -1196,7 +1215,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="32"/>
+      <c r="B20" s="28"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1209,7 +1228,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="32"/>
+      <c r="B21" s="28"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1223,7 +1242,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="32"/>
+      <c r="B22" s="28"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1236,7 +1255,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="32"/>
+      <c r="B23" s="28"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1249,7 +1268,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="32"/>
+      <c r="B24" s="28"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1262,7 +1281,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="32"/>
+      <c r="B25" s="28"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1275,7 +1294,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="32"/>
+      <c r="B26" s="28"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1288,7 +1307,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="33"/>
+      <c r="B27" s="29"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1301,45 +1320,61 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="34" t="str">
+      <c r="B28" s="30" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="35"/>
-      <c r="D28" s="35"/>
-      <c r="E28" s="36"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="32"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="4"/>
-      <c r="B29" s="31"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="6"/>
+      <c r="A29" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29" s="27">
+        <v>46142</v>
+      </c>
+      <c r="C29" s="5">
+        <v>60</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>61</v>
+      </c>
       <c r="E29" s="5"/>
     </row>
-    <row r="30" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="7"/>
-      <c r="B30" s="32"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="8"/>
+    <row r="30" spans="1:7" ht="54" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" s="28"/>
+      <c r="C30" s="8">
+        <v>60</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="E30" s="40" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="31" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7"/>
-      <c r="B31" s="32"/>
+      <c r="B31" s="28"/>
       <c r="C31" s="8"/>
       <c r="D31" s="9"/>
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="32"/>
+      <c r="B32" s="28"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="33"/>
+      <c r="B33" s="29"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1348,42 +1383,45 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="34"/>
-      <c r="C34" s="35"/>
-      <c r="D34" s="35"/>
-      <c r="E34" s="36"/>
+      <c r="B34" s="30" t="str">
+        <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
+        <v>2h0</v>
+      </c>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="32"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
-      <c r="B35" s="31"/>
+      <c r="B35" s="35"/>
       <c r="C35" s="5"/>
       <c r="D35" s="6"/>
       <c r="E35" s="5"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7"/>
-      <c r="B36" s="32"/>
+      <c r="B36" s="28"/>
       <c r="C36" s="8"/>
       <c r="D36" s="9"/>
       <c r="E36" s="8"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="32"/>
+      <c r="B37" s="28"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="7"/>
-      <c r="B38" s="32"/>
+      <c r="B38" s="28"/>
       <c r="C38" s="8"/>
       <c r="D38" s="9"/>
       <c r="E38" s="8"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="10"/>
-      <c r="B39" s="33"/>
+      <c r="B39" s="29"/>
       <c r="C39" s="10"/>
       <c r="D39" s="11"/>
       <c r="E39" s="10"/>
@@ -1392,42 +1430,42 @@
       <c r="A40" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B40" s="34"/>
-      <c r="C40" s="35"/>
-      <c r="D40" s="35"/>
-      <c r="E40" s="36"/>
+      <c r="B40" s="30"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
+      <c r="E40" s="32"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="13"/>
-      <c r="B41" s="31"/>
+      <c r="B41" s="35"/>
       <c r="C41" s="13"/>
       <c r="D41" s="14"/>
       <c r="E41" s="13"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8"/>
-      <c r="B42" s="32"/>
+      <c r="B42" s="28"/>
       <c r="C42" s="8"/>
       <c r="D42" s="9"/>
       <c r="E42" s="8"/>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8"/>
-      <c r="B43" s="32"/>
+      <c r="B43" s="28"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8"/>
-      <c r="B44" s="32"/>
+      <c r="B44" s="28"/>
       <c r="C44" s="8"/>
       <c r="D44" s="9"/>
       <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="8"/>
-      <c r="B45" s="33"/>
+      <c r="B45" s="29"/>
       <c r="C45" s="8"/>
       <c r="D45" s="9"/>
       <c r="E45" s="8"/>
@@ -1436,42 +1474,42 @@
       <c r="A46" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="34"/>
-      <c r="C46" s="35"/>
-      <c r="D46" s="35"/>
-      <c r="E46" s="36"/>
+      <c r="B46" s="30"/>
+      <c r="C46" s="31"/>
+      <c r="D46" s="31"/>
+      <c r="E46" s="32"/>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="4"/>
-      <c r="B47" s="37"/>
+      <c r="B47" s="27"/>
       <c r="C47" s="5"/>
       <c r="D47" s="6"/>
       <c r="E47" s="5"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="7"/>
-      <c r="B48" s="32"/>
+      <c r="B48" s="28"/>
       <c r="C48" s="8"/>
       <c r="D48" s="9"/>
       <c r="E48" s="8"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="32"/>
+      <c r="B49" s="28"/>
       <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="32"/>
+      <c r="B50" s="28"/>
       <c r="C50" s="8"/>
       <c r="D50" s="9"/>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="10"/>
-      <c r="B51" s="33"/>
+      <c r="B51" s="29"/>
       <c r="C51" s="10"/>
       <c r="D51" s="11"/>
       <c r="E51" s="10"/>
@@ -1480,42 +1518,42 @@
       <c r="A52" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B52" s="34"/>
-      <c r="C52" s="35"/>
-      <c r="D52" s="35"/>
-      <c r="E52" s="36"/>
+      <c r="B52" s="30"/>
+      <c r="C52" s="31"/>
+      <c r="D52" s="31"/>
+      <c r="E52" s="32"/>
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4"/>
-      <c r="B53" s="31"/>
+      <c r="B53" s="35"/>
       <c r="C53" s="5"/>
       <c r="D53" s="6"/>
       <c r="E53" s="5"/>
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="7"/>
-      <c r="B54" s="32"/>
+      <c r="B54" s="28"/>
       <c r="C54" s="8"/>
       <c r="D54" s="9"/>
       <c r="E54" s="8"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="7"/>
-      <c r="B55" s="32"/>
+      <c r="B55" s="28"/>
       <c r="C55" s="8"/>
       <c r="D55" s="9"/>
       <c r="E55" s="8"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
-      <c r="B56" s="32"/>
+      <c r="B56" s="28"/>
       <c r="C56" s="8"/>
       <c r="D56" s="9"/>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="10"/>
-      <c r="B57" s="33"/>
+      <c r="B57" s="29"/>
       <c r="C57" s="10"/>
       <c r="D57" s="11"/>
       <c r="E57" s="10"/>
@@ -1524,42 +1562,42 @@
       <c r="A58" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B58" s="34"/>
-      <c r="C58" s="35"/>
-      <c r="D58" s="35"/>
-      <c r="E58" s="36"/>
+      <c r="B58" s="30"/>
+      <c r="C58" s="31"/>
+      <c r="D58" s="31"/>
+      <c r="E58" s="32"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4"/>
-      <c r="B59" s="31"/>
+      <c r="B59" s="35"/>
       <c r="C59" s="5"/>
       <c r="D59" s="6"/>
       <c r="E59" s="5"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="7"/>
-      <c r="B60" s="32"/>
+      <c r="B60" s="28"/>
       <c r="C60" s="8"/>
       <c r="D60" s="9"/>
       <c r="E60" s="8"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="7"/>
-      <c r="B61" s="32"/>
+      <c r="B61" s="28"/>
       <c r="C61" s="8"/>
       <c r="D61" s="9"/>
       <c r="E61" s="8"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="7"/>
-      <c r="B62" s="32"/>
+      <c r="B62" s="28"/>
       <c r="C62" s="8"/>
       <c r="D62" s="9"/>
       <c r="E62" s="8"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="10"/>
-      <c r="B63" s="33"/>
+      <c r="B63" s="29"/>
       <c r="C63" s="10"/>
       <c r="D63" s="11"/>
       <c r="E63" s="10"/>
@@ -1568,42 +1606,42 @@
       <c r="A64" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B64" s="34"/>
-      <c r="C64" s="35"/>
-      <c r="D64" s="35"/>
-      <c r="E64" s="36"/>
+      <c r="B64" s="30"/>
+      <c r="C64" s="31"/>
+      <c r="D64" s="31"/>
+      <c r="E64" s="32"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4"/>
-      <c r="B65" s="31"/>
+      <c r="B65" s="35"/>
       <c r="C65" s="5"/>
       <c r="D65" s="6"/>
       <c r="E65" s="5"/>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="7"/>
-      <c r="B66" s="32"/>
+      <c r="B66" s="28"/>
       <c r="C66" s="8"/>
       <c r="D66" s="9"/>
       <c r="E66" s="8"/>
     </row>
     <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="7"/>
-      <c r="B67" s="32"/>
+      <c r="B67" s="28"/>
       <c r="C67" s="8"/>
       <c r="D67" s="9"/>
       <c r="E67" s="8"/>
     </row>
     <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7"/>
-      <c r="B68" s="32"/>
+      <c r="B68" s="28"/>
       <c r="C68" s="8"/>
       <c r="D68" s="9"/>
       <c r="E68" s="8"/>
     </row>
     <row r="69" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="10"/>
-      <c r="B69" s="33"/>
+      <c r="B69" s="29"/>
       <c r="C69" s="10"/>
       <c r="D69" s="11"/>
       <c r="E69" s="10"/>
@@ -1612,42 +1650,42 @@
       <c r="A70" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B70" s="34"/>
-      <c r="C70" s="35"/>
-      <c r="D70" s="35"/>
-      <c r="E70" s="36"/>
+      <c r="B70" s="30"/>
+      <c r="C70" s="31"/>
+      <c r="D70" s="31"/>
+      <c r="E70" s="32"/>
     </row>
     <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="13"/>
-      <c r="B71" s="31"/>
+      <c r="B71" s="35"/>
       <c r="C71" s="13"/>
       <c r="D71" s="14"/>
       <c r="E71" s="13"/>
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8"/>
-      <c r="B72" s="32"/>
+      <c r="B72" s="28"/>
       <c r="C72" s="8"/>
       <c r="D72" s="9"/>
       <c r="E72" s="8"/>
     </row>
     <row r="73" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8"/>
-      <c r="B73" s="32"/>
+      <c r="B73" s="28"/>
       <c r="C73" s="8"/>
       <c r="D73" s="9"/>
       <c r="E73" s="8"/>
     </row>
     <row r="74" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8"/>
-      <c r="B74" s="32"/>
+      <c r="B74" s="28"/>
       <c r="C74" s="8"/>
       <c r="D74" s="9"/>
       <c r="E74" s="8"/>
     </row>
     <row r="75" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="8"/>
-      <c r="B75" s="33"/>
+      <c r="B75" s="29"/>
       <c r="C75" s="8"/>
       <c r="D75" s="9"/>
       <c r="E75" s="8"/>
@@ -1656,19 +1694,19 @@
       <c r="A76" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B76" s="34"/>
-      <c r="C76" s="35"/>
-      <c r="D76" s="35"/>
-      <c r="E76" s="36"/>
+      <c r="B76" s="30"/>
+      <c r="C76" s="31"/>
+      <c r="D76" s="31"/>
+      <c r="E76" s="32"/>
     </row>
     <row r="77" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="38" t="s">
+      <c r="A77" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="B77" s="39"/>
+      <c r="B77" s="34"/>
       <c r="C77" s="15">
         <f>MROUND(SUM(C6:C76) /60,0.2)</f>
-        <v>12.600000000000001</v>
+        <v>14.600000000000001</v>
       </c>
       <c r="D77" s="16"/>
       <c r="E77" s="17"/>
@@ -1683,15 +1721,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B76:E76"/>
-    <mergeCell ref="A77:B77"/>
-    <mergeCell ref="B53:B57"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B59:B63"/>
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="B65:B69"/>
-    <mergeCell ref="B70:E70"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -1708,6 +1737,15 @@
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="B41:B45"/>
     <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B76:E76"/>
+    <mergeCell ref="A77:B77"/>
+    <mergeCell ref="B53:B57"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="B65:B69"/>
+    <mergeCell ref="B70:E70"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C65:C69 C59:C63 C47:C51 C53:C57 C29:C33 B6 C6:C17 C35:C39 C41:C45 C71:C75 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1717,14 +1755,17 @@
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="E30" r:id="rId1" xr:uid="{F187DE9B-B8D0-41A3-8491-0AAD2D53ABFB}"/>
+  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="49" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="48" orientation="portrait" r:id="rId2"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
   </headerFooter>
-  <legacyDrawingHF r:id="rId2"/>
+  <legacyDrawingHF r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -1908,12 +1949,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -2075,6 +2110,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
@@ -2084,15 +2125,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2108,4 +2140,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
change model and update projec trepport
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4228423-44FD-4EFC-BC2A-226399F89347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8960A6F6-ABCE-45F6-82B7-FCE668246C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="66">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -246,6 +246,9 @@
   </si>
   <si>
     <t>http://weka.ch/themes/ressources-humaines/contrats-de-travail-et-reglements/protection-des-donnees/article/donnees-rh-quels-sont-les-delais-de-conservation-des-donnees-des-collaborateurs/</t>
+  </si>
+  <si>
+    <t>J'avais envie d'un peu avancer dans mon rapport et c'est ce que j'ai fait j'ai notement réaliser la partie des exigences et les maquettes (pas encore terminé)</t>
   </si>
 </sst>
 </file>
@@ -573,55 +576,55 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -955,10 +958,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="36"/>
+      <c r="C1" s="28"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -970,10 +973,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="36"/>
+      <c r="C2" s="28"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -985,10 +988,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="36"/>
+      <c r="C3" s="28"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1000,12 +1003,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="39"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="31"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1028,7 +1031,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="27">
+      <c r="B6" s="38">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1041,7 +1044,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="28"/>
+      <c r="B7" s="33"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1054,7 +1057,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="28"/>
+      <c r="B8" s="33"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1067,7 +1070,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="28"/>
+      <c r="B9" s="33"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1078,7 +1081,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="28"/>
+      <c r="B10" s="33"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1091,7 +1094,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="28"/>
+      <c r="B11" s="33"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1106,7 +1109,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="28"/>
+      <c r="B12" s="33"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1121,7 +1124,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="28"/>
+      <c r="B13" s="33"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1136,7 +1139,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="28"/>
+      <c r="B14" s="33"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1151,7 +1154,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="28"/>
+      <c r="B15" s="33"/>
       <c r="C15" s="10">
         <v>40</v>
       </c>
@@ -1166,7 +1169,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="28"/>
+      <c r="B16" s="33"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1179,7 +1182,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="29"/>
+      <c r="B17" s="34"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1188,19 +1191,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="30" t="str">
+      <c r="B18" s="35" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="32"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="37"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="27">
+      <c r="B19" s="38">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1215,7 +1218,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="28"/>
+      <c r="B20" s="33"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1228,7 +1231,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="28"/>
+      <c r="B21" s="33"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1242,7 +1245,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="28"/>
+      <c r="B22" s="33"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1255,7 +1258,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="28"/>
+      <c r="B23" s="33"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1268,7 +1271,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="28"/>
+      <c r="B24" s="33"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1281,7 +1284,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="28"/>
+      <c r="B25" s="33"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1294,7 +1297,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="28"/>
+      <c r="B26" s="33"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1307,7 +1310,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="29"/>
+      <c r="B27" s="34"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1320,19 +1323,19 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="30" t="str">
+      <c r="B28" s="35" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="32"/>
+      <c r="C28" s="36"/>
+      <c r="D28" s="36"/>
+      <c r="E28" s="37"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="27">
+      <c r="B29" s="38">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1347,34 +1350,40 @@
       <c r="A30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="28"/>
+      <c r="B30" s="33"/>
       <c r="C30" s="8">
         <v>60</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="E30" s="40" t="s">
+      <c r="E30" s="27" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="7"/>
-      <c r="B31" s="28"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="9"/>
+    <row r="31" spans="1:7" ht="27" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" s="33"/>
+      <c r="C31" s="8">
+        <v>70</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>65</v>
+      </c>
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="28"/>
+      <c r="B32" s="33"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="29"/>
+      <c r="B33" s="34"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1383,45 +1392,45 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="30" t="str">
+      <c r="B34" s="35" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
-        <v>2h0</v>
-      </c>
-      <c r="C34" s="31"/>
-      <c r="D34" s="31"/>
-      <c r="E34" s="32"/>
+        <v>3h10</v>
+      </c>
+      <c r="C34" s="36"/>
+      <c r="D34" s="36"/>
+      <c r="E34" s="37"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
-      <c r="B35" s="35"/>
+      <c r="B35" s="32"/>
       <c r="C35" s="5"/>
       <c r="D35" s="6"/>
       <c r="E35" s="5"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7"/>
-      <c r="B36" s="28"/>
+      <c r="B36" s="33"/>
       <c r="C36" s="8"/>
       <c r="D36" s="9"/>
       <c r="E36" s="8"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="28"/>
+      <c r="B37" s="33"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="7"/>
-      <c r="B38" s="28"/>
+      <c r="B38" s="33"/>
       <c r="C38" s="8"/>
       <c r="D38" s="9"/>
       <c r="E38" s="8"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="10"/>
-      <c r="B39" s="29"/>
+      <c r="B39" s="34"/>
       <c r="C39" s="10"/>
       <c r="D39" s="11"/>
       <c r="E39" s="10"/>
@@ -1430,42 +1439,42 @@
       <c r="A40" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B40" s="30"/>
-      <c r="C40" s="31"/>
-      <c r="D40" s="31"/>
-      <c r="E40" s="32"/>
+      <c r="B40" s="35"/>
+      <c r="C40" s="36"/>
+      <c r="D40" s="36"/>
+      <c r="E40" s="37"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="13"/>
-      <c r="B41" s="35"/>
+      <c r="B41" s="32"/>
       <c r="C41" s="13"/>
       <c r="D41" s="14"/>
       <c r="E41" s="13"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8"/>
-      <c r="B42" s="28"/>
+      <c r="B42" s="33"/>
       <c r="C42" s="8"/>
       <c r="D42" s="9"/>
       <c r="E42" s="8"/>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8"/>
-      <c r="B43" s="28"/>
+      <c r="B43" s="33"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8"/>
-      <c r="B44" s="28"/>
+      <c r="B44" s="33"/>
       <c r="C44" s="8"/>
       <c r="D44" s="9"/>
       <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="8"/>
-      <c r="B45" s="29"/>
+      <c r="B45" s="34"/>
       <c r="C45" s="8"/>
       <c r="D45" s="9"/>
       <c r="E45" s="8"/>
@@ -1474,42 +1483,42 @@
       <c r="A46" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="30"/>
-      <c r="C46" s="31"/>
-      <c r="D46" s="31"/>
-      <c r="E46" s="32"/>
+      <c r="B46" s="35"/>
+      <c r="C46" s="36"/>
+      <c r="D46" s="36"/>
+      <c r="E46" s="37"/>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="4"/>
-      <c r="B47" s="27"/>
+      <c r="B47" s="38"/>
       <c r="C47" s="5"/>
       <c r="D47" s="6"/>
       <c r="E47" s="5"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="7"/>
-      <c r="B48" s="28"/>
+      <c r="B48" s="33"/>
       <c r="C48" s="8"/>
       <c r="D48" s="9"/>
       <c r="E48" s="8"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="28"/>
+      <c r="B49" s="33"/>
       <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="28"/>
+      <c r="B50" s="33"/>
       <c r="C50" s="8"/>
       <c r="D50" s="9"/>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="10"/>
-      <c r="B51" s="29"/>
+      <c r="B51" s="34"/>
       <c r="C51" s="10"/>
       <c r="D51" s="11"/>
       <c r="E51" s="10"/>
@@ -1518,42 +1527,42 @@
       <c r="A52" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B52" s="30"/>
-      <c r="C52" s="31"/>
-      <c r="D52" s="31"/>
-      <c r="E52" s="32"/>
+      <c r="B52" s="35"/>
+      <c r="C52" s="36"/>
+      <c r="D52" s="36"/>
+      <c r="E52" s="37"/>
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4"/>
-      <c r="B53" s="35"/>
+      <c r="B53" s="32"/>
       <c r="C53" s="5"/>
       <c r="D53" s="6"/>
       <c r="E53" s="5"/>
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="7"/>
-      <c r="B54" s="28"/>
+      <c r="B54" s="33"/>
       <c r="C54" s="8"/>
       <c r="D54" s="9"/>
       <c r="E54" s="8"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="7"/>
-      <c r="B55" s="28"/>
+      <c r="B55" s="33"/>
       <c r="C55" s="8"/>
       <c r="D55" s="9"/>
       <c r="E55" s="8"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
-      <c r="B56" s="28"/>
+      <c r="B56" s="33"/>
       <c r="C56" s="8"/>
       <c r="D56" s="9"/>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="10"/>
-      <c r="B57" s="29"/>
+      <c r="B57" s="34"/>
       <c r="C57" s="10"/>
       <c r="D57" s="11"/>
       <c r="E57" s="10"/>
@@ -1562,42 +1571,42 @@
       <c r="A58" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B58" s="30"/>
-      <c r="C58" s="31"/>
-      <c r="D58" s="31"/>
-      <c r="E58" s="32"/>
+      <c r="B58" s="35"/>
+      <c r="C58" s="36"/>
+      <c r="D58" s="36"/>
+      <c r="E58" s="37"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4"/>
-      <c r="B59" s="35"/>
+      <c r="B59" s="32"/>
       <c r="C59" s="5"/>
       <c r="D59" s="6"/>
       <c r="E59" s="5"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="7"/>
-      <c r="B60" s="28"/>
+      <c r="B60" s="33"/>
       <c r="C60" s="8"/>
       <c r="D60" s="9"/>
       <c r="E60" s="8"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="7"/>
-      <c r="B61" s="28"/>
+      <c r="B61" s="33"/>
       <c r="C61" s="8"/>
       <c r="D61" s="9"/>
       <c r="E61" s="8"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="7"/>
-      <c r="B62" s="28"/>
+      <c r="B62" s="33"/>
       <c r="C62" s="8"/>
       <c r="D62" s="9"/>
       <c r="E62" s="8"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="10"/>
-      <c r="B63" s="29"/>
+      <c r="B63" s="34"/>
       <c r="C63" s="10"/>
       <c r="D63" s="11"/>
       <c r="E63" s="10"/>
@@ -1606,42 +1615,42 @@
       <c r="A64" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B64" s="30"/>
-      <c r="C64" s="31"/>
-      <c r="D64" s="31"/>
-      <c r="E64" s="32"/>
+      <c r="B64" s="35"/>
+      <c r="C64" s="36"/>
+      <c r="D64" s="36"/>
+      <c r="E64" s="37"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4"/>
-      <c r="B65" s="35"/>
+      <c r="B65" s="32"/>
       <c r="C65" s="5"/>
       <c r="D65" s="6"/>
       <c r="E65" s="5"/>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="7"/>
-      <c r="B66" s="28"/>
+      <c r="B66" s="33"/>
       <c r="C66" s="8"/>
       <c r="D66" s="9"/>
       <c r="E66" s="8"/>
     </row>
     <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="7"/>
-      <c r="B67" s="28"/>
+      <c r="B67" s="33"/>
       <c r="C67" s="8"/>
       <c r="D67" s="9"/>
       <c r="E67" s="8"/>
     </row>
     <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7"/>
-      <c r="B68" s="28"/>
+      <c r="B68" s="33"/>
       <c r="C68" s="8"/>
       <c r="D68" s="9"/>
       <c r="E68" s="8"/>
     </row>
     <row r="69" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="10"/>
-      <c r="B69" s="29"/>
+      <c r="B69" s="34"/>
       <c r="C69" s="10"/>
       <c r="D69" s="11"/>
       <c r="E69" s="10"/>
@@ -1650,42 +1659,42 @@
       <c r="A70" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B70" s="30"/>
-      <c r="C70" s="31"/>
-      <c r="D70" s="31"/>
-      <c r="E70" s="32"/>
+      <c r="B70" s="35"/>
+      <c r="C70" s="36"/>
+      <c r="D70" s="36"/>
+      <c r="E70" s="37"/>
     </row>
     <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="13"/>
-      <c r="B71" s="35"/>
+      <c r="B71" s="32"/>
       <c r="C71" s="13"/>
       <c r="D71" s="14"/>
       <c r="E71" s="13"/>
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8"/>
-      <c r="B72" s="28"/>
+      <c r="B72" s="33"/>
       <c r="C72" s="8"/>
       <c r="D72" s="9"/>
       <c r="E72" s="8"/>
     </row>
     <row r="73" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8"/>
-      <c r="B73" s="28"/>
+      <c r="B73" s="33"/>
       <c r="C73" s="8"/>
       <c r="D73" s="9"/>
       <c r="E73" s="8"/>
     </row>
     <row r="74" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8"/>
-      <c r="B74" s="28"/>
+      <c r="B74" s="33"/>
       <c r="C74" s="8"/>
       <c r="D74" s="9"/>
       <c r="E74" s="8"/>
     </row>
     <row r="75" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="8"/>
-      <c r="B75" s="29"/>
+      <c r="B75" s="34"/>
       <c r="C75" s="8"/>
       <c r="D75" s="9"/>
       <c r="E75" s="8"/>
@@ -1694,19 +1703,19 @@
       <c r="A76" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B76" s="30"/>
-      <c r="C76" s="31"/>
-      <c r="D76" s="31"/>
-      <c r="E76" s="32"/>
+      <c r="B76" s="35"/>
+      <c r="C76" s="36"/>
+      <c r="D76" s="36"/>
+      <c r="E76" s="37"/>
     </row>
     <row r="77" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="33" t="s">
+      <c r="A77" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B77" s="34"/>
+      <c r="B77" s="40"/>
       <c r="C77" s="15">
         <f>MROUND(SUM(C6:C76) /60,0.2)</f>
-        <v>14.600000000000001</v>
+        <v>15.600000000000001</v>
       </c>
       <c r="D77" s="16"/>
       <c r="E77" s="17"/>
@@ -1721,6 +1730,15 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B76:E76"/>
+    <mergeCell ref="A77:B77"/>
+    <mergeCell ref="B53:B57"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="B65:B69"/>
+    <mergeCell ref="B70:E70"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -1737,15 +1755,6 @@
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="B41:B45"/>
     <mergeCell ref="B46:E46"/>
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B76:E76"/>
-    <mergeCell ref="A77:B77"/>
-    <mergeCell ref="B53:B57"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B59:B63"/>
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="B65:B69"/>
-    <mergeCell ref="B70:E70"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C65:C69 C59:C63 C47:C51 C53:C57 C29:C33 B6 C6:C17 C35:C39 C41:C45 C71:C75 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1760,7 +1769,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="48" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="47" orientation="portrait" r:id="rId2"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -1887,7 +1896,8 @@
         <v>1.0416666666666666E-2</v>
       </c>
       <c r="I9" s="26">
-        <v>0.13194444444444445</v>
+        <f>G9-F9-H9</f>
+        <v>0.13194444444444439</v>
       </c>
     </row>
     <row r="10" spans="3:9" x14ac:dyDescent="0.25">
@@ -1949,6 +1959,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -2110,12 +2126,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
@@ -2125,6 +2135,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2140,13 +2159,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor(global): change tables names and update project repport
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8960A6F6-ABCE-45F6-82B7-FCE668246C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C94FED5-7F74-40F8-BF80-CD352340E467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="68">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -249,6 +249,12 @@
   </si>
   <si>
     <t>J'avais envie d'un peu avancer dans mon rapport et c'est ce que j'ai fait j'ai notement réaliser la partie des exigences et les maquettes (pas encore terminé)</t>
+  </si>
+  <si>
+    <t>J'ai pas mal avancé sur mon rapport j'ai notament modifié certaines choses dans la partie maqeutte (par ex mettre les légendes) et j'ai commencé/ bien avancé dans la aprtie de la base de donnée</t>
+  </si>
+  <si>
+    <t>J'ai continué mon rapport où j'explique notament chaque table de la DB avec leurs relations</t>
   </si>
 </sst>
 </file>
@@ -580,51 +586,51 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -958,10 +964,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="28"/>
+      <c r="C1" s="37"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -973,10 +979,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="28"/>
+      <c r="C2" s="37"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -988,10 +994,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="28"/>
+      <c r="C3" s="37"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1003,12 +1009,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="31"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="40"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1031,7 +1037,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="38">
+      <c r="B6" s="28">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1044,7 +1050,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="33"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1057,7 +1063,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="33"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1070,7 +1076,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="33"/>
+      <c r="B9" s="29"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1081,7 +1087,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="33"/>
+      <c r="B10" s="29"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1094,7 +1100,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="33"/>
+      <c r="B11" s="29"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1109,7 +1115,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="33"/>
+      <c r="B12" s="29"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1124,7 +1130,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="33"/>
+      <c r="B13" s="29"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1139,7 +1145,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="33"/>
+      <c r="B14" s="29"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1154,7 +1160,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="33"/>
+      <c r="B15" s="29"/>
       <c r="C15" s="10">
         <v>40</v>
       </c>
@@ -1169,7 +1175,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="33"/>
+      <c r="B16" s="29"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1182,7 +1188,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="34"/>
+      <c r="B17" s="30"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1191,19 +1197,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="35" t="str">
+      <c r="B18" s="31" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="37"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="33"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="38">
+      <c r="B19" s="28">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1218,7 +1224,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="33"/>
+      <c r="B20" s="29"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1231,7 +1237,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="33"/>
+      <c r="B21" s="29"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1245,7 +1251,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="33"/>
+      <c r="B22" s="29"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1258,7 +1264,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="33"/>
+      <c r="B23" s="29"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1271,7 +1277,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="33"/>
+      <c r="B24" s="29"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1284,7 +1290,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="33"/>
+      <c r="B25" s="29"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1297,7 +1303,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="33"/>
+      <c r="B26" s="29"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1310,7 +1316,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="34"/>
+      <c r="B27" s="30"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1323,19 +1329,19 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="35" t="str">
+      <c r="B28" s="31" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="36"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="37"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="33"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="38">
+      <c r="B29" s="28">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1350,7 +1356,7 @@
       <c r="A30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="33"/>
+      <c r="B30" s="29"/>
       <c r="C30" s="8">
         <v>60</v>
       </c>
@@ -1365,7 +1371,7 @@
       <c r="A31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="33"/>
+      <c r="B31" s="29"/>
       <c r="C31" s="8">
         <v>70</v>
       </c>
@@ -1376,14 +1382,14 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="33"/>
+      <c r="B32" s="29"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="34"/>
+      <c r="B33" s="30"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1392,45 +1398,59 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="35" t="str">
+      <c r="B34" s="31" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C34" s="36"/>
-      <c r="D34" s="36"/>
-      <c r="E34" s="37"/>
-    </row>
-    <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="4"/>
-      <c r="B35" s="32"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="6"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="33"/>
+    </row>
+    <row r="35" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B35" s="28">
+        <v>46143</v>
+      </c>
+      <c r="C35" s="5">
+        <v>60</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>66</v>
+      </c>
       <c r="E35" s="5"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="7"/>
-      <c r="B36" s="33"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="9"/>
+      <c r="A36" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="29"/>
+      <c r="C36" s="8">
+        <v>35</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>67</v>
+      </c>
       <c r="E36" s="8"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="33"/>
+      <c r="B37" s="29"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="7"/>
-      <c r="B38" s="33"/>
+      <c r="B38" s="29"/>
       <c r="C38" s="8"/>
       <c r="D38" s="9"/>
       <c r="E38" s="8"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="10"/>
-      <c r="B39" s="34"/>
+      <c r="B39" s="30"/>
       <c r="C39" s="10"/>
       <c r="D39" s="11"/>
       <c r="E39" s="10"/>
@@ -1439,42 +1459,45 @@
       <c r="A40" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B40" s="35"/>
-      <c r="C40" s="36"/>
-      <c r="D40" s="36"/>
-      <c r="E40" s="37"/>
+      <c r="B40" s="31" t="str">
+        <f>INT(SUM(C35:C39)/60)&amp;"h"&amp;MOD(SUM(C35:C39),60)</f>
+        <v>1h35</v>
+      </c>
+      <c r="C40" s="32"/>
+      <c r="D40" s="32"/>
+      <c r="E40" s="33"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="13"/>
-      <c r="B41" s="32"/>
+      <c r="B41" s="36"/>
       <c r="C41" s="13"/>
       <c r="D41" s="14"/>
       <c r="E41" s="13"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8"/>
-      <c r="B42" s="33"/>
+      <c r="B42" s="29"/>
       <c r="C42" s="8"/>
       <c r="D42" s="9"/>
       <c r="E42" s="8"/>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8"/>
-      <c r="B43" s="33"/>
+      <c r="B43" s="29"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8"/>
-      <c r="B44" s="33"/>
+      <c r="B44" s="29"/>
       <c r="C44" s="8"/>
       <c r="D44" s="9"/>
       <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="8"/>
-      <c r="B45" s="34"/>
+      <c r="B45" s="30"/>
       <c r="C45" s="8"/>
       <c r="D45" s="9"/>
       <c r="E45" s="8"/>
@@ -1483,42 +1506,42 @@
       <c r="A46" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="35"/>
-      <c r="C46" s="36"/>
-      <c r="D46" s="36"/>
-      <c r="E46" s="37"/>
+      <c r="B46" s="31"/>
+      <c r="C46" s="32"/>
+      <c r="D46" s="32"/>
+      <c r="E46" s="33"/>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="4"/>
-      <c r="B47" s="38"/>
+      <c r="B47" s="28"/>
       <c r="C47" s="5"/>
       <c r="D47" s="6"/>
       <c r="E47" s="5"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="7"/>
-      <c r="B48" s="33"/>
+      <c r="B48" s="29"/>
       <c r="C48" s="8"/>
       <c r="D48" s="9"/>
       <c r="E48" s="8"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="33"/>
+      <c r="B49" s="29"/>
       <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="33"/>
+      <c r="B50" s="29"/>
       <c r="C50" s="8"/>
       <c r="D50" s="9"/>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="10"/>
-      <c r="B51" s="34"/>
+      <c r="B51" s="30"/>
       <c r="C51" s="10"/>
       <c r="D51" s="11"/>
       <c r="E51" s="10"/>
@@ -1527,42 +1550,42 @@
       <c r="A52" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B52" s="35"/>
-      <c r="C52" s="36"/>
-      <c r="D52" s="36"/>
-      <c r="E52" s="37"/>
+      <c r="B52" s="31"/>
+      <c r="C52" s="32"/>
+      <c r="D52" s="32"/>
+      <c r="E52" s="33"/>
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4"/>
-      <c r="B53" s="32"/>
+      <c r="B53" s="36"/>
       <c r="C53" s="5"/>
       <c r="D53" s="6"/>
       <c r="E53" s="5"/>
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="7"/>
-      <c r="B54" s="33"/>
+      <c r="B54" s="29"/>
       <c r="C54" s="8"/>
       <c r="D54" s="9"/>
       <c r="E54" s="8"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="7"/>
-      <c r="B55" s="33"/>
+      <c r="B55" s="29"/>
       <c r="C55" s="8"/>
       <c r="D55" s="9"/>
       <c r="E55" s="8"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
-      <c r="B56" s="33"/>
+      <c r="B56" s="29"/>
       <c r="C56" s="8"/>
       <c r="D56" s="9"/>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="10"/>
-      <c r="B57" s="34"/>
+      <c r="B57" s="30"/>
       <c r="C57" s="10"/>
       <c r="D57" s="11"/>
       <c r="E57" s="10"/>
@@ -1571,42 +1594,42 @@
       <c r="A58" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B58" s="35"/>
-      <c r="C58" s="36"/>
-      <c r="D58" s="36"/>
-      <c r="E58" s="37"/>
+      <c r="B58" s="31"/>
+      <c r="C58" s="32"/>
+      <c r="D58" s="32"/>
+      <c r="E58" s="33"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4"/>
-      <c r="B59" s="32"/>
+      <c r="B59" s="36"/>
       <c r="C59" s="5"/>
       <c r="D59" s="6"/>
       <c r="E59" s="5"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="7"/>
-      <c r="B60" s="33"/>
+      <c r="B60" s="29"/>
       <c r="C60" s="8"/>
       <c r="D60" s="9"/>
       <c r="E60" s="8"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="7"/>
-      <c r="B61" s="33"/>
+      <c r="B61" s="29"/>
       <c r="C61" s="8"/>
       <c r="D61" s="9"/>
       <c r="E61" s="8"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="7"/>
-      <c r="B62" s="33"/>
+      <c r="B62" s="29"/>
       <c r="C62" s="8"/>
       <c r="D62" s="9"/>
       <c r="E62" s="8"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="10"/>
-      <c r="B63" s="34"/>
+      <c r="B63" s="30"/>
       <c r="C63" s="10"/>
       <c r="D63" s="11"/>
       <c r="E63" s="10"/>
@@ -1615,42 +1638,42 @@
       <c r="A64" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B64" s="35"/>
-      <c r="C64" s="36"/>
-      <c r="D64" s="36"/>
-      <c r="E64" s="37"/>
+      <c r="B64" s="31"/>
+      <c r="C64" s="32"/>
+      <c r="D64" s="32"/>
+      <c r="E64" s="33"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4"/>
-      <c r="B65" s="32"/>
+      <c r="B65" s="36"/>
       <c r="C65" s="5"/>
       <c r="D65" s="6"/>
       <c r="E65" s="5"/>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="7"/>
-      <c r="B66" s="33"/>
+      <c r="B66" s="29"/>
       <c r="C66" s="8"/>
       <c r="D66" s="9"/>
       <c r="E66" s="8"/>
     </row>
     <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="7"/>
-      <c r="B67" s="33"/>
+      <c r="B67" s="29"/>
       <c r="C67" s="8"/>
       <c r="D67" s="9"/>
       <c r="E67" s="8"/>
     </row>
     <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7"/>
-      <c r="B68" s="33"/>
+      <c r="B68" s="29"/>
       <c r="C68" s="8"/>
       <c r="D68" s="9"/>
       <c r="E68" s="8"/>
     </row>
     <row r="69" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="10"/>
-      <c r="B69" s="34"/>
+      <c r="B69" s="30"/>
       <c r="C69" s="10"/>
       <c r="D69" s="11"/>
       <c r="E69" s="10"/>
@@ -1659,42 +1682,42 @@
       <c r="A70" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B70" s="35"/>
-      <c r="C70" s="36"/>
-      <c r="D70" s="36"/>
-      <c r="E70" s="37"/>
+      <c r="B70" s="31"/>
+      <c r="C70" s="32"/>
+      <c r="D70" s="32"/>
+      <c r="E70" s="33"/>
     </row>
     <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="13"/>
-      <c r="B71" s="32"/>
+      <c r="B71" s="36"/>
       <c r="C71" s="13"/>
       <c r="D71" s="14"/>
       <c r="E71" s="13"/>
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8"/>
-      <c r="B72" s="33"/>
+      <c r="B72" s="29"/>
       <c r="C72" s="8"/>
       <c r="D72" s="9"/>
       <c r="E72" s="8"/>
     </row>
     <row r="73" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8"/>
-      <c r="B73" s="33"/>
+      <c r="B73" s="29"/>
       <c r="C73" s="8"/>
       <c r="D73" s="9"/>
       <c r="E73" s="8"/>
     </row>
     <row r="74" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8"/>
-      <c r="B74" s="33"/>
+      <c r="B74" s="29"/>
       <c r="C74" s="8"/>
       <c r="D74" s="9"/>
       <c r="E74" s="8"/>
     </row>
     <row r="75" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="8"/>
-      <c r="B75" s="34"/>
+      <c r="B75" s="30"/>
       <c r="C75" s="8"/>
       <c r="D75" s="9"/>
       <c r="E75" s="8"/>
@@ -1703,19 +1726,19 @@
       <c r="A76" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B76" s="35"/>
-      <c r="C76" s="36"/>
-      <c r="D76" s="36"/>
-      <c r="E76" s="37"/>
+      <c r="B76" s="31"/>
+      <c r="C76" s="32"/>
+      <c r="D76" s="32"/>
+      <c r="E76" s="33"/>
     </row>
     <row r="77" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="39" t="s">
+      <c r="A77" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="B77" s="40"/>
+      <c r="B77" s="35"/>
       <c r="C77" s="15">
         <f>MROUND(SUM(C6:C76) /60,0.2)</f>
-        <v>15.600000000000001</v>
+        <v>17.2</v>
       </c>
       <c r="D77" s="16"/>
       <c r="E77" s="17"/>
@@ -1730,15 +1753,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B76:E76"/>
-    <mergeCell ref="A77:B77"/>
-    <mergeCell ref="B53:B57"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B59:B63"/>
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="B65:B69"/>
-    <mergeCell ref="B70:E70"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -1755,6 +1769,15 @@
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="B41:B45"/>
     <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B76:E76"/>
+    <mergeCell ref="A77:B77"/>
+    <mergeCell ref="B53:B57"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="B65:B69"/>
+    <mergeCell ref="B70:E70"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C65:C69 C59:C63 C47:C51 C53:C57 C29:C33 B6 C6:C17 C35:C39 C41:C45 C71:C75 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1959,12 +1982,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -2126,6 +2143,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
@@ -2135,15 +2158,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2159,4 +2173,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor(doc): update JDT and project repport
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C94FED5-7F74-40F8-BF80-CD352340E467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DC4E4BF-9A14-4309-A167-A3A96F0376E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="71">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -255,6 +255,15 @@
   </si>
   <si>
     <t>J'ai continué mon rapport où j'explique notament chaque table de la DB avec leurs relations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai continué mon rapport </t>
+  </si>
+  <si>
+    <t>J'ai avancé dans mon rapport j'ai notament fait la partie explication du système d'auth des admin et la aprtie des choix technnique</t>
+  </si>
+  <si>
+    <t>11h20</t>
   </si>
 </sst>
 </file>
@@ -586,51 +595,51 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -964,10 +973,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="37" t="s">
+      <c r="B1" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="37"/>
+      <c r="C1" s="28"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -979,10 +988,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="37"/>
+      <c r="C2" s="28"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -994,10 +1003,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="B3" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="37"/>
+      <c r="C3" s="28"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1009,12 +1018,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="40"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="31"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1037,7 +1046,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="28">
+      <c r="B6" s="38">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1050,7 +1059,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="29"/>
+      <c r="B7" s="33"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1063,7 +1072,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="29"/>
+      <c r="B8" s="33"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1076,7 +1085,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="29"/>
+      <c r="B9" s="33"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1087,7 +1096,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="29"/>
+      <c r="B10" s="33"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1100,7 +1109,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="29"/>
+      <c r="B11" s="33"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1115,7 +1124,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="29"/>
+      <c r="B12" s="33"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1130,7 +1139,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="29"/>
+      <c r="B13" s="33"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1145,7 +1154,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="29"/>
+      <c r="B14" s="33"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1160,7 +1169,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="29"/>
+      <c r="B15" s="33"/>
       <c r="C15" s="10">
         <v>40</v>
       </c>
@@ -1175,7 +1184,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="29"/>
+      <c r="B16" s="33"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1188,7 +1197,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="30"/>
+      <c r="B17" s="34"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1197,19 +1206,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="31" t="str">
+      <c r="B18" s="35" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="33"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="37"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="28">
+      <c r="B19" s="38">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1224,7 +1233,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="29"/>
+      <c r="B20" s="33"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1237,7 +1246,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="29"/>
+      <c r="B21" s="33"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1251,7 +1260,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="29"/>
+      <c r="B22" s="33"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1264,7 +1273,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="29"/>
+      <c r="B23" s="33"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1277,7 +1286,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="29"/>
+      <c r="B24" s="33"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1290,7 +1299,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="29"/>
+      <c r="B25" s="33"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1303,7 +1312,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="29"/>
+      <c r="B26" s="33"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1316,7 +1325,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="30"/>
+      <c r="B27" s="34"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1329,19 +1338,19 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="31" t="str">
+      <c r="B28" s="35" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="33"/>
+      <c r="C28" s="36"/>
+      <c r="D28" s="36"/>
+      <c r="E28" s="37"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="28">
+      <c r="B29" s="38">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1356,7 +1365,7 @@
       <c r="A30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="29"/>
+      <c r="B30" s="33"/>
       <c r="C30" s="8">
         <v>60</v>
       </c>
@@ -1371,7 +1380,7 @@
       <c r="A31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="29"/>
+      <c r="B31" s="33"/>
       <c r="C31" s="8">
         <v>70</v>
       </c>
@@ -1382,14 +1391,14 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="29"/>
+      <c r="B32" s="33"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="30"/>
+      <c r="B33" s="34"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1398,19 +1407,19 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="31" t="str">
+      <c r="B34" s="35" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C34" s="32"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="33"/>
+      <c r="C34" s="36"/>
+      <c r="D34" s="36"/>
+      <c r="E34" s="37"/>
     </row>
     <row r="35" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="28">
+      <c r="B35" s="38">
         <v>46143</v>
       </c>
       <c r="C35" s="5">
@@ -1425,7 +1434,7 @@
       <c r="A36" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="29"/>
+      <c r="B36" s="33"/>
       <c r="C36" s="8">
         <v>35</v>
       </c>
@@ -1435,22 +1444,36 @@
       <c r="E36" s="8"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="7"/>
-      <c r="B37" s="29"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="9"/>
+      <c r="A37" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37" s="33"/>
+      <c r="C37" s="8">
+        <v>60</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>68</v>
+      </c>
       <c r="E37" s="8"/>
     </row>
-    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="7"/>
-      <c r="B38" s="29"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="8"/>
+    <row r="38" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A38" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B38" s="33"/>
+      <c r="C38" s="8">
+        <v>30</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="10"/>
-      <c r="B39" s="30"/>
+      <c r="B39" s="34"/>
       <c r="C39" s="10"/>
       <c r="D39" s="11"/>
       <c r="E39" s="10"/>
@@ -1459,45 +1482,45 @@
       <c r="A40" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B40" s="31" t="str">
+      <c r="B40" s="35" t="str">
         <f>INT(SUM(C35:C39)/60)&amp;"h"&amp;MOD(SUM(C35:C39),60)</f>
-        <v>1h35</v>
-      </c>
-      <c r="C40" s="32"/>
-      <c r="D40" s="32"/>
-      <c r="E40" s="33"/>
+        <v>3h5</v>
+      </c>
+      <c r="C40" s="36"/>
+      <c r="D40" s="36"/>
+      <c r="E40" s="37"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="13"/>
-      <c r="B41" s="36"/>
+      <c r="B41" s="32"/>
       <c r="C41" s="13"/>
       <c r="D41" s="14"/>
       <c r="E41" s="13"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8"/>
-      <c r="B42" s="29"/>
+      <c r="B42" s="33"/>
       <c r="C42" s="8"/>
       <c r="D42" s="9"/>
       <c r="E42" s="8"/>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8"/>
-      <c r="B43" s="29"/>
+      <c r="B43" s="33"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8"/>
-      <c r="B44" s="29"/>
+      <c r="B44" s="33"/>
       <c r="C44" s="8"/>
       <c r="D44" s="9"/>
       <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="8"/>
-      <c r="B45" s="30"/>
+      <c r="B45" s="34"/>
       <c r="C45" s="8"/>
       <c r="D45" s="9"/>
       <c r="E45" s="8"/>
@@ -1506,42 +1529,42 @@
       <c r="A46" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="31"/>
-      <c r="C46" s="32"/>
-      <c r="D46" s="32"/>
-      <c r="E46" s="33"/>
+      <c r="B46" s="35"/>
+      <c r="C46" s="36"/>
+      <c r="D46" s="36"/>
+      <c r="E46" s="37"/>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="4"/>
-      <c r="B47" s="28"/>
+      <c r="B47" s="38"/>
       <c r="C47" s="5"/>
       <c r="D47" s="6"/>
       <c r="E47" s="5"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="7"/>
-      <c r="B48" s="29"/>
+      <c r="B48" s="33"/>
       <c r="C48" s="8"/>
       <c r="D48" s="9"/>
       <c r="E48" s="8"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="29"/>
+      <c r="B49" s="33"/>
       <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="29"/>
+      <c r="B50" s="33"/>
       <c r="C50" s="8"/>
       <c r="D50" s="9"/>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="10"/>
-      <c r="B51" s="30"/>
+      <c r="B51" s="34"/>
       <c r="C51" s="10"/>
       <c r="D51" s="11"/>
       <c r="E51" s="10"/>
@@ -1550,42 +1573,42 @@
       <c r="A52" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B52" s="31"/>
-      <c r="C52" s="32"/>
-      <c r="D52" s="32"/>
-      <c r="E52" s="33"/>
+      <c r="B52" s="35"/>
+      <c r="C52" s="36"/>
+      <c r="D52" s="36"/>
+      <c r="E52" s="37"/>
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4"/>
-      <c r="B53" s="36"/>
+      <c r="B53" s="32"/>
       <c r="C53" s="5"/>
       <c r="D53" s="6"/>
       <c r="E53" s="5"/>
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="7"/>
-      <c r="B54" s="29"/>
+      <c r="B54" s="33"/>
       <c r="C54" s="8"/>
       <c r="D54" s="9"/>
       <c r="E54" s="8"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="7"/>
-      <c r="B55" s="29"/>
+      <c r="B55" s="33"/>
       <c r="C55" s="8"/>
       <c r="D55" s="9"/>
       <c r="E55" s="8"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
-      <c r="B56" s="29"/>
+      <c r="B56" s="33"/>
       <c r="C56" s="8"/>
       <c r="D56" s="9"/>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="10"/>
-      <c r="B57" s="30"/>
+      <c r="B57" s="34"/>
       <c r="C57" s="10"/>
       <c r="D57" s="11"/>
       <c r="E57" s="10"/>
@@ -1594,42 +1617,42 @@
       <c r="A58" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B58" s="31"/>
-      <c r="C58" s="32"/>
-      <c r="D58" s="32"/>
-      <c r="E58" s="33"/>
+      <c r="B58" s="35"/>
+      <c r="C58" s="36"/>
+      <c r="D58" s="36"/>
+      <c r="E58" s="37"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4"/>
-      <c r="B59" s="36"/>
+      <c r="B59" s="32"/>
       <c r="C59" s="5"/>
       <c r="D59" s="6"/>
       <c r="E59" s="5"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="7"/>
-      <c r="B60" s="29"/>
+      <c r="B60" s="33"/>
       <c r="C60" s="8"/>
       <c r="D60" s="9"/>
       <c r="E60" s="8"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="7"/>
-      <c r="B61" s="29"/>
+      <c r="B61" s="33"/>
       <c r="C61" s="8"/>
       <c r="D61" s="9"/>
       <c r="E61" s="8"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="7"/>
-      <c r="B62" s="29"/>
+      <c r="B62" s="33"/>
       <c r="C62" s="8"/>
       <c r="D62" s="9"/>
       <c r="E62" s="8"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="10"/>
-      <c r="B63" s="30"/>
+      <c r="B63" s="34"/>
       <c r="C63" s="10"/>
       <c r="D63" s="11"/>
       <c r="E63" s="10"/>
@@ -1638,42 +1661,42 @@
       <c r="A64" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B64" s="31"/>
-      <c r="C64" s="32"/>
-      <c r="D64" s="32"/>
-      <c r="E64" s="33"/>
+      <c r="B64" s="35"/>
+      <c r="C64" s="36"/>
+      <c r="D64" s="36"/>
+      <c r="E64" s="37"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4"/>
-      <c r="B65" s="36"/>
+      <c r="B65" s="32"/>
       <c r="C65" s="5"/>
       <c r="D65" s="6"/>
       <c r="E65" s="5"/>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="7"/>
-      <c r="B66" s="29"/>
+      <c r="B66" s="33"/>
       <c r="C66" s="8"/>
       <c r="D66" s="9"/>
       <c r="E66" s="8"/>
     </row>
     <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="7"/>
-      <c r="B67" s="29"/>
+      <c r="B67" s="33"/>
       <c r="C67" s="8"/>
       <c r="D67" s="9"/>
       <c r="E67" s="8"/>
     </row>
     <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7"/>
-      <c r="B68" s="29"/>
+      <c r="B68" s="33"/>
       <c r="C68" s="8"/>
       <c r="D68" s="9"/>
       <c r="E68" s="8"/>
     </row>
     <row r="69" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="10"/>
-      <c r="B69" s="30"/>
+      <c r="B69" s="34"/>
       <c r="C69" s="10"/>
       <c r="D69" s="11"/>
       <c r="E69" s="10"/>
@@ -1682,42 +1705,42 @@
       <c r="A70" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B70" s="31"/>
-      <c r="C70" s="32"/>
-      <c r="D70" s="32"/>
-      <c r="E70" s="33"/>
+      <c r="B70" s="35"/>
+      <c r="C70" s="36"/>
+      <c r="D70" s="36"/>
+      <c r="E70" s="37"/>
     </row>
     <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="13"/>
-      <c r="B71" s="36"/>
+      <c r="B71" s="32"/>
       <c r="C71" s="13"/>
       <c r="D71" s="14"/>
       <c r="E71" s="13"/>
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8"/>
-      <c r="B72" s="29"/>
+      <c r="B72" s="33"/>
       <c r="C72" s="8"/>
       <c r="D72" s="9"/>
       <c r="E72" s="8"/>
     </row>
     <row r="73" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8"/>
-      <c r="B73" s="29"/>
+      <c r="B73" s="33"/>
       <c r="C73" s="8"/>
       <c r="D73" s="9"/>
       <c r="E73" s="8"/>
     </row>
     <row r="74" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8"/>
-      <c r="B74" s="29"/>
+      <c r="B74" s="33"/>
       <c r="C74" s="8"/>
       <c r="D74" s="9"/>
       <c r="E74" s="8"/>
     </row>
     <row r="75" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="8"/>
-      <c r="B75" s="30"/>
+      <c r="B75" s="34"/>
       <c r="C75" s="8"/>
       <c r="D75" s="9"/>
       <c r="E75" s="8"/>
@@ -1726,19 +1749,19 @@
       <c r="A76" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B76" s="31"/>
-      <c r="C76" s="32"/>
-      <c r="D76" s="32"/>
-      <c r="E76" s="33"/>
+      <c r="B76" s="35"/>
+      <c r="C76" s="36"/>
+      <c r="D76" s="36"/>
+      <c r="E76" s="37"/>
     </row>
     <row r="77" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="34" t="s">
+      <c r="A77" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B77" s="35"/>
+      <c r="B77" s="40"/>
       <c r="C77" s="15">
         <f>MROUND(SUM(C6:C76) /60,0.2)</f>
-        <v>17.2</v>
+        <v>18.8</v>
       </c>
       <c r="D77" s="16"/>
       <c r="E77" s="17"/>
@@ -1753,6 +1776,15 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B76:E76"/>
+    <mergeCell ref="A77:B77"/>
+    <mergeCell ref="B53:B57"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="B65:B69"/>
+    <mergeCell ref="B70:E70"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -1769,15 +1801,6 @@
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="B41:B45"/>
     <mergeCell ref="B46:E46"/>
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B76:E76"/>
-    <mergeCell ref="A77:B77"/>
-    <mergeCell ref="B53:B57"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B59:B63"/>
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="B65:B69"/>
-    <mergeCell ref="B70:E70"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C65:C69 C59:C63 C47:C51 C53:C57 C29:C33 B6 C6:C17 C35:C39 C41:C45 C71:C75 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1954,17 +1977,17 @@
         <v>0.95138888888888884</v>
       </c>
     </row>
+    <row r="16" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="E16" s="26">
+        <f>E10-D10-(H10/2)</f>
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
     <row r="19" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E19" s="26">
-        <f>E6-D6-H6/2</f>
-        <v>0.13194444444444445</v>
-      </c>
+      <c r="E19" s="26"/>
     </row>
     <row r="20" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E20" s="26">
-        <f>E8-D8-(H8/2)</f>
-        <v>0.16666666666666666</v>
-      </c>
+      <c r="E20" s="26"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1982,6 +2005,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -2143,12 +2172,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
@@ -2158,6 +2181,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2173,13 +2205,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(app): finish lobby page
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DC4E4BF-9A14-4309-A167-A3A96F0376E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEF1CADE-DDCB-427A-BEED-CDBF20E49B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$77</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$81</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="76">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -263,7 +263,22 @@
     <t>J'ai avancé dans mon rapport j'ai notament fait la partie explication du système d'auth des admin et la aprtie des choix technnique</t>
   </si>
   <si>
-    <t>11h20</t>
+    <t>Système de login</t>
+  </si>
+  <si>
+    <t>J'ai fait le système de login pour les admins</t>
+  </si>
+  <si>
+    <t>Dashboard</t>
+  </si>
+  <si>
+    <t>J'ai commencé le dashboard</t>
+  </si>
+  <si>
+    <t>J'ai fais l'affichage des datas dans le dashboard</t>
+  </si>
+  <si>
+    <t>J'ai terminé la page d'accueil du dashboard</t>
   </si>
 </sst>
 </file>
@@ -503,7 +518,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -592,6 +607,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -957,7 +976,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -973,10 +992,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="28"/>
+      <c r="C1" s="29"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -988,10 +1007,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="28"/>
+      <c r="C2" s="29"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -1003,10 +1022,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="28"/>
+      <c r="C3" s="29"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1018,12 +1037,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="32"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1046,7 +1065,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="38">
+      <c r="B6" s="39">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1059,7 +1078,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="33"/>
+      <c r="B7" s="34"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1072,7 +1091,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="33"/>
+      <c r="B8" s="34"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1085,7 +1104,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="33"/>
+      <c r="B9" s="34"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1096,7 +1115,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="33"/>
+      <c r="B10" s="34"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1109,7 +1128,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="33"/>
+      <c r="B11" s="34"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1124,7 +1143,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="33"/>
+      <c r="B12" s="34"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1139,7 +1158,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="33"/>
+      <c r="B13" s="34"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1154,7 +1173,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="33"/>
+      <c r="B14" s="34"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1169,7 +1188,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="33"/>
+      <c r="B15" s="34"/>
       <c r="C15" s="10">
         <v>40</v>
       </c>
@@ -1184,7 +1203,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="33"/>
+      <c r="B16" s="34"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1197,7 +1216,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="34"/>
+      <c r="B17" s="35"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1206,19 +1225,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="35" t="str">
+      <c r="B18" s="36" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="38"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="38">
+      <c r="B19" s="39">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1233,7 +1252,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="33"/>
+      <c r="B20" s="34"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1246,7 +1265,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="33"/>
+      <c r="B21" s="34"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1260,7 +1279,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="33"/>
+      <c r="B22" s="34"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1273,7 +1292,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="33"/>
+      <c r="B23" s="34"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1286,7 +1305,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="33"/>
+      <c r="B24" s="34"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1299,7 +1318,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="33"/>
+      <c r="B25" s="34"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1312,7 +1331,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="33"/>
+      <c r="B26" s="34"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1325,7 +1344,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="34"/>
+      <c r="B27" s="35"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1338,19 +1357,19 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="35" t="str">
+      <c r="B28" s="36" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="36"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="37"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="38"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="38">
+      <c r="B29" s="39">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1365,7 +1384,7 @@
       <c r="A30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="33"/>
+      <c r="B30" s="34"/>
       <c r="C30" s="8">
         <v>60</v>
       </c>
@@ -1380,7 +1399,7 @@
       <c r="A31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="33"/>
+      <c r="B31" s="34"/>
       <c r="C31" s="8">
         <v>70</v>
       </c>
@@ -1391,14 +1410,14 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="33"/>
+      <c r="B32" s="34"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="34"/>
+      <c r="B33" s="35"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1407,19 +1426,19 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="35" t="str">
+      <c r="B34" s="36" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C34" s="36"/>
-      <c r="D34" s="36"/>
-      <c r="E34" s="37"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="38"/>
     </row>
     <row r="35" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="38">
+      <c r="B35" s="39">
         <v>46143</v>
       </c>
       <c r="C35" s="5">
@@ -1434,7 +1453,7 @@
       <c r="A36" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="33"/>
+      <c r="B36" s="34"/>
       <c r="C36" s="8">
         <v>35</v>
       </c>
@@ -1447,7 +1466,7 @@
       <c r="A37" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="33"/>
+      <c r="B37" s="34"/>
       <c r="C37" s="8">
         <v>60</v>
       </c>
@@ -1460,353 +1479,403 @@
       <c r="A38" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="33"/>
+      <c r="B38" s="34"/>
       <c r="C38" s="8">
         <v>30</v>
       </c>
       <c r="D38" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="E38" s="8" t="s">
+      <c r="E38" s="8"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="28" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="10"/>
       <c r="B39" s="34"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="11"/>
+      <c r="C39" s="10">
+        <v>35</v>
+      </c>
+      <c r="D39" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="E39" s="10"/>
     </row>
-    <row r="40" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="12" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B40" s="34"/>
+      <c r="C40" s="10">
+        <v>20</v>
+      </c>
+      <c r="D40" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E40" s="10"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B41" s="34"/>
+      <c r="C41" s="10">
+        <v>50</v>
+      </c>
+      <c r="D41" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="E41" s="10"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B42" s="34"/>
+      <c r="C42" s="10">
+        <v>45</v>
+      </c>
+      <c r="D42" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="E42" s="10"/>
+    </row>
+    <row r="43" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="10"/>
+      <c r="B43" s="35"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="10"/>
+    </row>
+    <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B40" s="35" t="str">
-        <f>INT(SUM(C35:C39)/60)&amp;"h"&amp;MOD(SUM(C35:C39),60)</f>
-        <v>3h5</v>
-      </c>
-      <c r="C40" s="36"/>
-      <c r="D40" s="36"/>
-      <c r="E40" s="37"/>
-    </row>
-    <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="13"/>
-      <c r="B41" s="32"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="13"/>
-    </row>
-    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="8"/>
-      <c r="B42" s="33"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="8"/>
-    </row>
-    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="8"/>
-      <c r="B43" s="33"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="8"/>
-    </row>
-    <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="8"/>
-      <c r="B44" s="33"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="8"/>
-    </row>
-    <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="8"/>
-      <c r="B45" s="34"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="8"/>
-    </row>
-    <row r="46" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B46" s="35"/>
-      <c r="C46" s="36"/>
-      <c r="D46" s="36"/>
-      <c r="E46" s="37"/>
+      <c r="B44" s="36" t="str">
+        <f>INT(SUM(C35:C43)/60)&amp;"h"&amp;MOD(SUM(C35:C43),60)</f>
+        <v>5h35</v>
+      </c>
+      <c r="C44" s="37"/>
+      <c r="D44" s="37"/>
+      <c r="E44" s="38"/>
+    </row>
+    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="13"/>
+      <c r="B45" s="33"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="13"/>
+    </row>
+    <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="8"/>
+      <c r="B46" s="34"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="8"/>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="4"/>
-      <c r="B47" s="38"/>
-      <c r="C47" s="5"/>
-      <c r="D47" s="6"/>
-      <c r="E47" s="5"/>
+      <c r="A47" s="8"/>
+      <c r="B47" s="34"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="8"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="7"/>
-      <c r="B48" s="33"/>
+      <c r="A48" s="8"/>
+      <c r="B48" s="34"/>
       <c r="C48" s="8"/>
       <c r="D48" s="9"/>
       <c r="E48" s="8"/>
     </row>
-    <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="7"/>
-      <c r="B49" s="33"/>
+    <row r="49" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="8"/>
+      <c r="B49" s="35"/>
       <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
-    <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="7"/>
-      <c r="B50" s="33"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="8"/>
-    </row>
-    <row r="51" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="10"/>
-      <c r="B51" s="34"/>
-      <c r="C51" s="10"/>
-      <c r="D51" s="11"/>
-      <c r="E51" s="10"/>
-    </row>
-    <row r="52" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="12" t="s">
+    <row r="50" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B52" s="35"/>
-      <c r="C52" s="36"/>
-      <c r="D52" s="36"/>
-      <c r="E52" s="37"/>
+      <c r="B50" s="36"/>
+      <c r="C50" s="37"/>
+      <c r="D50" s="37"/>
+      <c r="E50" s="38"/>
+    </row>
+    <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="4"/>
+      <c r="B51" s="39"/>
+      <c r="C51" s="5"/>
+      <c r="D51" s="6"/>
+      <c r="E51" s="5"/>
+    </row>
+    <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="7"/>
+      <c r="B52" s="34"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="8"/>
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="4"/>
-      <c r="B53" s="32"/>
-      <c r="C53" s="5"/>
-      <c r="D53" s="6"/>
-      <c r="E53" s="5"/>
+      <c r="A53" s="7"/>
+      <c r="B53" s="34"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="8"/>
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="7"/>
-      <c r="B54" s="33"/>
+      <c r="B54" s="34"/>
       <c r="C54" s="8"/>
       <c r="D54" s="9"/>
       <c r="E54" s="8"/>
     </row>
-    <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="7"/>
-      <c r="B55" s="33"/>
-      <c r="C55" s="8"/>
-      <c r="D55" s="9"/>
-      <c r="E55" s="8"/>
-    </row>
-    <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="7"/>
-      <c r="B56" s="33"/>
-      <c r="C56" s="8"/>
-      <c r="D56" s="9"/>
-      <c r="E56" s="8"/>
-    </row>
-    <row r="57" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="10"/>
-      <c r="B57" s="34"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="11"/>
-      <c r="E57" s="10"/>
-    </row>
-    <row r="58" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="12" t="s">
+    <row r="55" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="10"/>
+      <c r="B55" s="35"/>
+      <c r="C55" s="10"/>
+      <c r="D55" s="11"/>
+      <c r="E55" s="10"/>
+    </row>
+    <row r="56" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B58" s="35"/>
-      <c r="C58" s="36"/>
-      <c r="D58" s="36"/>
-      <c r="E58" s="37"/>
+      <c r="B56" s="36"/>
+      <c r="C56" s="37"/>
+      <c r="D56" s="37"/>
+      <c r="E56" s="38"/>
+    </row>
+    <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="4"/>
+      <c r="B57" s="33"/>
+      <c r="C57" s="5"/>
+      <c r="D57" s="6"/>
+      <c r="E57" s="5"/>
+    </row>
+    <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="7"/>
+      <c r="B58" s="34"/>
+      <c r="C58" s="8"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="4"/>
-      <c r="B59" s="32"/>
-      <c r="C59" s="5"/>
-      <c r="D59" s="6"/>
-      <c r="E59" s="5"/>
+      <c r="A59" s="7"/>
+      <c r="B59" s="34"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="8"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="7"/>
-      <c r="B60" s="33"/>
+      <c r="B60" s="34"/>
       <c r="C60" s="8"/>
       <c r="D60" s="9"/>
       <c r="E60" s="8"/>
     </row>
-    <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="7"/>
-      <c r="B61" s="33"/>
-      <c r="C61" s="8"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="8"/>
-    </row>
-    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="7"/>
-      <c r="B62" s="33"/>
-      <c r="C62" s="8"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="8"/>
-    </row>
-    <row r="63" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="10"/>
-      <c r="B63" s="34"/>
-      <c r="C63" s="10"/>
-      <c r="D63" s="11"/>
-      <c r="E63" s="10"/>
-    </row>
-    <row r="64" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="12" t="s">
+    <row r="61" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="10"/>
+      <c r="B61" s="35"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="11"/>
+      <c r="E61" s="10"/>
+    </row>
+    <row r="62" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B64" s="35"/>
-      <c r="C64" s="36"/>
-      <c r="D64" s="36"/>
-      <c r="E64" s="37"/>
+      <c r="B62" s="36"/>
+      <c r="C62" s="37"/>
+      <c r="D62" s="37"/>
+      <c r="E62" s="38"/>
+    </row>
+    <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="4"/>
+      <c r="B63" s="33"/>
+      <c r="C63" s="5"/>
+      <c r="D63" s="6"/>
+      <c r="E63" s="5"/>
+    </row>
+    <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="7"/>
+      <c r="B64" s="34"/>
+      <c r="C64" s="8"/>
+      <c r="D64" s="9"/>
+      <c r="E64" s="8"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="4"/>
-      <c r="B65" s="32"/>
-      <c r="C65" s="5"/>
-      <c r="D65" s="6"/>
-      <c r="E65" s="5"/>
+      <c r="A65" s="7"/>
+      <c r="B65" s="34"/>
+      <c r="C65" s="8"/>
+      <c r="D65" s="9"/>
+      <c r="E65" s="8"/>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="7"/>
-      <c r="B66" s="33"/>
+      <c r="B66" s="34"/>
       <c r="C66" s="8"/>
       <c r="D66" s="9"/>
       <c r="E66" s="8"/>
     </row>
-    <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="7"/>
-      <c r="B67" s="33"/>
-      <c r="C67" s="8"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="8"/>
-    </row>
-    <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="7"/>
-      <c r="B68" s="33"/>
-      <c r="C68" s="8"/>
-      <c r="D68" s="9"/>
-      <c r="E68" s="8"/>
-    </row>
-    <row r="69" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="10"/>
-      <c r="B69" s="34"/>
-      <c r="C69" s="10"/>
-      <c r="D69" s="11"/>
-      <c r="E69" s="10"/>
-    </row>
-    <row r="70" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="12" t="s">
+    <row r="67" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="10"/>
+      <c r="B67" s="35"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="11"/>
+      <c r="E67" s="10"/>
+    </row>
+    <row r="68" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B70" s="35"/>
-      <c r="C70" s="36"/>
-      <c r="D70" s="36"/>
-      <c r="E70" s="37"/>
+      <c r="B68" s="36"/>
+      <c r="C68" s="37"/>
+      <c r="D68" s="37"/>
+      <c r="E68" s="38"/>
+    </row>
+    <row r="69" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="4"/>
+      <c r="B69" s="33"/>
+      <c r="C69" s="5"/>
+      <c r="D69" s="6"/>
+      <c r="E69" s="5"/>
+    </row>
+    <row r="70" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="7"/>
+      <c r="B70" s="34"/>
+      <c r="C70" s="8"/>
+      <c r="D70" s="9"/>
+      <c r="E70" s="8"/>
     </row>
     <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="13"/>
-      <c r="B71" s="32"/>
-      <c r="C71" s="13"/>
-      <c r="D71" s="14"/>
-      <c r="E71" s="13"/>
+      <c r="A71" s="7"/>
+      <c r="B71" s="34"/>
+      <c r="C71" s="8"/>
+      <c r="D71" s="9"/>
+      <c r="E71" s="8"/>
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="8"/>
-      <c r="B72" s="33"/>
+      <c r="A72" s="7"/>
+      <c r="B72" s="34"/>
       <c r="C72" s="8"/>
       <c r="D72" s="9"/>
       <c r="E72" s="8"/>
     </row>
-    <row r="73" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="8"/>
-      <c r="B73" s="33"/>
-      <c r="C73" s="8"/>
-      <c r="D73" s="9"/>
-      <c r="E73" s="8"/>
-    </row>
-    <row r="74" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="8"/>
-      <c r="B74" s="33"/>
-      <c r="C74" s="8"/>
-      <c r="D74" s="9"/>
-      <c r="E74" s="8"/>
-    </row>
-    <row r="75" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="8"/>
-      <c r="B75" s="34"/>
-      <c r="C75" s="8"/>
-      <c r="D75" s="9"/>
-      <c r="E75" s="8"/>
-    </row>
-    <row r="76" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="12" t="s">
+    <row r="73" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="10"/>
+      <c r="B73" s="35"/>
+      <c r="C73" s="10"/>
+      <c r="D73" s="11"/>
+      <c r="E73" s="10"/>
+    </row>
+    <row r="74" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B76" s="35"/>
-      <c r="C76" s="36"/>
-      <c r="D76" s="36"/>
-      <c r="E76" s="37"/>
-    </row>
-    <row r="77" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="39" t="s">
+      <c r="B74" s="36"/>
+      <c r="C74" s="37"/>
+      <c r="D74" s="37"/>
+      <c r="E74" s="38"/>
+    </row>
+    <row r="75" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="13"/>
+      <c r="B75" s="33"/>
+      <c r="C75" s="13"/>
+      <c r="D75" s="14"/>
+      <c r="E75" s="13"/>
+    </row>
+    <row r="76" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="8"/>
+      <c r="B76" s="34"/>
+      <c r="C76" s="8"/>
+      <c r="D76" s="9"/>
+      <c r="E76" s="8"/>
+    </row>
+    <row r="77" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="8"/>
+      <c r="B77" s="34"/>
+      <c r="C77" s="8"/>
+      <c r="D77" s="9"/>
+      <c r="E77" s="8"/>
+    </row>
+    <row r="78" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="8"/>
+      <c r="B78" s="34"/>
+      <c r="C78" s="8"/>
+      <c r="D78" s="9"/>
+      <c r="E78" s="8"/>
+    </row>
+    <row r="79" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="8"/>
+      <c r="B79" s="35"/>
+      <c r="C79" s="8"/>
+      <c r="D79" s="9"/>
+      <c r="E79" s="8"/>
+    </row>
+    <row r="80" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B80" s="36"/>
+      <c r="C80" s="37"/>
+      <c r="D80" s="37"/>
+      <c r="E80" s="38"/>
+    </row>
+    <row r="81" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="B77" s="40"/>
-      <c r="C77" s="15">
-        <f>MROUND(SUM(C6:C76) /60,0.2)</f>
-        <v>18.8</v>
-      </c>
-      <c r="D77" s="16"/>
-      <c r="E77" s="17"/>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" s="18" t="s">
+      <c r="B81" s="41"/>
+      <c r="C81" s="15">
+        <f>MROUND(SUM(C6:C80) /60,0.2)</f>
+        <v>21.200000000000003</v>
+      </c>
+      <c r="D81" s="16"/>
+      <c r="E81" s="17"/>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A80" s="18"/>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="B76:E76"/>
-    <mergeCell ref="A77:B77"/>
-    <mergeCell ref="B53:B57"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B59:B63"/>
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="B65:B69"/>
-    <mergeCell ref="B70:E70"/>
+    <mergeCell ref="B51:B55"/>
+    <mergeCell ref="B80:E80"/>
+    <mergeCell ref="A81:B81"/>
+    <mergeCell ref="B57:B61"/>
+    <mergeCell ref="B62:E62"/>
+    <mergeCell ref="B63:B67"/>
+    <mergeCell ref="B68:E68"/>
+    <mergeCell ref="B69:B73"/>
+    <mergeCell ref="B74:E74"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B71:B75"/>
-    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="B75:B79"/>
+    <mergeCell ref="B56:E56"/>
     <mergeCell ref="B6:B17"/>
     <mergeCell ref="B18:E18"/>
     <mergeCell ref="B19:B27"/>
     <mergeCell ref="B28:E28"/>
     <mergeCell ref="B29:B33"/>
     <mergeCell ref="B34:E34"/>
-    <mergeCell ref="B35:B39"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B41:B45"/>
-    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B35:B43"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="B45:B49"/>
+    <mergeCell ref="B50:E50"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C65:C69 C59:C63 C47:C51 C53:C57 C29:C33 B6 C6:C17 C35:C39 C41:C45 C71:C75 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C69:C73 C63:C67 C51:C55 C57:C61 C29:C33 B6 C6:C17 C35:C43 C45:C49 C75:C79 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B39 B41:B45 B47:B51 B53:B57 B59:B63 B65:B69 B71:B75" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B43 B45:B49 B51:B55 B57:B61 B63:B67 B69:B73 B75:B79" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(mail): add overwrited links system
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E02C421-B5D5-43A5-BA4B-3231DFCBB73F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A845DC07-43F4-45FD-89C4-09FE73C8CD46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$82</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$85</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="88">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -302,7 +302,21 @@
     <t>J'ai modifié certain point de mon rapport pour qu'ils corspondent à mon CDC</t>
   </si>
   <si>
-    <t>11h25</t>
+    <t>Pixel tracking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je suis entrain de travailler sur le pixel tracking mais je but sur un petit problème qui est que vu que mon environnement est local le mail ne charge pas l'image </t>
+  </si>
+  <si>
+    <t>J'ai terminé le système de tacking par pixel pour tester c'est que j'ai ouvert le lien directement depuis mon navigateur</t>
+  </si>
+  <si>
+    <t>Link tracking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je me suis renseigner sur la réecriture des lien et je me suis servit de l'IA pour qu'elle me donne les regex et aussi pour que les lien affiché soient toujours ce que l'utilisateur veut par exemple :
+si il met ca [Duck Duck Go](https://duckduckgo.com) le html affichera Duck Duck go avec comme lien le lien réecrit
+Si il met juste ca https://duckduckgo.com alors ce sera juste le texte affiché et derrière sera le lien réecrit </t>
   </si>
 </sst>
 </file>
@@ -646,6 +660,48 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="20" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="20" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -657,48 +713,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="20" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1016,7 +1030,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -1032,10 +1046,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="31"/>
+      <c r="C1" s="42"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -1047,10 +1061,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="31"/>
+      <c r="C2" s="42"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -1062,10 +1076,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="31"/>
+      <c r="C3" s="42"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1077,12 +1091,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="34"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="45"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1105,7 +1119,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="41">
+      <c r="B6" s="33">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1118,7 +1132,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="36"/>
+      <c r="B7" s="34"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1131,7 +1145,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="36"/>
+      <c r="B8" s="34"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1144,7 +1158,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="36"/>
+      <c r="B9" s="34"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1155,7 +1169,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="36"/>
+      <c r="B10" s="34"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1168,7 +1182,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="36"/>
+      <c r="B11" s="34"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1183,7 +1197,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="36"/>
+      <c r="B12" s="34"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1198,7 +1212,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="36"/>
+      <c r="B13" s="34"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1213,7 +1227,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="36"/>
+      <c r="B14" s="34"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1228,7 +1242,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="36"/>
+      <c r="B15" s="34"/>
       <c r="C15" s="10">
         <v>40</v>
       </c>
@@ -1243,7 +1257,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="36"/>
+      <c r="B16" s="34"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1256,7 +1270,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="37"/>
+      <c r="B17" s="35"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1265,19 +1279,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="38" t="str">
+      <c r="B18" s="36" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="40"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="38"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="41">
+      <c r="B19" s="33">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1292,7 +1306,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="36"/>
+      <c r="B20" s="34"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1305,7 +1319,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="36"/>
+      <c r="B21" s="34"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1319,7 +1333,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="36"/>
+      <c r="B22" s="34"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1332,7 +1346,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="36"/>
+      <c r="B23" s="34"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1345,7 +1359,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="36"/>
+      <c r="B24" s="34"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1358,7 +1372,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="36"/>
+      <c r="B25" s="34"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1371,7 +1385,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="36"/>
+      <c r="B26" s="34"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1384,7 +1398,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="37"/>
+      <c r="B27" s="35"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1397,19 +1411,19 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="38" t="str">
+      <c r="B28" s="36" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="39"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="40"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="38"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="41">
+      <c r="B29" s="33">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1424,7 +1438,7 @@
       <c r="A30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="36"/>
+      <c r="B30" s="34"/>
       <c r="C30" s="8">
         <v>60</v>
       </c>
@@ -1439,7 +1453,7 @@
       <c r="A31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="36"/>
+      <c r="B31" s="34"/>
       <c r="C31" s="8">
         <v>70</v>
       </c>
@@ -1450,14 +1464,14 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="36"/>
+      <c r="B32" s="34"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="37"/>
+      <c r="B33" s="35"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1466,19 +1480,19 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="38" t="str">
+      <c r="B34" s="36" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C34" s="39"/>
-      <c r="D34" s="39"/>
-      <c r="E34" s="40"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="38"/>
     </row>
     <row r="35" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="41">
+      <c r="B35" s="33">
         <v>46143</v>
       </c>
       <c r="C35" s="5">
@@ -1493,7 +1507,7 @@
       <c r="A36" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="36"/>
+      <c r="B36" s="34"/>
       <c r="C36" s="8">
         <v>35</v>
       </c>
@@ -1506,7 +1520,7 @@
       <c r="A37" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="36"/>
+      <c r="B37" s="34"/>
       <c r="C37" s="8">
         <v>60</v>
       </c>
@@ -1519,7 +1533,7 @@
       <c r="A38" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="36"/>
+      <c r="B38" s="34"/>
       <c r="C38" s="8">
         <v>30</v>
       </c>
@@ -1532,7 +1546,7 @@
       <c r="A39" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="B39" s="36"/>
+      <c r="B39" s="34"/>
       <c r="C39" s="10">
         <v>35</v>
       </c>
@@ -1545,7 +1559,7 @@
       <c r="A40" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B40" s="36"/>
+      <c r="B40" s="34"/>
       <c r="C40" s="10">
         <v>20</v>
       </c>
@@ -1558,7 +1572,7 @@
       <c r="A41" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B41" s="36"/>
+      <c r="B41" s="34"/>
       <c r="C41" s="10">
         <v>50</v>
       </c>
@@ -1571,7 +1585,7 @@
       <c r="A42" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="36"/>
+      <c r="B42" s="34"/>
       <c r="C42" s="10">
         <v>45</v>
       </c>
@@ -1584,7 +1598,7 @@
       <c r="A43" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B43" s="36"/>
+      <c r="B43" s="34"/>
       <c r="C43" s="10">
         <v>60</v>
       </c>
@@ -1597,7 +1611,7 @@
       <c r="A44" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="37"/>
+      <c r="B44" s="35"/>
       <c r="C44" s="10">
         <v>35</v>
       </c>
@@ -1610,19 +1624,19 @@
       <c r="A45" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="38" t="str">
+      <c r="B45" s="36" t="str">
         <f>INT(SUM(C35:C44)/60)&amp;"h"&amp;MOD(SUM(C35:C44),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C45" s="39"/>
-      <c r="D45" s="39"/>
-      <c r="E45" s="40"/>
+      <c r="C45" s="37"/>
+      <c r="D45" s="37"/>
+      <c r="E45" s="38"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B46" s="41">
+      <c r="B46" s="33">
         <v>46146</v>
       </c>
       <c r="C46" s="13">
@@ -1637,319 +1651,347 @@
       <c r="A47" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B47" s="36"/>
+      <c r="B47" s="34"/>
       <c r="C47" s="8">
         <v>45</v>
       </c>
       <c r="D47" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="E47" s="44"/>
+      <c r="E47" s="31"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="36"/>
+      <c r="B48" s="34"/>
       <c r="C48" s="8">
         <v>60</v>
       </c>
       <c r="D48" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E48" s="44"/>
+      <c r="E48" s="31"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B49" s="36"/>
+      <c r="B49" s="34"/>
       <c r="C49" s="8">
         <v>35</v>
       </c>
       <c r="D49" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="E49" s="44" t="s">
+      <c r="E49" s="31"/>
+    </row>
+    <row r="50" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A50" s="8" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="8"/>
-      <c r="B50" s="37"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="45"/>
-      <c r="E50" s="44"/>
-    </row>
-    <row r="51" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="12" t="s">
+      <c r="B50" s="34"/>
+      <c r="C50" s="8">
+        <v>60</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="E50" s="31"/>
+    </row>
+    <row r="51" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A51" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B51" s="34"/>
+      <c r="C51" s="8">
+        <v>20</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="E51" s="31"/>
+    </row>
+    <row r="52" spans="1:5" ht="108" x14ac:dyDescent="0.25">
+      <c r="A52" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B52" s="34"/>
+      <c r="C52" s="8">
+        <v>50</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E52" s="31"/>
+    </row>
+    <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="8"/>
+      <c r="B53" s="35"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="32"/>
+      <c r="E53" s="31"/>
+    </row>
+    <row r="54" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B51" s="38" t="str">
-        <f>INT(SUM(C46:C50)/60)&amp;"h"&amp;MOD(SUM(C46:C50),60)</f>
-        <v>3h10</v>
-      </c>
-      <c r="C51" s="39"/>
-      <c r="D51" s="39"/>
-      <c r="E51" s="40"/>
-    </row>
-    <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="4"/>
-      <c r="B52" s="41"/>
-      <c r="C52" s="5"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="5"/>
-    </row>
-    <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="7"/>
-      <c r="B53" s="36"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="8"/>
-    </row>
-    <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="7"/>
-      <c r="B54" s="36"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="8"/>
+      <c r="B54" s="36" t="str">
+        <f>INT(SUM(C46:C53)/60)&amp;"h"&amp;MOD(SUM(C46:C53),60)</f>
+        <v>5h20</v>
+      </c>
+      <c r="C54" s="37"/>
+      <c r="D54" s="37"/>
+      <c r="E54" s="38"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="7"/>
-      <c r="B55" s="36"/>
-      <c r="C55" s="8"/>
-      <c r="D55" s="9"/>
-      <c r="E55" s="8"/>
-    </row>
-    <row r="56" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="10"/>
-      <c r="B56" s="37"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="10"/>
-    </row>
-    <row r="57" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="12" t="s">
+      <c r="A55" s="4"/>
+      <c r="B55" s="33"/>
+      <c r="C55" s="5"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="5"/>
+    </row>
+    <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="7"/>
+      <c r="B56" s="34"/>
+      <c r="C56" s="8"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="8"/>
+    </row>
+    <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="7"/>
+      <c r="B57" s="34"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="9"/>
+      <c r="E57" s="8"/>
+    </row>
+    <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="7"/>
+      <c r="B58" s="34"/>
+      <c r="C58" s="8"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="8"/>
+    </row>
+    <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="10"/>
+      <c r="B59" s="35"/>
+      <c r="C59" s="10"/>
+      <c r="D59" s="11"/>
+      <c r="E59" s="10"/>
+    </row>
+    <row r="60" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B57" s="38"/>
-      <c r="C57" s="39"/>
-      <c r="D57" s="39"/>
-      <c r="E57" s="40"/>
-    </row>
-    <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="4"/>
-      <c r="B58" s="35"/>
-      <c r="C58" s="5"/>
-      <c r="D58" s="6"/>
-      <c r="E58" s="5"/>
-    </row>
-    <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="7"/>
-      <c r="B59" s="36"/>
-      <c r="C59" s="8"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="8"/>
-    </row>
-    <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="7"/>
       <c r="B60" s="36"/>
-      <c r="C60" s="8"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="8"/>
+      <c r="C60" s="37"/>
+      <c r="D60" s="37"/>
+      <c r="E60" s="38"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="7"/>
-      <c r="B61" s="36"/>
-      <c r="C61" s="8"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="8"/>
-    </row>
-    <row r="62" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="10"/>
-      <c r="B62" s="37"/>
-      <c r="C62" s="10"/>
-      <c r="D62" s="11"/>
-      <c r="E62" s="10"/>
-    </row>
-    <row r="63" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="12" t="s">
+      <c r="A61" s="4"/>
+      <c r="B61" s="41"/>
+      <c r="C61" s="5"/>
+      <c r="D61" s="6"/>
+      <c r="E61" s="5"/>
+    </row>
+    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="7"/>
+      <c r="B62" s="34"/>
+      <c r="C62" s="8"/>
+      <c r="D62" s="9"/>
+      <c r="E62" s="8"/>
+    </row>
+    <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="7"/>
+      <c r="B63" s="34"/>
+      <c r="C63" s="8"/>
+      <c r="D63" s="9"/>
+      <c r="E63" s="8"/>
+    </row>
+    <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="7"/>
+      <c r="B64" s="34"/>
+      <c r="C64" s="8"/>
+      <c r="D64" s="9"/>
+      <c r="E64" s="8"/>
+    </row>
+    <row r="65" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="10"/>
+      <c r="B65" s="35"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="11"/>
+      <c r="E65" s="10"/>
+    </row>
+    <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B63" s="38"/>
-      <c r="C63" s="39"/>
-      <c r="D63" s="39"/>
-      <c r="E63" s="40"/>
-    </row>
-    <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="4"/>
-      <c r="B64" s="35"/>
-      <c r="C64" s="5"/>
-      <c r="D64" s="6"/>
-      <c r="E64" s="5"/>
-    </row>
-    <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="7"/>
-      <c r="B65" s="36"/>
-      <c r="C65" s="8"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="8"/>
-    </row>
-    <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="7"/>
       <c r="B66" s="36"/>
-      <c r="C66" s="8"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="8"/>
+      <c r="C66" s="37"/>
+      <c r="D66" s="37"/>
+      <c r="E66" s="38"/>
     </row>
     <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="7"/>
-      <c r="B67" s="36"/>
-      <c r="C67" s="8"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="8"/>
-    </row>
-    <row r="68" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="10"/>
-      <c r="B68" s="37"/>
-      <c r="C68" s="10"/>
-      <c r="D68" s="11"/>
-      <c r="E68" s="10"/>
-    </row>
-    <row r="69" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="12" t="s">
+      <c r="A67" s="4"/>
+      <c r="B67" s="41"/>
+      <c r="C67" s="5"/>
+      <c r="D67" s="6"/>
+      <c r="E67" s="5"/>
+    </row>
+    <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="7"/>
+      <c r="B68" s="34"/>
+      <c r="C68" s="8"/>
+      <c r="D68" s="9"/>
+      <c r="E68" s="8"/>
+    </row>
+    <row r="69" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="7"/>
+      <c r="B69" s="34"/>
+      <c r="C69" s="8"/>
+      <c r="D69" s="9"/>
+      <c r="E69" s="8"/>
+    </row>
+    <row r="70" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="7"/>
+      <c r="B70" s="34"/>
+      <c r="C70" s="8"/>
+      <c r="D70" s="9"/>
+      <c r="E70" s="8"/>
+    </row>
+    <row r="71" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="10"/>
+      <c r="B71" s="35"/>
+      <c r="C71" s="10"/>
+      <c r="D71" s="11"/>
+      <c r="E71" s="10"/>
+    </row>
+    <row r="72" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B69" s="38"/>
-      <c r="C69" s="39"/>
-      <c r="D69" s="39"/>
-      <c r="E69" s="40"/>
-    </row>
-    <row r="70" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="4"/>
-      <c r="B70" s="35"/>
-      <c r="C70" s="5"/>
-      <c r="D70" s="6"/>
-      <c r="E70" s="5"/>
-    </row>
-    <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="7"/>
-      <c r="B71" s="36"/>
-      <c r="C71" s="8"/>
-      <c r="D71" s="9"/>
-      <c r="E71" s="8"/>
-    </row>
-    <row r="72" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="7"/>
       <c r="B72" s="36"/>
-      <c r="C72" s="8"/>
-      <c r="D72" s="9"/>
-      <c r="E72" s="8"/>
+      <c r="C72" s="37"/>
+      <c r="D72" s="37"/>
+      <c r="E72" s="38"/>
     </row>
     <row r="73" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="7"/>
-      <c r="B73" s="36"/>
-      <c r="C73" s="8"/>
-      <c r="D73" s="9"/>
-      <c r="E73" s="8"/>
-    </row>
-    <row r="74" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="10"/>
-      <c r="B74" s="37"/>
-      <c r="C74" s="10"/>
-      <c r="D74" s="11"/>
-      <c r="E74" s="10"/>
-    </row>
-    <row r="75" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="12" t="s">
+      <c r="A73" s="4"/>
+      <c r="B73" s="41"/>
+      <c r="C73" s="5"/>
+      <c r="D73" s="6"/>
+      <c r="E73" s="5"/>
+    </row>
+    <row r="74" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="7"/>
+      <c r="B74" s="34"/>
+      <c r="C74" s="8"/>
+      <c r="D74" s="9"/>
+      <c r="E74" s="8"/>
+    </row>
+    <row r="75" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="7"/>
+      <c r="B75" s="34"/>
+      <c r="C75" s="8"/>
+      <c r="D75" s="9"/>
+      <c r="E75" s="8"/>
+    </row>
+    <row r="76" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="7"/>
+      <c r="B76" s="34"/>
+      <c r="C76" s="8"/>
+      <c r="D76" s="9"/>
+      <c r="E76" s="8"/>
+    </row>
+    <row r="77" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="10"/>
+      <c r="B77" s="35"/>
+      <c r="C77" s="10"/>
+      <c r="D77" s="11"/>
+      <c r="E77" s="10"/>
+    </row>
+    <row r="78" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B75" s="38"/>
-      <c r="C75" s="39"/>
-      <c r="D75" s="39"/>
-      <c r="E75" s="40"/>
-    </row>
-    <row r="76" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="13"/>
-      <c r="B76" s="35"/>
-      <c r="C76" s="13"/>
-      <c r="D76" s="14"/>
-      <c r="E76" s="13"/>
-    </row>
-    <row r="77" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="8"/>
-      <c r="B77" s="36"/>
-      <c r="C77" s="8"/>
-      <c r="D77" s="9"/>
-      <c r="E77" s="8"/>
-    </row>
-    <row r="78" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="8"/>
       <c r="B78" s="36"/>
-      <c r="C78" s="8"/>
-      <c r="D78" s="9"/>
-      <c r="E78" s="8"/>
+      <c r="C78" s="37"/>
+      <c r="D78" s="37"/>
+      <c r="E78" s="38"/>
     </row>
     <row r="79" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="8"/>
-      <c r="B79" s="36"/>
-      <c r="C79" s="8"/>
-      <c r="D79" s="9"/>
-      <c r="E79" s="8"/>
-    </row>
-    <row r="80" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="13"/>
+      <c r="B79" s="41"/>
+      <c r="C79" s="13"/>
+      <c r="D79" s="14"/>
+      <c r="E79" s="13"/>
+    </row>
+    <row r="80" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="8"/>
-      <c r="B80" s="37"/>
+      <c r="B80" s="34"/>
       <c r="C80" s="8"/>
       <c r="D80" s="9"/>
       <c r="E80" s="8"/>
     </row>
-    <row r="81" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="12" t="s">
+    <row r="81" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="8"/>
+      <c r="B81" s="34"/>
+      <c r="C81" s="8"/>
+      <c r="D81" s="9"/>
+      <c r="E81" s="8"/>
+    </row>
+    <row r="82" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="8"/>
+      <c r="B82" s="34"/>
+      <c r="C82" s="8"/>
+      <c r="D82" s="9"/>
+      <c r="E82" s="8"/>
+    </row>
+    <row r="83" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="8"/>
+      <c r="B83" s="35"/>
+      <c r="C83" s="8"/>
+      <c r="D83" s="9"/>
+      <c r="E83" s="8"/>
+    </row>
+    <row r="84" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B81" s="38"/>
-      <c r="C81" s="39"/>
-      <c r="D81" s="39"/>
-      <c r="E81" s="40"/>
-    </row>
-    <row r="82" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="42" t="s">
+      <c r="B84" s="36"/>
+      <c r="C84" s="37"/>
+      <c r="D84" s="37"/>
+      <c r="E84" s="38"/>
+    </row>
+    <row r="85" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B82" s="43"/>
-      <c r="C82" s="15">
-        <f>MROUND(SUM(C6:C81) /60,0.2)</f>
-        <v>26</v>
-      </c>
-      <c r="D82" s="16"/>
-      <c r="E82" s="17"/>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="18" t="s">
+      <c r="B85" s="40"/>
+      <c r="C85" s="15">
+        <f>MROUND(SUM(C6:C84) /60,0.2)</f>
+        <v>28.200000000000003</v>
+      </c>
+      <c r="D85" s="16"/>
+      <c r="E85" s="17"/>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" s="18"/>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B81:E81"/>
-    <mergeCell ref="A82:B82"/>
-    <mergeCell ref="B58:B62"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="B64:B68"/>
-    <mergeCell ref="B69:E69"/>
-    <mergeCell ref="B70:B74"/>
-    <mergeCell ref="B75:E75"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B76:B80"/>
-    <mergeCell ref="B57:E57"/>
+    <mergeCell ref="B79:B83"/>
+    <mergeCell ref="B60:E60"/>
     <mergeCell ref="B6:B17"/>
     <mergeCell ref="B18:E18"/>
     <mergeCell ref="B19:B27"/>
@@ -1958,14 +2000,23 @@
     <mergeCell ref="B34:E34"/>
     <mergeCell ref="B35:B44"/>
     <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B46:B50"/>
-    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="B46:B53"/>
+    <mergeCell ref="B54:E54"/>
+    <mergeCell ref="B55:B59"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="A85:B85"/>
+    <mergeCell ref="B61:B65"/>
+    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="B67:B71"/>
+    <mergeCell ref="B72:E72"/>
+    <mergeCell ref="B73:B77"/>
+    <mergeCell ref="B78:E78"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C70:C74 C64:C68 C52:C56 C58:C62 C29:C33 B6 C6:C17 C35:C44 C46:C50 C76:C80 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C73:C77 C67:C71 C55:C59 C61:C65 C29:C33 B6 C6:C17 C35:C44 C46:C53 C79:C83 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B50 B52:B56 B58:B62 B64:B68 B70:B74 B76:B80" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B59 B61:B65 B67:B71 B73:B77 B79:B83" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -1974,7 +2025,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="46" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="41" orientation="portrait" r:id="rId2"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -2164,12 +2215,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -2331,6 +2376,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
@@ -2340,15 +2391,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2364,4 +2406,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(NL): add create system
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A845DC07-43F4-45FD-89C4-09FE73C8CD46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E6BD12B-40AA-43A7-8AD2-C09207FE6220}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="93">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -317,6 +317,21 @@
     <t xml:space="preserve">Je me suis renseigner sur la réecriture des lien et je me suis servit de l'IA pour qu'elle me donne les regex et aussi pour que les lien affiché soient toujours ce que l'utilisateur veut par exemple :
 si il met ca [Duck Duck Go](https://duckduckgo.com) le html affichera Duck Duck go avec comme lien le lien réecrit
 Si il met juste ca https://duckduckgo.com alors ce sera juste le texte affiché et derrière sera le lien réecrit </t>
+  </si>
+  <si>
+    <t>création</t>
+  </si>
+  <si>
+    <t>J'ai commencé la page de création d'un campagne</t>
+  </si>
+  <si>
+    <t>creation</t>
+  </si>
+  <si>
+    <t>J'ai continué mon editeur simple et j'ai presque terminé</t>
+  </si>
+  <si>
+    <t>J'ai terminé la page de création mais j'ai un problème avec mon API</t>
   </si>
 </sst>
 </file>
@@ -668,51 +683,51 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1046,10 +1061,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="42"/>
+      <c r="C1" s="33"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -1061,10 +1076,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="42"/>
+      <c r="C2" s="33"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -1076,10 +1091,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="42"/>
+      <c r="C3" s="33"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1091,12 +1106,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="43" t="s">
+      <c r="B4" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="45"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="36"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1119,7 +1134,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="33">
+      <c r="B6" s="43">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1132,7 +1147,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="34"/>
+      <c r="B7" s="38"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1145,7 +1160,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="34"/>
+      <c r="B8" s="38"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1158,7 +1173,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="34"/>
+      <c r="B9" s="38"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1169,7 +1184,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="34"/>
+      <c r="B10" s="38"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1182,7 +1197,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="34"/>
+      <c r="B11" s="38"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1197,7 +1212,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="34"/>
+      <c r="B12" s="38"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1212,7 +1227,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="34"/>
+      <c r="B13" s="38"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1227,7 +1242,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="34"/>
+      <c r="B14" s="38"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1242,7 +1257,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="34"/>
+      <c r="B15" s="38"/>
       <c r="C15" s="10">
         <v>40</v>
       </c>
@@ -1257,7 +1272,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="34"/>
+      <c r="B16" s="38"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1270,7 +1285,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="35"/>
+      <c r="B17" s="39"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1279,19 +1294,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="36" t="str">
+      <c r="B18" s="40" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="38"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="42"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="33">
+      <c r="B19" s="43">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1306,7 +1321,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="34"/>
+      <c r="B20" s="38"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1319,7 +1334,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="34"/>
+      <c r="B21" s="38"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1333,7 +1348,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="34"/>
+      <c r="B22" s="38"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1346,7 +1361,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="34"/>
+      <c r="B23" s="38"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1359,7 +1374,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="34"/>
+      <c r="B24" s="38"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1372,7 +1387,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="34"/>
+      <c r="B25" s="38"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1385,7 +1400,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="34"/>
+      <c r="B26" s="38"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1398,7 +1413,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="35"/>
+      <c r="B27" s="39"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1411,19 +1426,19 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="36" t="str">
+      <c r="B28" s="40" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="37"/>
-      <c r="D28" s="37"/>
-      <c r="E28" s="38"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="42"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="33">
+      <c r="B29" s="43">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1438,7 +1453,7 @@
       <c r="A30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="34"/>
+      <c r="B30" s="38"/>
       <c r="C30" s="8">
         <v>60</v>
       </c>
@@ -1453,7 +1468,7 @@
       <c r="A31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="34"/>
+      <c r="B31" s="38"/>
       <c r="C31" s="8">
         <v>70</v>
       </c>
@@ -1464,14 +1479,14 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="34"/>
+      <c r="B32" s="38"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="35"/>
+      <c r="B33" s="39"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1480,19 +1495,19 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="36" t="str">
+      <c r="B34" s="40" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C34" s="37"/>
-      <c r="D34" s="37"/>
-      <c r="E34" s="38"/>
+      <c r="C34" s="41"/>
+      <c r="D34" s="41"/>
+      <c r="E34" s="42"/>
     </row>
     <row r="35" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="33">
+      <c r="B35" s="43">
         <v>46143</v>
       </c>
       <c r="C35" s="5">
@@ -1507,7 +1522,7 @@
       <c r="A36" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="34"/>
+      <c r="B36" s="38"/>
       <c r="C36" s="8">
         <v>35</v>
       </c>
@@ -1520,7 +1535,7 @@
       <c r="A37" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="34"/>
+      <c r="B37" s="38"/>
       <c r="C37" s="8">
         <v>60</v>
       </c>
@@ -1533,7 +1548,7 @@
       <c r="A38" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="34"/>
+      <c r="B38" s="38"/>
       <c r="C38" s="8">
         <v>30</v>
       </c>
@@ -1546,7 +1561,7 @@
       <c r="A39" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="B39" s="34"/>
+      <c r="B39" s="38"/>
       <c r="C39" s="10">
         <v>35</v>
       </c>
@@ -1559,7 +1574,7 @@
       <c r="A40" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B40" s="34"/>
+      <c r="B40" s="38"/>
       <c r="C40" s="10">
         <v>20</v>
       </c>
@@ -1572,7 +1587,7 @@
       <c r="A41" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B41" s="34"/>
+      <c r="B41" s="38"/>
       <c r="C41" s="10">
         <v>50</v>
       </c>
@@ -1585,7 +1600,7 @@
       <c r="A42" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="34"/>
+      <c r="B42" s="38"/>
       <c r="C42" s="10">
         <v>45</v>
       </c>
@@ -1598,7 +1613,7 @@
       <c r="A43" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B43" s="34"/>
+      <c r="B43" s="38"/>
       <c r="C43" s="10">
         <v>60</v>
       </c>
@@ -1611,7 +1626,7 @@
       <c r="A44" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="35"/>
+      <c r="B44" s="39"/>
       <c r="C44" s="10">
         <v>35</v>
       </c>
@@ -1624,19 +1639,19 @@
       <c r="A45" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="36" t="str">
+      <c r="B45" s="40" t="str">
         <f>INT(SUM(C35:C44)/60)&amp;"h"&amp;MOD(SUM(C35:C44),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C45" s="37"/>
-      <c r="D45" s="37"/>
-      <c r="E45" s="38"/>
+      <c r="C45" s="41"/>
+      <c r="D45" s="41"/>
+      <c r="E45" s="42"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B46" s="33">
+      <c r="B46" s="43">
         <v>46146</v>
       </c>
       <c r="C46" s="13">
@@ -1651,7 +1666,7 @@
       <c r="A47" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B47" s="34"/>
+      <c r="B47" s="38"/>
       <c r="C47" s="8">
         <v>45</v>
       </c>
@@ -1664,7 +1679,7 @@
       <c r="A48" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="34"/>
+      <c r="B48" s="38"/>
       <c r="C48" s="8">
         <v>60</v>
       </c>
@@ -1677,7 +1692,7 @@
       <c r="A49" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B49" s="34"/>
+      <c r="B49" s="38"/>
       <c r="C49" s="8">
         <v>35</v>
       </c>
@@ -1690,7 +1705,7 @@
       <c r="A50" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B50" s="34"/>
+      <c r="B50" s="38"/>
       <c r="C50" s="8">
         <v>60</v>
       </c>
@@ -1703,7 +1718,7 @@
       <c r="A51" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B51" s="34"/>
+      <c r="B51" s="38"/>
       <c r="C51" s="8">
         <v>20</v>
       </c>
@@ -1716,7 +1731,7 @@
       <c r="A52" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B52" s="34"/>
+      <c r="B52" s="38"/>
       <c r="C52" s="8">
         <v>50</v>
       </c>
@@ -1727,7 +1742,7 @@
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="8"/>
-      <c r="B53" s="35"/>
+      <c r="B53" s="39"/>
       <c r="C53" s="8"/>
       <c r="D53" s="32"/>
       <c r="E53" s="31"/>
@@ -1736,45 +1751,65 @@
       <c r="A54" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B54" s="36" t="str">
+      <c r="B54" s="40" t="str">
         <f>INT(SUM(C46:C53)/60)&amp;"h"&amp;MOD(SUM(C46:C53),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C54" s="37"/>
-      <c r="D54" s="37"/>
-      <c r="E54" s="38"/>
+      <c r="C54" s="41"/>
+      <c r="D54" s="41"/>
+      <c r="E54" s="42"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="4"/>
-      <c r="B55" s="33"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="6"/>
+      <c r="A55" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B55" s="43">
+        <v>46148</v>
+      </c>
+      <c r="C55" s="5">
+        <v>60</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>89</v>
+      </c>
       <c r="E55" s="5"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="7"/>
-      <c r="B56" s="34"/>
-      <c r="C56" s="8"/>
-      <c r="D56" s="9"/>
+      <c r="A56" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B56" s="38"/>
+      <c r="C56" s="8">
+        <v>35</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>91</v>
+      </c>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="7"/>
-      <c r="B57" s="34"/>
-      <c r="C57" s="8"/>
-      <c r="D57" s="9"/>
+      <c r="A57" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B57" s="38"/>
+      <c r="C57" s="8">
+        <v>60</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>92</v>
+      </c>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="34"/>
+      <c r="B58" s="38"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="10"/>
-      <c r="B59" s="35"/>
+      <c r="B59" s="39"/>
       <c r="C59" s="10"/>
       <c r="D59" s="11"/>
       <c r="E59" s="10"/>
@@ -1783,42 +1818,42 @@
       <c r="A60" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B60" s="36"/>
-      <c r="C60" s="37"/>
-      <c r="D60" s="37"/>
-      <c r="E60" s="38"/>
+      <c r="B60" s="40"/>
+      <c r="C60" s="41"/>
+      <c r="D60" s="41"/>
+      <c r="E60" s="42"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="4"/>
-      <c r="B61" s="41"/>
+      <c r="B61" s="37"/>
       <c r="C61" s="5"/>
       <c r="D61" s="6"/>
       <c r="E61" s="5"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="7"/>
-      <c r="B62" s="34"/>
+      <c r="B62" s="38"/>
       <c r="C62" s="8"/>
       <c r="D62" s="9"/>
       <c r="E62" s="8"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="34"/>
+      <c r="B63" s="38"/>
       <c r="C63" s="8"/>
       <c r="D63" s="9"/>
       <c r="E63" s="8"/>
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="34"/>
+      <c r="B64" s="38"/>
       <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="10"/>
-      <c r="B65" s="35"/>
+      <c r="B65" s="39"/>
       <c r="C65" s="10"/>
       <c r="D65" s="11"/>
       <c r="E65" s="10"/>
@@ -1827,42 +1862,42 @@
       <c r="A66" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B66" s="36"/>
-      <c r="C66" s="37"/>
-      <c r="D66" s="37"/>
-      <c r="E66" s="38"/>
+      <c r="B66" s="40"/>
+      <c r="C66" s="41"/>
+      <c r="D66" s="41"/>
+      <c r="E66" s="42"/>
     </row>
     <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="4"/>
-      <c r="B67" s="41"/>
+      <c r="B67" s="37"/>
       <c r="C67" s="5"/>
       <c r="D67" s="6"/>
       <c r="E67" s="5"/>
     </row>
     <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7"/>
-      <c r="B68" s="34"/>
+      <c r="B68" s="38"/>
       <c r="C68" s="8"/>
       <c r="D68" s="9"/>
       <c r="E68" s="8"/>
     </row>
     <row r="69" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="7"/>
-      <c r="B69" s="34"/>
+      <c r="B69" s="38"/>
       <c r="C69" s="8"/>
       <c r="D69" s="9"/>
       <c r="E69" s="8"/>
     </row>
     <row r="70" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="7"/>
-      <c r="B70" s="34"/>
+      <c r="B70" s="38"/>
       <c r="C70" s="8"/>
       <c r="D70" s="9"/>
       <c r="E70" s="8"/>
     </row>
     <row r="71" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="10"/>
-      <c r="B71" s="35"/>
+      <c r="B71" s="39"/>
       <c r="C71" s="10"/>
       <c r="D71" s="11"/>
       <c r="E71" s="10"/>
@@ -1871,42 +1906,42 @@
       <c r="A72" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B72" s="36"/>
-      <c r="C72" s="37"/>
-      <c r="D72" s="37"/>
-      <c r="E72" s="38"/>
+      <c r="B72" s="40"/>
+      <c r="C72" s="41"/>
+      <c r="D72" s="41"/>
+      <c r="E72" s="42"/>
     </row>
     <row r="73" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="4"/>
-      <c r="B73" s="41"/>
+      <c r="B73" s="37"/>
       <c r="C73" s="5"/>
       <c r="D73" s="6"/>
       <c r="E73" s="5"/>
     </row>
     <row r="74" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="7"/>
-      <c r="B74" s="34"/>
+      <c r="B74" s="38"/>
       <c r="C74" s="8"/>
       <c r="D74" s="9"/>
       <c r="E74" s="8"/>
     </row>
     <row r="75" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="7"/>
-      <c r="B75" s="34"/>
+      <c r="B75" s="38"/>
       <c r="C75" s="8"/>
       <c r="D75" s="9"/>
       <c r="E75" s="8"/>
     </row>
     <row r="76" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="7"/>
-      <c r="B76" s="34"/>
+      <c r="B76" s="38"/>
       <c r="C76" s="8"/>
       <c r="D76" s="9"/>
       <c r="E76" s="8"/>
     </row>
     <row r="77" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="10"/>
-      <c r="B77" s="35"/>
+      <c r="B77" s="39"/>
       <c r="C77" s="10"/>
       <c r="D77" s="11"/>
       <c r="E77" s="10"/>
@@ -1915,42 +1950,42 @@
       <c r="A78" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B78" s="36"/>
-      <c r="C78" s="37"/>
-      <c r="D78" s="37"/>
-      <c r="E78" s="38"/>
+      <c r="B78" s="40"/>
+      <c r="C78" s="41"/>
+      <c r="D78" s="41"/>
+      <c r="E78" s="42"/>
     </row>
     <row r="79" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="13"/>
-      <c r="B79" s="41"/>
+      <c r="B79" s="37"/>
       <c r="C79" s="13"/>
       <c r="D79" s="14"/>
       <c r="E79" s="13"/>
     </row>
     <row r="80" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="8"/>
-      <c r="B80" s="34"/>
+      <c r="B80" s="38"/>
       <c r="C80" s="8"/>
       <c r="D80" s="9"/>
       <c r="E80" s="8"/>
     </row>
     <row r="81" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="8"/>
-      <c r="B81" s="34"/>
+      <c r="B81" s="38"/>
       <c r="C81" s="8"/>
       <c r="D81" s="9"/>
       <c r="E81" s="8"/>
     </row>
     <row r="82" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="8"/>
-      <c r="B82" s="34"/>
+      <c r="B82" s="38"/>
       <c r="C82" s="8"/>
       <c r="D82" s="9"/>
       <c r="E82" s="8"/>
     </row>
     <row r="83" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="8"/>
-      <c r="B83" s="35"/>
+      <c r="B83" s="39"/>
       <c r="C83" s="8"/>
       <c r="D83" s="9"/>
       <c r="E83" s="8"/>
@@ -1959,19 +1994,19 @@
       <c r="A84" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="36"/>
-      <c r="C84" s="37"/>
-      <c r="D84" s="37"/>
-      <c r="E84" s="38"/>
+      <c r="B84" s="40"/>
+      <c r="C84" s="41"/>
+      <c r="D84" s="41"/>
+      <c r="E84" s="42"/>
     </row>
     <row r="85" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="39" t="s">
+      <c r="A85" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="B85" s="40"/>
+      <c r="B85" s="45"/>
       <c r="C85" s="15">
         <f>MROUND(SUM(C6:C84) /60,0.2)</f>
-        <v>28.200000000000003</v>
+        <v>30.8</v>
       </c>
       <c r="D85" s="16"/>
       <c r="E85" s="17"/>
@@ -1986,6 +2021,15 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B55:B59"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="A85:B85"/>
+    <mergeCell ref="B61:B65"/>
+    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="B67:B71"/>
+    <mergeCell ref="B72:E72"/>
+    <mergeCell ref="B73:B77"/>
+    <mergeCell ref="B78:E78"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -2002,15 +2046,6 @@
     <mergeCell ref="B45:E45"/>
     <mergeCell ref="B46:B53"/>
     <mergeCell ref="B54:E54"/>
-    <mergeCell ref="B55:B59"/>
-    <mergeCell ref="B84:E84"/>
-    <mergeCell ref="A85:B85"/>
-    <mergeCell ref="B61:B65"/>
-    <mergeCell ref="B66:E66"/>
-    <mergeCell ref="B67:B71"/>
-    <mergeCell ref="B72:E72"/>
-    <mergeCell ref="B73:B77"/>
-    <mergeCell ref="B78:E78"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C73:C77 C67:C71 C55:C59 C61:C65 C29:C33 B6 C6:C17 C35:C44 C46:C53 C79:C83 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -2215,6 +2250,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -2376,12 +2417,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
@@ -2391,6 +2426,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2406,13 +2450,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(NL): add NL details page
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E6BD12B-40AA-43A7-8AD2-C09207FE6220}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A90A8ADD-BA17-4B8F-B320-4F6ECBE8B549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,9 +17,10 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$85</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$89</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="102">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -332,6 +333,33 @@
   </si>
   <si>
     <t>J'ai terminé la page de création mais j'ai un problème avec mon API</t>
+  </si>
+  <si>
+    <t>Modification</t>
+  </si>
+  <si>
+    <t>J'ai ajouté le sstème de modification d'une campagne</t>
+  </si>
+  <si>
+    <t>Page des détails</t>
+  </si>
+  <si>
+    <t>J'ai commencé la page de détails d'une campagne</t>
+  </si>
+  <si>
+    <t>J'ai contuné la page des détails</t>
+  </si>
+  <si>
+    <t>Discussion avec Expert 2</t>
+  </si>
+  <si>
+    <t>J'ai eu la visite du deuxième expert afin de faire le point</t>
+  </si>
+  <si>
+    <t>J'ai terminé la page des détails</t>
+  </si>
+  <si>
+    <t>14h00</t>
   </si>
 </sst>
 </file>
@@ -683,51 +711,51 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1045,7 +1073,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -1061,10 +1089,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="33"/>
+      <c r="C1" s="42"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -1076,10 +1104,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="33"/>
+      <c r="C2" s="42"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -1091,10 +1119,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="33"/>
+      <c r="C3" s="42"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1106,12 +1134,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="36"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="45"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1134,7 +1162,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="43">
+      <c r="B6" s="33">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1147,7 +1175,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="38"/>
+      <c r="B7" s="34"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1160,7 +1188,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="38"/>
+      <c r="B8" s="34"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1173,7 +1201,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="38"/>
+      <c r="B9" s="34"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1184,7 +1212,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="38"/>
+      <c r="B10" s="34"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1197,7 +1225,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="38"/>
+      <c r="B11" s="34"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1212,7 +1240,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="34"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1227,7 +1255,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="38"/>
+      <c r="B13" s="34"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1242,7 +1270,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="38"/>
+      <c r="B14" s="34"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1257,7 +1285,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="38"/>
+      <c r="B15" s="34"/>
       <c r="C15" s="10">
         <v>40</v>
       </c>
@@ -1272,7 +1300,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="34"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1285,7 +1313,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="39"/>
+      <c r="B17" s="35"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1294,19 +1322,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="40" t="str">
+      <c r="B18" s="36" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C18" s="41"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="42"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="38"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="43">
+      <c r="B19" s="33">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1321,7 +1349,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="38"/>
+      <c r="B20" s="34"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1334,7 +1362,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="38"/>
+      <c r="B21" s="34"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1348,7 +1376,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="38"/>
+      <c r="B22" s="34"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1361,7 +1389,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="38"/>
+      <c r="B23" s="34"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1374,7 +1402,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="38"/>
+      <c r="B24" s="34"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1387,7 +1415,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="38"/>
+      <c r="B25" s="34"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1400,7 +1428,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="38"/>
+      <c r="B26" s="34"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1413,7 +1441,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="39"/>
+      <c r="B27" s="35"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1426,19 +1454,19 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="40" t="str">
+      <c r="B28" s="36" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="41"/>
-      <c r="D28" s="41"/>
-      <c r="E28" s="42"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="38"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="43">
+      <c r="B29" s="33">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1453,7 +1481,7 @@
       <c r="A30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="38"/>
+      <c r="B30" s="34"/>
       <c r="C30" s="8">
         <v>60</v>
       </c>
@@ -1468,7 +1496,7 @@
       <c r="A31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="38"/>
+      <c r="B31" s="34"/>
       <c r="C31" s="8">
         <v>70</v>
       </c>
@@ -1479,14 +1507,14 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="38"/>
+      <c r="B32" s="34"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="39"/>
+      <c r="B33" s="35"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1495,19 +1523,19 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="40" t="str">
+      <c r="B34" s="36" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C34" s="41"/>
-      <c r="D34" s="41"/>
-      <c r="E34" s="42"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="38"/>
     </row>
     <row r="35" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="43">
+      <c r="B35" s="33">
         <v>46143</v>
       </c>
       <c r="C35" s="5">
@@ -1522,7 +1550,7 @@
       <c r="A36" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="38"/>
+      <c r="B36" s="34"/>
       <c r="C36" s="8">
         <v>35</v>
       </c>
@@ -1535,7 +1563,7 @@
       <c r="A37" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="38"/>
+      <c r="B37" s="34"/>
       <c r="C37" s="8">
         <v>60</v>
       </c>
@@ -1548,7 +1576,7 @@
       <c r="A38" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="38"/>
+      <c r="B38" s="34"/>
       <c r="C38" s="8">
         <v>30</v>
       </c>
@@ -1561,7 +1589,7 @@
       <c r="A39" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="B39" s="38"/>
+      <c r="B39" s="34"/>
       <c r="C39" s="10">
         <v>35</v>
       </c>
@@ -1574,7 +1602,7 @@
       <c r="A40" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B40" s="38"/>
+      <c r="B40" s="34"/>
       <c r="C40" s="10">
         <v>20</v>
       </c>
@@ -1587,7 +1615,7 @@
       <c r="A41" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B41" s="38"/>
+      <c r="B41" s="34"/>
       <c r="C41" s="10">
         <v>50</v>
       </c>
@@ -1600,7 +1628,7 @@
       <c r="A42" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="38"/>
+      <c r="B42" s="34"/>
       <c r="C42" s="10">
         <v>45</v>
       </c>
@@ -1613,7 +1641,7 @@
       <c r="A43" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B43" s="38"/>
+      <c r="B43" s="34"/>
       <c r="C43" s="10">
         <v>60</v>
       </c>
@@ -1626,7 +1654,7 @@
       <c r="A44" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="39"/>
+      <c r="B44" s="35"/>
       <c r="C44" s="10">
         <v>35</v>
       </c>
@@ -1639,19 +1667,19 @@
       <c r="A45" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="40" t="str">
+      <c r="B45" s="36" t="str">
         <f>INT(SUM(C35:C44)/60)&amp;"h"&amp;MOD(SUM(C35:C44),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C45" s="41"/>
-      <c r="D45" s="41"/>
-      <c r="E45" s="42"/>
+      <c r="C45" s="37"/>
+      <c r="D45" s="37"/>
+      <c r="E45" s="38"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B46" s="43">
+      <c r="B46" s="33">
         <v>46146</v>
       </c>
       <c r="C46" s="13">
@@ -1666,7 +1694,7 @@
       <c r="A47" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B47" s="38"/>
+      <c r="B47" s="34"/>
       <c r="C47" s="8">
         <v>45</v>
       </c>
@@ -1679,7 +1707,7 @@
       <c r="A48" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="38"/>
+      <c r="B48" s="34"/>
       <c r="C48" s="8">
         <v>60</v>
       </c>
@@ -1692,7 +1720,7 @@
       <c r="A49" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B49" s="38"/>
+      <c r="B49" s="34"/>
       <c r="C49" s="8">
         <v>35</v>
       </c>
@@ -1705,7 +1733,7 @@
       <c r="A50" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B50" s="38"/>
+      <c r="B50" s="34"/>
       <c r="C50" s="8">
         <v>60</v>
       </c>
@@ -1718,7 +1746,7 @@
       <c r="A51" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B51" s="38"/>
+      <c r="B51" s="34"/>
       <c r="C51" s="8">
         <v>20</v>
       </c>
@@ -1731,7 +1759,7 @@
       <c r="A52" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B52" s="38"/>
+      <c r="B52" s="34"/>
       <c r="C52" s="8">
         <v>50</v>
       </c>
@@ -1742,7 +1770,7 @@
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="8"/>
-      <c r="B53" s="39"/>
+      <c r="B53" s="35"/>
       <c r="C53" s="8"/>
       <c r="D53" s="32"/>
       <c r="E53" s="31"/>
@@ -1751,19 +1779,19 @@
       <c r="A54" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B54" s="40" t="str">
+      <c r="B54" s="36" t="str">
         <f>INT(SUM(C46:C53)/60)&amp;"h"&amp;MOD(SUM(C46:C53),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C54" s="41"/>
-      <c r="D54" s="41"/>
-      <c r="E54" s="42"/>
+      <c r="C54" s="37"/>
+      <c r="D54" s="37"/>
+      <c r="E54" s="38"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B55" s="43">
+      <c r="B55" s="33">
         <v>46148</v>
       </c>
       <c r="C55" s="5">
@@ -1778,7 +1806,7 @@
       <c r="A56" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B56" s="38"/>
+      <c r="B56" s="34"/>
       <c r="C56" s="8">
         <v>35</v>
       </c>
@@ -1791,7 +1819,7 @@
       <c r="A57" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B57" s="38"/>
+      <c r="B57" s="34"/>
       <c r="C57" s="8">
         <v>60</v>
       </c>
@@ -1801,241 +1829,295 @@
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="7"/>
-      <c r="B58" s="38"/>
-      <c r="C58" s="8"/>
-      <c r="D58" s="9"/>
+      <c r="A58" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B58" s="34"/>
+      <c r="C58" s="8">
+        <v>60</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>94</v>
+      </c>
       <c r="E58" s="8"/>
     </row>
-    <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="10"/>
-      <c r="B59" s="39"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="11"/>
+    <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="B59" s="34"/>
+      <c r="C59" s="10">
+        <v>40</v>
+      </c>
+      <c r="D59" s="11" t="s">
+        <v>96</v>
+      </c>
       <c r="E59" s="10"/>
     </row>
-    <row r="60" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="12" t="s">
+    <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="B60" s="34"/>
+      <c r="C60" s="10">
+        <v>10</v>
+      </c>
+      <c r="D60" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="E60" s="10"/>
+    </row>
+    <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="28" t="s">
+        <v>98</v>
+      </c>
+      <c r="B61" s="34"/>
+      <c r="C61" s="10">
+        <v>20</v>
+      </c>
+      <c r="D61" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="E61" s="10"/>
+    </row>
+    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="B62" s="34"/>
+      <c r="C62" s="10">
+        <v>20</v>
+      </c>
+      <c r="D62" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="E62" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="10"/>
+      <c r="B63" s="35"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="11"/>
+      <c r="E63" s="10"/>
+    </row>
+    <row r="64" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B60" s="40"/>
-      <c r="C60" s="41"/>
-      <c r="D60" s="41"/>
-      <c r="E60" s="42"/>
-    </row>
-    <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="4"/>
-      <c r="B61" s="37"/>
-      <c r="C61" s="5"/>
-      <c r="D61" s="6"/>
-      <c r="E61" s="5"/>
-    </row>
-    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="7"/>
-      <c r="B62" s="38"/>
-      <c r="C62" s="8"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="8"/>
-    </row>
-    <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="7"/>
-      <c r="B63" s="38"/>
-      <c r="C63" s="8"/>
-      <c r="D63" s="9"/>
-      <c r="E63" s="8"/>
-    </row>
-    <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="7"/>
-      <c r="B64" s="38"/>
-      <c r="C64" s="8"/>
-      <c r="D64" s="9"/>
-      <c r="E64" s="8"/>
-    </row>
-    <row r="65" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="10"/>
-      <c r="B65" s="39"/>
-      <c r="C65" s="10"/>
-      <c r="D65" s="11"/>
-      <c r="E65" s="10"/>
-    </row>
-    <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B66" s="40"/>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="42"/>
+      <c r="B64" s="36" t="str">
+        <f>INT(SUM(C55:C63)/60)&amp;"h"&amp;MOD(SUM(C55:C63),60)</f>
+        <v>5h5</v>
+      </c>
+      <c r="C64" s="37"/>
+      <c r="D64" s="37"/>
+      <c r="E64" s="38"/>
+    </row>
+    <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="4"/>
+      <c r="B65" s="41"/>
+      <c r="C65" s="5"/>
+      <c r="D65" s="6"/>
+      <c r="E65" s="5"/>
+    </row>
+    <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="7"/>
+      <c r="B66" s="34"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="9"/>
+      <c r="E66" s="8"/>
     </row>
     <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="4"/>
-      <c r="B67" s="37"/>
-      <c r="C67" s="5"/>
-      <c r="D67" s="6"/>
-      <c r="E67" s="5"/>
+      <c r="A67" s="7"/>
+      <c r="B67" s="34"/>
+      <c r="C67" s="8"/>
+      <c r="D67" s="9"/>
+      <c r="E67" s="8"/>
     </row>
     <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7"/>
-      <c r="B68" s="38"/>
+      <c r="B68" s="34"/>
       <c r="C68" s="8"/>
       <c r="D68" s="9"/>
       <c r="E68" s="8"/>
     </row>
-    <row r="69" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="7"/>
-      <c r="B69" s="38"/>
-      <c r="C69" s="8"/>
-      <c r="D69" s="9"/>
-      <c r="E69" s="8"/>
-    </row>
-    <row r="70" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="7"/>
-      <c r="B70" s="38"/>
-      <c r="C70" s="8"/>
-      <c r="D70" s="9"/>
-      <c r="E70" s="8"/>
-    </row>
-    <row r="71" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="10"/>
-      <c r="B71" s="39"/>
-      <c r="C71" s="10"/>
-      <c r="D71" s="11"/>
-      <c r="E71" s="10"/>
-    </row>
-    <row r="72" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="12" t="s">
+    <row r="69" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="10"/>
+      <c r="B69" s="35"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="11"/>
+      <c r="E69" s="10"/>
+    </row>
+    <row r="70" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B72" s="40"/>
-      <c r="C72" s="41"/>
-      <c r="D72" s="41"/>
-      <c r="E72" s="42"/>
+      <c r="B70" s="36"/>
+      <c r="C70" s="37"/>
+      <c r="D70" s="37"/>
+      <c r="E70" s="38"/>
+    </row>
+    <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="4"/>
+      <c r="B71" s="41"/>
+      <c r="C71" s="5"/>
+      <c r="D71" s="6"/>
+      <c r="E71" s="5"/>
+    </row>
+    <row r="72" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="7"/>
+      <c r="B72" s="34"/>
+      <c r="C72" s="8"/>
+      <c r="D72" s="9"/>
+      <c r="E72" s="8"/>
     </row>
     <row r="73" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="4"/>
-      <c r="B73" s="37"/>
-      <c r="C73" s="5"/>
-      <c r="D73" s="6"/>
-      <c r="E73" s="5"/>
+      <c r="A73" s="7"/>
+      <c r="B73" s="34"/>
+      <c r="C73" s="8"/>
+      <c r="D73" s="9"/>
+      <c r="E73" s="8"/>
     </row>
     <row r="74" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="7"/>
-      <c r="B74" s="38"/>
+      <c r="B74" s="34"/>
       <c r="C74" s="8"/>
       <c r="D74" s="9"/>
       <c r="E74" s="8"/>
     </row>
-    <row r="75" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="7"/>
-      <c r="B75" s="38"/>
-      <c r="C75" s="8"/>
-      <c r="D75" s="9"/>
-      <c r="E75" s="8"/>
-    </row>
-    <row r="76" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="7"/>
-      <c r="B76" s="38"/>
-      <c r="C76" s="8"/>
-      <c r="D76" s="9"/>
-      <c r="E76" s="8"/>
-    </row>
-    <row r="77" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="10"/>
-      <c r="B77" s="39"/>
-      <c r="C77" s="10"/>
-      <c r="D77" s="11"/>
-      <c r="E77" s="10"/>
-    </row>
-    <row r="78" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="12" t="s">
+    <row r="75" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="10"/>
+      <c r="B75" s="35"/>
+      <c r="C75" s="10"/>
+      <c r="D75" s="11"/>
+      <c r="E75" s="10"/>
+    </row>
+    <row r="76" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B78" s="40"/>
-      <c r="C78" s="41"/>
-      <c r="D78" s="41"/>
-      <c r="E78" s="42"/>
+      <c r="B76" s="36"/>
+      <c r="C76" s="37"/>
+      <c r="D76" s="37"/>
+      <c r="E76" s="38"/>
+    </row>
+    <row r="77" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="4"/>
+      <c r="B77" s="41"/>
+      <c r="C77" s="5"/>
+      <c r="D77" s="6"/>
+      <c r="E77" s="5"/>
+    </row>
+    <row r="78" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="7"/>
+      <c r="B78" s="34"/>
+      <c r="C78" s="8"/>
+      <c r="D78" s="9"/>
+      <c r="E78" s="8"/>
     </row>
     <row r="79" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="13"/>
-      <c r="B79" s="37"/>
-      <c r="C79" s="13"/>
-      <c r="D79" s="14"/>
-      <c r="E79" s="13"/>
+      <c r="A79" s="7"/>
+      <c r="B79" s="34"/>
+      <c r="C79" s="8"/>
+      <c r="D79" s="9"/>
+      <c r="E79" s="8"/>
     </row>
     <row r="80" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="8"/>
-      <c r="B80" s="38"/>
+      <c r="A80" s="7"/>
+      <c r="B80" s="34"/>
       <c r="C80" s="8"/>
       <c r="D80" s="9"/>
       <c r="E80" s="8"/>
     </row>
-    <row r="81" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="8"/>
-      <c r="B81" s="38"/>
-      <c r="C81" s="8"/>
-      <c r="D81" s="9"/>
-      <c r="E81" s="8"/>
-    </row>
-    <row r="82" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="8"/>
-      <c r="B82" s="38"/>
-      <c r="C82" s="8"/>
-      <c r="D82" s="9"/>
-      <c r="E82" s="8"/>
-    </row>
-    <row r="83" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="8"/>
-      <c r="B83" s="39"/>
-      <c r="C83" s="8"/>
-      <c r="D83" s="9"/>
-      <c r="E83" s="8"/>
-    </row>
-    <row r="84" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="12" t="s">
+    <row r="81" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="10"/>
+      <c r="B81" s="35"/>
+      <c r="C81" s="10"/>
+      <c r="D81" s="11"/>
+      <c r="E81" s="10"/>
+    </row>
+    <row r="82" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="40"/>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="42"/>
-    </row>
-    <row r="85" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="44" t="s">
+      <c r="B82" s="36"/>
+      <c r="C82" s="37"/>
+      <c r="D82" s="37"/>
+      <c r="E82" s="38"/>
+    </row>
+    <row r="83" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="13"/>
+      <c r="B83" s="41"/>
+      <c r="C83" s="13"/>
+      <c r="D83" s="14"/>
+      <c r="E83" s="13"/>
+    </row>
+    <row r="84" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="8"/>
+      <c r="B84" s="34"/>
+      <c r="C84" s="8"/>
+      <c r="D84" s="9"/>
+      <c r="E84" s="8"/>
+    </row>
+    <row r="85" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="8"/>
+      <c r="B85" s="34"/>
+      <c r="C85" s="8"/>
+      <c r="D85" s="9"/>
+      <c r="E85" s="8"/>
+    </row>
+    <row r="86" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="8"/>
+      <c r="B86" s="34"/>
+      <c r="C86" s="8"/>
+      <c r="D86" s="9"/>
+      <c r="E86" s="8"/>
+    </row>
+    <row r="87" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="8"/>
+      <c r="B87" s="35"/>
+      <c r="C87" s="8"/>
+      <c r="D87" s="9"/>
+      <c r="E87" s="8"/>
+    </row>
+    <row r="88" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B88" s="36"/>
+      <c r="C88" s="37"/>
+      <c r="D88" s="37"/>
+      <c r="E88" s="38"/>
+    </row>
+    <row r="89" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B85" s="45"/>
-      <c r="C85" s="15">
-        <f>MROUND(SUM(C6:C84) /60,0.2)</f>
-        <v>30.8</v>
-      </c>
-      <c r="D85" s="16"/>
-      <c r="E85" s="17"/>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" s="18" t="s">
+      <c r="B89" s="40"/>
+      <c r="C89" s="15">
+        <f>MROUND(SUM(C6:C88) /60,0.2)</f>
+        <v>33.200000000000003</v>
+      </c>
+      <c r="D89" s="16"/>
+      <c r="E89" s="17"/>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" s="18"/>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B55:B59"/>
-    <mergeCell ref="B84:E84"/>
-    <mergeCell ref="A85:B85"/>
-    <mergeCell ref="B61:B65"/>
-    <mergeCell ref="B66:E66"/>
-    <mergeCell ref="B67:B71"/>
-    <mergeCell ref="B72:E72"/>
-    <mergeCell ref="B73:B77"/>
-    <mergeCell ref="B78:E78"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B79:B83"/>
-    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="B83:B87"/>
+    <mergeCell ref="B64:E64"/>
     <mergeCell ref="B6:B17"/>
     <mergeCell ref="B18:E18"/>
     <mergeCell ref="B19:B27"/>
@@ -2046,12 +2128,21 @@
     <mergeCell ref="B45:E45"/>
     <mergeCell ref="B46:B53"/>
     <mergeCell ref="B54:E54"/>
+    <mergeCell ref="B55:B63"/>
+    <mergeCell ref="B88:E88"/>
+    <mergeCell ref="A89:B89"/>
+    <mergeCell ref="B65:B69"/>
+    <mergeCell ref="B70:E70"/>
+    <mergeCell ref="B71:B75"/>
+    <mergeCell ref="B76:E76"/>
+    <mergeCell ref="B77:B81"/>
+    <mergeCell ref="B82:E82"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C73:C77 C67:C71 C55:C59 C61:C65 C29:C33 B6 C6:C17 C35:C44 C46:C53 C79:C83 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C77:C81 C71:C75 C55:C63 C65:C69 C29:C33 B6 C6:C17 C35:C44 C46:C53 C83:C87 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B59 B61:B65 B67:B71 B73:B77 B79:B83" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B63 B65:B69 B71:B75 B77:B81 B83:B87" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -2060,7 +2151,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="41" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="38" orientation="portrait" r:id="rId2"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -2222,6 +2313,12 @@
         <v>0.95138888888888884</v>
       </c>
     </row>
+    <row r="15" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="E15" s="26">
+        <f>E8-D8</f>
+        <v>0.17708333333333331</v>
+      </c>
+    </row>
     <row r="16" spans="3:9" x14ac:dyDescent="0.25">
       <c r="E16" s="26"/>
     </row>
@@ -2250,12 +2347,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -2417,6 +2508,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
@@ -2426,15 +2523,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2450,4 +2538,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(app): add delete for readers and nl
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B912D91-3B54-4537-BC72-B6ADD80FFB6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9C04C20-AC7E-4214-B355-4DB7EC6DC7EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="110">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -368,6 +368,21 @@
   </si>
   <si>
     <t>J'ai terminé la planification d'une campagne et jai commencé l'envoie mais j'ai pas encore temriné j'ai quelques soucis</t>
+  </si>
+  <si>
+    <t>J'ai fais quelques ajustement au niveau de l'app ou j'ai notament ajouté la possiblité de delete des campagne/lecteur (j'avais oublié de le faire)</t>
+  </si>
+  <si>
+    <t>Disccussion + ajustement</t>
+  </si>
+  <si>
+    <t>J'ai continué mes ajustement et j'ai notament discuté avec M. Melly histoire de faire un point de situation il m'a notament fais la remsrque de mettre de colone en plus dans la table de campagne et de laissé 30s de delais pour supprimer une campagne qui vient d'être envoyé</t>
+  </si>
+  <si>
+    <t>J'ai fait les ajustement voulu par M. Melly et j'ai aussi reglé quelques petit bugs et j'ai discuté concernant les 30s avant l'envoie et on en a conclu que je devais abondonner cette partie car le script ne me premet pas de une : connaitre la prochaine execution du script de deux, si au moment il veut supprimer ne pas excuter le script pour la campagne et la supprimer</t>
+  </si>
+  <si>
+    <t>discussion</t>
   </si>
 </sst>
 </file>
@@ -719,51 +734,51 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1097,10 +1112,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="33"/>
+      <c r="C1" s="42"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -1112,10 +1127,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="33"/>
+      <c r="C2" s="42"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -1127,10 +1142,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="33"/>
+      <c r="C3" s="42"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1142,12 +1157,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="36"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="45"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1170,7 +1185,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="43">
+      <c r="B6" s="33">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1183,7 +1198,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="38"/>
+      <c r="B7" s="34"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1196,7 +1211,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="38"/>
+      <c r="B8" s="34"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1209,7 +1224,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="38"/>
+      <c r="B9" s="34"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1220,7 +1235,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="38"/>
+      <c r="B10" s="34"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1233,7 +1248,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="38"/>
+      <c r="B11" s="34"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1248,7 +1263,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="34"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1263,7 +1278,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="38"/>
+      <c r="B13" s="34"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1278,7 +1293,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="38"/>
+      <c r="B14" s="34"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1293,7 +1308,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="38"/>
+      <c r="B15" s="34"/>
       <c r="C15" s="10">
         <v>40</v>
       </c>
@@ -1308,7 +1323,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="34"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1321,7 +1336,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="39"/>
+      <c r="B17" s="35"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1330,19 +1345,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="40" t="str">
+      <c r="B18" s="36" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C18" s="41"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="42"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="38"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="43">
+      <c r="B19" s="33">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1357,7 +1372,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="38"/>
+      <c r="B20" s="34"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1370,7 +1385,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="38"/>
+      <c r="B21" s="34"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1384,7 +1399,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="38"/>
+      <c r="B22" s="34"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1397,7 +1412,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="38"/>
+      <c r="B23" s="34"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1410,7 +1425,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="38"/>
+      <c r="B24" s="34"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1423,7 +1438,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="38"/>
+      <c r="B25" s="34"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1436,7 +1451,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="38"/>
+      <c r="B26" s="34"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1449,7 +1464,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="39"/>
+      <c r="B27" s="35"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1462,19 +1477,19 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="40" t="str">
+      <c r="B28" s="36" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="41"/>
-      <c r="D28" s="41"/>
-      <c r="E28" s="42"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="38"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="43">
+      <c r="B29" s="33">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1489,7 +1504,7 @@
       <c r="A30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="38"/>
+      <c r="B30" s="34"/>
       <c r="C30" s="8">
         <v>60</v>
       </c>
@@ -1504,7 +1519,7 @@
       <c r="A31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="38"/>
+      <c r="B31" s="34"/>
       <c r="C31" s="8">
         <v>70</v>
       </c>
@@ -1515,14 +1530,14 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="38"/>
+      <c r="B32" s="34"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="39"/>
+      <c r="B33" s="35"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1531,19 +1546,19 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="40" t="str">
+      <c r="B34" s="36" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C34" s="41"/>
-      <c r="D34" s="41"/>
-      <c r="E34" s="42"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="38"/>
     </row>
     <row r="35" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="43">
+      <c r="B35" s="33">
         <v>46143</v>
       </c>
       <c r="C35" s="5">
@@ -1558,7 +1573,7 @@
       <c r="A36" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="38"/>
+      <c r="B36" s="34"/>
       <c r="C36" s="8">
         <v>35</v>
       </c>
@@ -1571,7 +1586,7 @@
       <c r="A37" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="38"/>
+      <c r="B37" s="34"/>
       <c r="C37" s="8">
         <v>60</v>
       </c>
@@ -1584,7 +1599,7 @@
       <c r="A38" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="38"/>
+      <c r="B38" s="34"/>
       <c r="C38" s="8">
         <v>30</v>
       </c>
@@ -1597,7 +1612,7 @@
       <c r="A39" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="B39" s="38"/>
+      <c r="B39" s="34"/>
       <c r="C39" s="10">
         <v>35</v>
       </c>
@@ -1610,7 +1625,7 @@
       <c r="A40" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B40" s="38"/>
+      <c r="B40" s="34"/>
       <c r="C40" s="10">
         <v>20</v>
       </c>
@@ -1623,7 +1638,7 @@
       <c r="A41" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B41" s="38"/>
+      <c r="B41" s="34"/>
       <c r="C41" s="10">
         <v>50</v>
       </c>
@@ -1636,7 +1651,7 @@
       <c r="A42" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="38"/>
+      <c r="B42" s="34"/>
       <c r="C42" s="10">
         <v>45</v>
       </c>
@@ -1649,7 +1664,7 @@
       <c r="A43" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B43" s="38"/>
+      <c r="B43" s="34"/>
       <c r="C43" s="10">
         <v>60</v>
       </c>
@@ -1662,7 +1677,7 @@
       <c r="A44" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="39"/>
+      <c r="B44" s="35"/>
       <c r="C44" s="10">
         <v>35</v>
       </c>
@@ -1675,19 +1690,19 @@
       <c r="A45" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="40" t="str">
+      <c r="B45" s="36" t="str">
         <f>INT(SUM(C35:C44)/60)&amp;"h"&amp;MOD(SUM(C35:C44),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C45" s="41"/>
-      <c r="D45" s="41"/>
-      <c r="E45" s="42"/>
+      <c r="C45" s="37"/>
+      <c r="D45" s="37"/>
+      <c r="E45" s="38"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B46" s="43">
+      <c r="B46" s="33">
         <v>46146</v>
       </c>
       <c r="C46" s="13">
@@ -1702,7 +1717,7 @@
       <c r="A47" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B47" s="38"/>
+      <c r="B47" s="34"/>
       <c r="C47" s="8">
         <v>45</v>
       </c>
@@ -1715,7 +1730,7 @@
       <c r="A48" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="38"/>
+      <c r="B48" s="34"/>
       <c r="C48" s="8">
         <v>60</v>
       </c>
@@ -1728,7 +1743,7 @@
       <c r="A49" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B49" s="38"/>
+      <c r="B49" s="34"/>
       <c r="C49" s="8">
         <v>35</v>
       </c>
@@ -1741,7 +1756,7 @@
       <c r="A50" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B50" s="38"/>
+      <c r="B50" s="34"/>
       <c r="C50" s="8">
         <v>60</v>
       </c>
@@ -1754,7 +1769,7 @@
       <c r="A51" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B51" s="38"/>
+      <c r="B51" s="34"/>
       <c r="C51" s="8">
         <v>20</v>
       </c>
@@ -1767,7 +1782,7 @@
       <c r="A52" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B52" s="38"/>
+      <c r="B52" s="34"/>
       <c r="C52" s="8">
         <v>50</v>
       </c>
@@ -1778,7 +1793,7 @@
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="8"/>
-      <c r="B53" s="39"/>
+      <c r="B53" s="35"/>
       <c r="C53" s="8"/>
       <c r="D53" s="32"/>
       <c r="E53" s="31"/>
@@ -1787,19 +1802,19 @@
       <c r="A54" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B54" s="40" t="str">
+      <c r="B54" s="36" t="str">
         <f>INT(SUM(C46:C53)/60)&amp;"h"&amp;MOD(SUM(C46:C53),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C54" s="41"/>
-      <c r="D54" s="41"/>
-      <c r="E54" s="42"/>
+      <c r="C54" s="37"/>
+      <c r="D54" s="37"/>
+      <c r="E54" s="38"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B55" s="43">
+      <c r="B55" s="33">
         <v>46148</v>
       </c>
       <c r="C55" s="5">
@@ -1814,7 +1829,7 @@
       <c r="A56" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B56" s="38"/>
+      <c r="B56" s="34"/>
       <c r="C56" s="8">
         <v>35</v>
       </c>
@@ -1827,7 +1842,7 @@
       <c r="A57" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B57" s="38"/>
+      <c r="B57" s="34"/>
       <c r="C57" s="8">
         <v>60</v>
       </c>
@@ -1840,7 +1855,7 @@
       <c r="A58" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B58" s="38"/>
+      <c r="B58" s="34"/>
       <c r="C58" s="8">
         <v>60</v>
       </c>
@@ -1853,7 +1868,7 @@
       <c r="A59" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B59" s="38"/>
+      <c r="B59" s="34"/>
       <c r="C59" s="10">
         <v>40</v>
       </c>
@@ -1866,7 +1881,7 @@
       <c r="A60" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B60" s="38"/>
+      <c r="B60" s="34"/>
       <c r="C60" s="10">
         <v>10</v>
       </c>
@@ -1879,7 +1894,7 @@
       <c r="A61" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="B61" s="38"/>
+      <c r="B61" s="34"/>
       <c r="C61" s="10">
         <v>20</v>
       </c>
@@ -1892,7 +1907,7 @@
       <c r="A62" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B62" s="38"/>
+      <c r="B62" s="34"/>
       <c r="C62" s="10">
         <v>20</v>
       </c>
@@ -1905,7 +1920,7 @@
       <c r="A63" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="B63" s="38"/>
+      <c r="B63" s="34"/>
       <c r="C63" s="10">
         <v>35</v>
       </c>
@@ -1920,7 +1935,7 @@
       <c r="A64" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B64" s="38"/>
+      <c r="B64" s="34"/>
       <c r="C64" s="10">
         <v>45</v>
       </c>
@@ -1933,7 +1948,7 @@
       <c r="A65" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B65" s="38"/>
+      <c r="B65" s="34"/>
       <c r="C65" s="10">
         <v>45</v>
       </c>
@@ -1944,7 +1959,7 @@
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="39"/>
+      <c r="B66" s="35"/>
       <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="10"/>
@@ -1953,45 +1968,65 @@
       <c r="A67" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B67" s="40" t="str">
+      <c r="B67" s="36" t="str">
         <f>INT(SUM(C55:C66)/60)&amp;"h"&amp;MOD(SUM(C55:C66),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C67" s="41"/>
-      <c r="D67" s="41"/>
-      <c r="E67" s="42"/>
-    </row>
-    <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="4"/>
-      <c r="B68" s="37"/>
-      <c r="C68" s="5"/>
-      <c r="D68" s="6"/>
+      <c r="C67" s="37"/>
+      <c r="D67" s="37"/>
+      <c r="E67" s="38"/>
+    </row>
+    <row r="68" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A68" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B68" s="33">
+        <v>46149</v>
+      </c>
+      <c r="C68" s="5">
+        <v>60</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>105</v>
+      </c>
       <c r="E68" s="5"/>
     </row>
-    <row r="69" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="7"/>
-      <c r="B69" s="38"/>
-      <c r="C69" s="8"/>
-      <c r="D69" s="9"/>
+    <row r="69" spans="1:5" ht="54" x14ac:dyDescent="0.25">
+      <c r="A69" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B69" s="34"/>
+      <c r="C69" s="8">
+        <v>60</v>
+      </c>
+      <c r="D69" s="9" t="s">
+        <v>107</v>
+      </c>
       <c r="E69" s="8"/>
     </row>
-    <row r="70" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="7"/>
-      <c r="B70" s="38"/>
-      <c r="C70" s="8"/>
-      <c r="D70" s="9"/>
+    <row r="70" spans="1:5" ht="67.5" x14ac:dyDescent="0.25">
+      <c r="A70" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B70" s="34"/>
+      <c r="C70" s="8">
+        <v>55</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>108</v>
+      </c>
       <c r="E70" s="8"/>
     </row>
     <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="7"/>
-      <c r="B71" s="38"/>
+      <c r="B71" s="34"/>
       <c r="C71" s="8"/>
       <c r="D71" s="9"/>
       <c r="E71" s="8"/>
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="10"/>
-      <c r="B72" s="39"/>
+      <c r="B72" s="35"/>
       <c r="C72" s="10"/>
       <c r="D72" s="11"/>
       <c r="E72" s="10"/>
@@ -2000,42 +2035,45 @@
       <c r="A73" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B73" s="40"/>
-      <c r="C73" s="41"/>
-      <c r="D73" s="41"/>
-      <c r="E73" s="42"/>
+      <c r="B73" s="36" t="str">
+        <f>INT(SUM(C68:C72)/60)&amp;"h"&amp;MOD(SUM(C68:C72),60)</f>
+        <v>2h55</v>
+      </c>
+      <c r="C73" s="37"/>
+      <c r="D73" s="37"/>
+      <c r="E73" s="38"/>
     </row>
     <row r="74" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="4"/>
-      <c r="B74" s="37"/>
+      <c r="B74" s="41"/>
       <c r="C74" s="5"/>
       <c r="D74" s="6"/>
       <c r="E74" s="5"/>
     </row>
     <row r="75" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="7"/>
-      <c r="B75" s="38"/>
+      <c r="B75" s="34"/>
       <c r="C75" s="8"/>
       <c r="D75" s="9"/>
       <c r="E75" s="8"/>
     </row>
     <row r="76" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="7"/>
-      <c r="B76" s="38"/>
+      <c r="B76" s="34"/>
       <c r="C76" s="8"/>
       <c r="D76" s="9"/>
       <c r="E76" s="8"/>
     </row>
     <row r="77" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
-      <c r="B77" s="38"/>
+      <c r="B77" s="34"/>
       <c r="C77" s="8"/>
       <c r="D77" s="9"/>
       <c r="E77" s="8"/>
     </row>
     <row r="78" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="10"/>
-      <c r="B78" s="39"/>
+      <c r="B78" s="35"/>
       <c r="C78" s="10"/>
       <c r="D78" s="11"/>
       <c r="E78" s="10"/>
@@ -2044,42 +2082,42 @@
       <c r="A79" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B79" s="40"/>
-      <c r="C79" s="41"/>
-      <c r="D79" s="41"/>
-      <c r="E79" s="42"/>
+      <c r="B79" s="36"/>
+      <c r="C79" s="37"/>
+      <c r="D79" s="37"/>
+      <c r="E79" s="38"/>
     </row>
     <row r="80" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="4"/>
-      <c r="B80" s="37"/>
+      <c r="B80" s="41"/>
       <c r="C80" s="5"/>
       <c r="D80" s="6"/>
       <c r="E80" s="5"/>
     </row>
     <row r="81" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="7"/>
-      <c r="B81" s="38"/>
+      <c r="B81" s="34"/>
       <c r="C81" s="8"/>
       <c r="D81" s="9"/>
       <c r="E81" s="8"/>
     </row>
     <row r="82" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="7"/>
-      <c r="B82" s="38"/>
+      <c r="B82" s="34"/>
       <c r="C82" s="8"/>
       <c r="D82" s="9"/>
       <c r="E82" s="8"/>
     </row>
     <row r="83" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="7"/>
-      <c r="B83" s="38"/>
+      <c r="B83" s="34"/>
       <c r="C83" s="8"/>
       <c r="D83" s="9"/>
       <c r="E83" s="8"/>
     </row>
     <row r="84" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="10"/>
-      <c r="B84" s="39"/>
+      <c r="B84" s="35"/>
       <c r="C84" s="10"/>
       <c r="D84" s="11"/>
       <c r="E84" s="10"/>
@@ -2088,42 +2126,42 @@
       <c r="A85" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B85" s="40"/>
-      <c r="C85" s="41"/>
-      <c r="D85" s="41"/>
-      <c r="E85" s="42"/>
+      <c r="B85" s="36"/>
+      <c r="C85" s="37"/>
+      <c r="D85" s="37"/>
+      <c r="E85" s="38"/>
     </row>
     <row r="86" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="13"/>
-      <c r="B86" s="37"/>
+      <c r="B86" s="41"/>
       <c r="C86" s="13"/>
       <c r="D86" s="14"/>
       <c r="E86" s="13"/>
     </row>
     <row r="87" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="8"/>
-      <c r="B87" s="38"/>
+      <c r="B87" s="34"/>
       <c r="C87" s="8"/>
       <c r="D87" s="9"/>
       <c r="E87" s="8"/>
     </row>
     <row r="88" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="8"/>
-      <c r="B88" s="38"/>
+      <c r="B88" s="34"/>
       <c r="C88" s="8"/>
       <c r="D88" s="9"/>
       <c r="E88" s="8"/>
     </row>
     <row r="89" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="8"/>
-      <c r="B89" s="38"/>
+      <c r="B89" s="34"/>
       <c r="C89" s="8"/>
       <c r="D89" s="9"/>
       <c r="E89" s="8"/>
     </row>
     <row r="90" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="8"/>
-      <c r="B90" s="39"/>
+      <c r="B90" s="35"/>
       <c r="C90" s="8"/>
       <c r="D90" s="9"/>
       <c r="E90" s="8"/>
@@ -2132,19 +2170,19 @@
       <c r="A91" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B91" s="40"/>
-      <c r="C91" s="41"/>
-      <c r="D91" s="41"/>
-      <c r="E91" s="42"/>
+      <c r="B91" s="36"/>
+      <c r="C91" s="37"/>
+      <c r="D91" s="37"/>
+      <c r="E91" s="38"/>
     </row>
     <row r="92" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="44" t="s">
+      <c r="A92" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B92" s="45"/>
+      <c r="B92" s="40"/>
       <c r="C92" s="15">
         <f>MROUND(SUM(C6:C91) /60,0.2)</f>
-        <v>35.4</v>
+        <v>38.200000000000003</v>
       </c>
       <c r="D92" s="16"/>
       <c r="E92" s="17"/>
@@ -2159,15 +2197,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B55:B66"/>
-    <mergeCell ref="B91:E91"/>
-    <mergeCell ref="A92:B92"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B74:B78"/>
-    <mergeCell ref="B79:E79"/>
-    <mergeCell ref="B80:B84"/>
-    <mergeCell ref="B85:E85"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -2184,6 +2213,15 @@
     <mergeCell ref="B45:E45"/>
     <mergeCell ref="B46:B53"/>
     <mergeCell ref="B54:E54"/>
+    <mergeCell ref="B55:B66"/>
+    <mergeCell ref="B91:E91"/>
+    <mergeCell ref="A92:B92"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="B74:B78"/>
+    <mergeCell ref="B79:E79"/>
+    <mergeCell ref="B80:B84"/>
+    <mergeCell ref="B85:E85"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C80:C84 C74:C78 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C86:C90 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -2198,7 +2236,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="37" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="35" orientation="portrait" r:id="rId2"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -2394,12 +2432,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -2561,6 +2593,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
@@ -2570,15 +2608,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2594,4 +2623,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor(nl): change send nl system (set nl as scheduled for 5min later)
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F780C81-320D-41B9-81AB-FEACCD80F181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6897C2D-9B27-4E49-81EB-12E9CDA696D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="111">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -383,6 +383,9 @@
   </si>
   <si>
     <t>J'ai fait les ajustement voulu (colone en plus pour le nombre d'envoi et de click) par M. Melly et j'ai aussi reglé quelques petit bugs et j'ai discuté concernant les 30s avant l'envoie et on en a conclu que je devais abondonner cette partie car le script ne me premet pas de une : connaitre précisement la prochaine execution du script de deux, si au moment il veut supprimer ne pas excuter le script pour la campagne et la supprimer</t>
+  </si>
+  <si>
+    <t>J'ai un peu avancer sur mon rapport</t>
   </si>
 </sst>
 </file>
@@ -2018,10 +2021,16 @@
       <c r="E70" s="8"/>
     </row>
     <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="7"/>
+      <c r="A71" s="7" t="s">
+        <v>38</v>
+      </c>
       <c r="B71" s="34"/>
-      <c r="C71" s="8"/>
-      <c r="D71" s="9"/>
+      <c r="C71" s="8">
+        <v>15</v>
+      </c>
+      <c r="D71" s="9" t="s">
+        <v>110</v>
+      </c>
       <c r="E71" s="8"/>
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2037,7 +2046,7 @@
       </c>
       <c r="B73" s="36" t="str">
         <f>INT(SUM(C68:C72)/60)&amp;"h"&amp;MOD(SUM(C68:C72),60)</f>
-        <v>2h55</v>
+        <v>3h10</v>
       </c>
       <c r="C73" s="37"/>
       <c r="D73" s="37"/>
@@ -2182,7 +2191,7 @@
       <c r="B92" s="40"/>
       <c r="C92" s="15">
         <f>MROUND(SUM(C6:C91) /60,0.2)</f>
-        <v>38.200000000000003</v>
+        <v>38.6</v>
       </c>
       <c r="D92" s="16"/>
       <c r="E92" s="17"/>

</xml_diff>

<commit_message>
chore(app): add dev https and update project repport
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0468706-0A23-41BB-8988-265AC781181C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FA50091-E9B2-47F6-934D-8C765A73E3C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$97</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$98</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="124">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -413,6 +413,18 @@
   </si>
   <si>
     <t>"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai fait une petite relecture </t>
+  </si>
+  <si>
+    <t>Système de renvoi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai commencé le système de renvoi si une campagne est échouée </t>
+  </si>
+  <si>
+    <t>J'ai commencé la rédaction de la conclusion du rapport</t>
   </si>
 </sst>
 </file>
@@ -1126,7 +1138,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G100"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -2199,7 +2211,9 @@
       <c r="E82" s="10"/>
     </row>
     <row r="83" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="10"/>
+      <c r="A83" s="10" t="s">
+        <v>38</v>
+      </c>
       <c r="B83" s="35"/>
       <c r="C83" s="10">
         <v>10</v>
@@ -2222,62 +2236,95 @@
       <c r="E84" s="38"/>
     </row>
     <row r="85" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="4"/>
+      <c r="A85" s="4" t="s">
+        <v>38</v>
+      </c>
       <c r="B85" s="41"/>
-      <c r="C85" s="5"/>
-      <c r="D85" s="6"/>
+      <c r="C85" s="5">
+        <v>20</v>
+      </c>
+      <c r="D85" s="6" t="s">
+        <v>120</v>
+      </c>
       <c r="E85" s="5"/>
     </row>
     <row r="86" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="7"/>
+      <c r="A86" s="7" t="s">
+        <v>121</v>
+      </c>
       <c r="B86" s="34"/>
-      <c r="C86" s="8"/>
-      <c r="D86" s="9"/>
+      <c r="C86" s="8">
+        <v>40</v>
+      </c>
+      <c r="D86" s="9" t="s">
+        <v>122</v>
+      </c>
       <c r="E86" s="8"/>
     </row>
     <row r="87" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="7"/>
+      <c r="A87" s="7" t="s">
+        <v>38</v>
+      </c>
       <c r="B87" s="34"/>
-      <c r="C87" s="8"/>
-      <c r="D87" s="9"/>
+      <c r="C87" s="8">
+        <v>60</v>
+      </c>
+      <c r="D87" s="9" t="s">
+        <v>123</v>
+      </c>
       <c r="E87" s="8"/>
     </row>
     <row r="88" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="7"/>
+      <c r="A88" s="7" t="s">
+        <v>38</v>
+      </c>
       <c r="B88" s="34"/>
-      <c r="C88" s="8"/>
-      <c r="D88" s="9"/>
+      <c r="C88" s="8">
+        <v>60</v>
+      </c>
+      <c r="D88" s="9" t="s">
+        <v>113</v>
+      </c>
       <c r="E88" s="8"/>
     </row>
-    <row r="89" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="10"/>
-      <c r="B89" s="35"/>
-      <c r="C89" s="10"/>
-      <c r="D89" s="11"/>
+    <row r="89" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B89" s="34"/>
+      <c r="C89" s="10">
+        <v>10</v>
+      </c>
+      <c r="D89" s="11" t="s">
+        <v>119</v>
+      </c>
       <c r="E89" s="10"/>
     </row>
     <row r="90" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="12" t="s">
+      <c r="A90" s="10"/>
+      <c r="B90" s="35"/>
+      <c r="C90" s="10"/>
+      <c r="D90" s="11"/>
+      <c r="E90" s="10"/>
+    </row>
+    <row r="91" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B90" s="36"/>
-      <c r="C90" s="37"/>
-      <c r="D90" s="37"/>
-      <c r="E90" s="38"/>
-    </row>
-    <row r="91" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="13"/>
-      <c r="B91" s="41"/>
-      <c r="C91" s="13"/>
-      <c r="D91" s="14"/>
-      <c r="E91" s="13"/>
+      <c r="B91" s="36" t="str">
+        <f>INT(SUM(C85:C90)/60)&amp;"h"&amp;MOD(SUM(C85:C90),60)</f>
+        <v>3h10</v>
+      </c>
+      <c r="C91" s="37"/>
+      <c r="D91" s="37"/>
+      <c r="E91" s="38"/>
     </row>
     <row r="92" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="8"/>
-      <c r="B92" s="34"/>
-      <c r="C92" s="8"/>
-      <c r="D92" s="9"/>
-      <c r="E92" s="8"/>
+      <c r="A92" s="13"/>
+      <c r="B92" s="41"/>
+      <c r="C92" s="13"/>
+      <c r="D92" s="14"/>
+      <c r="E92" s="13"/>
     </row>
     <row r="93" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="8"/>
@@ -2293,41 +2340,48 @@
       <c r="D94" s="9"/>
       <c r="E94" s="8"/>
     </row>
-    <row r="95" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="8"/>
-      <c r="B95" s="35"/>
+      <c r="B95" s="34"/>
       <c r="C95" s="8"/>
       <c r="D95" s="9"/>
       <c r="E95" s="8"/>
     </row>
     <row r="96" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="12" t="s">
+      <c r="A96" s="8"/>
+      <c r="B96" s="35"/>
+      <c r="C96" s="8"/>
+      <c r="D96" s="9"/>
+      <c r="E96" s="8"/>
+    </row>
+    <row r="97" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B96" s="36"/>
-      <c r="C96" s="37"/>
-      <c r="D96" s="37"/>
-      <c r="E96" s="38"/>
-    </row>
-    <row r="97" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="39" t="s">
+      <c r="B97" s="36"/>
+      <c r="C97" s="37"/>
+      <c r="D97" s="37"/>
+      <c r="E97" s="38"/>
+    </row>
+    <row r="98" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B97" s="40"/>
-      <c r="C97" s="15">
-        <f>MROUND(SUM(C6:C96) /60,0.2)</f>
-        <v>45.6</v>
-      </c>
-      <c r="D97" s="16"/>
-      <c r="E97" s="17"/>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A99" s="18" t="s">
+      <c r="B98" s="40"/>
+      <c r="C98" s="15">
+        <f>MROUND(SUM(C6:C97) /60,0.2)</f>
+        <v>48.800000000000004</v>
+      </c>
+      <c r="D98" s="16"/>
+      <c r="E98" s="17"/>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" s="18"/>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="25">
@@ -2335,7 +2389,7 @@
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B91:B95"/>
+    <mergeCell ref="B92:B96"/>
     <mergeCell ref="B67:E67"/>
     <mergeCell ref="B6:B17"/>
     <mergeCell ref="B18:E18"/>
@@ -2348,20 +2402,20 @@
     <mergeCell ref="B46:B53"/>
     <mergeCell ref="B54:E54"/>
     <mergeCell ref="B55:B66"/>
-    <mergeCell ref="B96:E96"/>
-    <mergeCell ref="A97:B97"/>
+    <mergeCell ref="B97:E97"/>
+    <mergeCell ref="A98:B98"/>
     <mergeCell ref="B68:B72"/>
     <mergeCell ref="B73:E73"/>
     <mergeCell ref="B74:B83"/>
     <mergeCell ref="B84:E84"/>
-    <mergeCell ref="B85:B89"/>
-    <mergeCell ref="B90:E90"/>
+    <mergeCell ref="B85:B90"/>
+    <mergeCell ref="B91:E91"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C89 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C91:C95 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C90 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C92:C96 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B89 B91:B95" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B90 B92:B96" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -2370,7 +2424,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="34" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="32" orientation="portrait" r:id="rId2"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -2534,8 +2588,8 @@
     </row>
     <row r="15" spans="3:9" x14ac:dyDescent="0.25">
       <c r="E15" s="26">
-        <f>E8-D8</f>
-        <v>0.17708333333333331</v>
+        <f>E6-D6-(H6/2)</f>
+        <v>0.13194444444444445</v>
       </c>
     </row>
     <row r="16" spans="3:9" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
refactor(doc): update project repport
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FA50091-E9B2-47F6-934D-8C765A73E3C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D853128-8E5C-41C4-B925-ACE7E7217720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$98</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$100</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="126">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -425,6 +425,12 @@
   </si>
   <si>
     <t>J'ai commencé la rédaction de la conclusion du rapport</t>
+  </si>
+  <si>
+    <t>J'ai terminé la partie 1 du rapport</t>
+  </si>
+  <si>
+    <t>J'ai commencé la partie 2 du rapport j'ai notament fais la partie de l'installation du projet</t>
   </si>
 </sst>
 </file>
@@ -776,51 +782,51 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1138,7 +1144,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -1154,10 +1160,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="42"/>
+      <c r="C1" s="33"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -1169,10 +1175,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="42"/>
+      <c r="C2" s="33"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -1184,10 +1190,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="42"/>
+      <c r="C3" s="33"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1199,12 +1205,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="43" t="s">
+      <c r="B4" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="45"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="36"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1227,7 +1233,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="33">
+      <c r="B6" s="43">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1240,7 +1246,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="34"/>
+      <c r="B7" s="38"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1253,7 +1259,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="34"/>
+      <c r="B8" s="38"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1266,7 +1272,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="34"/>
+      <c r="B9" s="38"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1277,7 +1283,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="34"/>
+      <c r="B10" s="38"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1290,7 +1296,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="34"/>
+      <c r="B11" s="38"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1305,7 +1311,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="34"/>
+      <c r="B12" s="38"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1320,7 +1326,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="34"/>
+      <c r="B13" s="38"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1335,7 +1341,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="34"/>
+      <c r="B14" s="38"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1350,7 +1356,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="34"/>
+      <c r="B15" s="38"/>
       <c r="C15" s="10">
         <v>40</v>
       </c>
@@ -1365,7 +1371,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="34"/>
+      <c r="B16" s="38"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1378,7 +1384,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="35"/>
+      <c r="B17" s="39"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1387,19 +1393,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="36" t="str">
+      <c r="B18" s="40" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="38"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="42"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="33">
+      <c r="B19" s="43">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1414,7 +1420,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="34"/>
+      <c r="B20" s="38"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1427,7 +1433,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="34"/>
+      <c r="B21" s="38"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1441,7 +1447,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="34"/>
+      <c r="B22" s="38"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1454,7 +1460,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="34"/>
+      <c r="B23" s="38"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1467,7 +1473,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="34"/>
+      <c r="B24" s="38"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1480,7 +1486,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="34"/>
+      <c r="B25" s="38"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1493,7 +1499,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="34"/>
+      <c r="B26" s="38"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1506,7 +1512,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="35"/>
+      <c r="B27" s="39"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1519,19 +1525,19 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="36" t="str">
+      <c r="B28" s="40" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="37"/>
-      <c r="D28" s="37"/>
-      <c r="E28" s="38"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="42"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="33">
+      <c r="B29" s="43">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1546,7 +1552,7 @@
       <c r="A30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="34"/>
+      <c r="B30" s="38"/>
       <c r="C30" s="8">
         <v>60</v>
       </c>
@@ -1561,7 +1567,7 @@
       <c r="A31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="34"/>
+      <c r="B31" s="38"/>
       <c r="C31" s="8">
         <v>70</v>
       </c>
@@ -1572,14 +1578,14 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="34"/>
+      <c r="B32" s="38"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="35"/>
+      <c r="B33" s="39"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1588,19 +1594,19 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="36" t="str">
+      <c r="B34" s="40" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C34" s="37"/>
-      <c r="D34" s="37"/>
-      <c r="E34" s="38"/>
+      <c r="C34" s="41"/>
+      <c r="D34" s="41"/>
+      <c r="E34" s="42"/>
     </row>
     <row r="35" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="33">
+      <c r="B35" s="43">
         <v>46143</v>
       </c>
       <c r="C35" s="5">
@@ -1615,7 +1621,7 @@
       <c r="A36" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="34"/>
+      <c r="B36" s="38"/>
       <c r="C36" s="8">
         <v>35</v>
       </c>
@@ -1628,7 +1634,7 @@
       <c r="A37" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="34"/>
+      <c r="B37" s="38"/>
       <c r="C37" s="8">
         <v>60</v>
       </c>
@@ -1641,7 +1647,7 @@
       <c r="A38" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="34"/>
+      <c r="B38" s="38"/>
       <c r="C38" s="8">
         <v>30</v>
       </c>
@@ -1654,7 +1660,7 @@
       <c r="A39" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="B39" s="34"/>
+      <c r="B39" s="38"/>
       <c r="C39" s="10">
         <v>35</v>
       </c>
@@ -1667,7 +1673,7 @@
       <c r="A40" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B40" s="34"/>
+      <c r="B40" s="38"/>
       <c r="C40" s="10">
         <v>20</v>
       </c>
@@ -1680,7 +1686,7 @@
       <c r="A41" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B41" s="34"/>
+      <c r="B41" s="38"/>
       <c r="C41" s="10">
         <v>50</v>
       </c>
@@ -1693,7 +1699,7 @@
       <c r="A42" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="34"/>
+      <c r="B42" s="38"/>
       <c r="C42" s="10">
         <v>45</v>
       </c>
@@ -1706,7 +1712,7 @@
       <c r="A43" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B43" s="34"/>
+      <c r="B43" s="38"/>
       <c r="C43" s="10">
         <v>60</v>
       </c>
@@ -1719,7 +1725,7 @@
       <c r="A44" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="35"/>
+      <c r="B44" s="39"/>
       <c r="C44" s="10">
         <v>35</v>
       </c>
@@ -1732,19 +1738,19 @@
       <c r="A45" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="36" t="str">
+      <c r="B45" s="40" t="str">
         <f>INT(SUM(C35:C44)/60)&amp;"h"&amp;MOD(SUM(C35:C44),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C45" s="37"/>
-      <c r="D45" s="37"/>
-      <c r="E45" s="38"/>
+      <c r="C45" s="41"/>
+      <c r="D45" s="41"/>
+      <c r="E45" s="42"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B46" s="33">
+      <c r="B46" s="43">
         <v>46146</v>
       </c>
       <c r="C46" s="13">
@@ -1759,7 +1765,7 @@
       <c r="A47" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B47" s="34"/>
+      <c r="B47" s="38"/>
       <c r="C47" s="8">
         <v>45</v>
       </c>
@@ -1772,7 +1778,7 @@
       <c r="A48" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="34"/>
+      <c r="B48" s="38"/>
       <c r="C48" s="8">
         <v>60</v>
       </c>
@@ -1785,7 +1791,7 @@
       <c r="A49" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B49" s="34"/>
+      <c r="B49" s="38"/>
       <c r="C49" s="8">
         <v>35</v>
       </c>
@@ -1798,7 +1804,7 @@
       <c r="A50" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B50" s="34"/>
+      <c r="B50" s="38"/>
       <c r="C50" s="8">
         <v>60</v>
       </c>
@@ -1811,7 +1817,7 @@
       <c r="A51" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B51" s="34"/>
+      <c r="B51" s="38"/>
       <c r="C51" s="8">
         <v>20</v>
       </c>
@@ -1824,7 +1830,7 @@
       <c r="A52" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B52" s="34"/>
+      <c r="B52" s="38"/>
       <c r="C52" s="8">
         <v>50</v>
       </c>
@@ -1835,7 +1841,7 @@
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="8"/>
-      <c r="B53" s="35"/>
+      <c r="B53" s="39"/>
       <c r="C53" s="8"/>
       <c r="D53" s="32"/>
       <c r="E53" s="31"/>
@@ -1844,19 +1850,19 @@
       <c r="A54" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B54" s="36" t="str">
+      <c r="B54" s="40" t="str">
         <f>INT(SUM(C46:C53)/60)&amp;"h"&amp;MOD(SUM(C46:C53),60)</f>
         <v>5h20</v>
       </c>
-      <c r="C54" s="37"/>
-      <c r="D54" s="37"/>
-      <c r="E54" s="38"/>
+      <c r="C54" s="41"/>
+      <c r="D54" s="41"/>
+      <c r="E54" s="42"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B55" s="33">
+      <c r="B55" s="43">
         <v>46148</v>
       </c>
       <c r="C55" s="5">
@@ -1871,7 +1877,7 @@
       <c r="A56" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B56" s="34"/>
+      <c r="B56" s="38"/>
       <c r="C56" s="8">
         <v>35</v>
       </c>
@@ -1884,7 +1890,7 @@
       <c r="A57" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B57" s="34"/>
+      <c r="B57" s="38"/>
       <c r="C57" s="8">
         <v>60</v>
       </c>
@@ -1897,7 +1903,7 @@
       <c r="A58" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B58" s="34"/>
+      <c r="B58" s="38"/>
       <c r="C58" s="8">
         <v>60</v>
       </c>
@@ -1910,7 +1916,7 @@
       <c r="A59" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B59" s="34"/>
+      <c r="B59" s="38"/>
       <c r="C59" s="10">
         <v>40</v>
       </c>
@@ -1923,7 +1929,7 @@
       <c r="A60" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B60" s="34"/>
+      <c r="B60" s="38"/>
       <c r="C60" s="10">
         <v>10</v>
       </c>
@@ -1936,7 +1942,7 @@
       <c r="A61" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="B61" s="34"/>
+      <c r="B61" s="38"/>
       <c r="C61" s="10">
         <v>20</v>
       </c>
@@ -1949,7 +1955,7 @@
       <c r="A62" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B62" s="34"/>
+      <c r="B62" s="38"/>
       <c r="C62" s="10">
         <v>20</v>
       </c>
@@ -1962,7 +1968,7 @@
       <c r="A63" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="B63" s="34"/>
+      <c r="B63" s="38"/>
       <c r="C63" s="10">
         <v>35</v>
       </c>
@@ -1977,7 +1983,7 @@
       <c r="A64" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B64" s="34"/>
+      <c r="B64" s="38"/>
       <c r="C64" s="10">
         <v>45</v>
       </c>
@@ -1990,7 +1996,7 @@
       <c r="A65" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B65" s="34"/>
+      <c r="B65" s="38"/>
       <c r="C65" s="10">
         <v>45</v>
       </c>
@@ -2001,7 +2007,7 @@
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="35"/>
+      <c r="B66" s="39"/>
       <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="10"/>
@@ -2010,19 +2016,19 @@
       <c r="A67" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B67" s="36" t="str">
+      <c r="B67" s="40" t="str">
         <f>INT(SUM(C55:C66)/60)&amp;"h"&amp;MOD(SUM(C55:C66),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C67" s="37"/>
-      <c r="D67" s="37"/>
-      <c r="E67" s="38"/>
+      <c r="C67" s="41"/>
+      <c r="D67" s="41"/>
+      <c r="E67" s="42"/>
     </row>
     <row r="68" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B68" s="33">
+      <c r="B68" s="43">
         <v>46149</v>
       </c>
       <c r="C68" s="5">
@@ -2037,7 +2043,7 @@
       <c r="A69" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B69" s="34"/>
+      <c r="B69" s="38"/>
       <c r="C69" s="8">
         <v>60</v>
       </c>
@@ -2050,7 +2056,7 @@
       <c r="A70" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B70" s="34"/>
+      <c r="B70" s="38"/>
       <c r="C70" s="8">
         <v>55</v>
       </c>
@@ -2063,7 +2069,7 @@
       <c r="A71" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B71" s="34"/>
+      <c r="B71" s="38"/>
       <c r="C71" s="8">
         <v>15</v>
       </c>
@@ -2074,7 +2080,7 @@
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="10"/>
-      <c r="B72" s="35"/>
+      <c r="B72" s="39"/>
       <c r="C72" s="10"/>
       <c r="D72" s="11"/>
       <c r="E72" s="10"/>
@@ -2083,19 +2089,19 @@
       <c r="A73" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B73" s="36" t="str">
+      <c r="B73" s="40" t="str">
         <f>INT(SUM(C68:C72)/60)&amp;"h"&amp;MOD(SUM(C68:C72),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C73" s="37"/>
-      <c r="D73" s="37"/>
-      <c r="E73" s="38"/>
+      <c r="C73" s="41"/>
+      <c r="D73" s="41"/>
+      <c r="E73" s="42"/>
     </row>
     <row r="74" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B74" s="33">
+      <c r="B74" s="43">
         <v>46150</v>
       </c>
       <c r="C74" s="5">
@@ -2110,7 +2116,7 @@
       <c r="A75" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B75" s="34"/>
+      <c r="B75" s="38"/>
       <c r="C75" s="8">
         <v>50</v>
       </c>
@@ -2123,7 +2129,7 @@
       <c r="A76" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B76" s="34"/>
+      <c r="B76" s="38"/>
       <c r="C76" s="8">
         <v>35</v>
       </c>
@@ -2136,7 +2142,7 @@
       <c r="A77" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="B77" s="34"/>
+      <c r="B77" s="38"/>
       <c r="C77" s="8">
         <v>60</v>
       </c>
@@ -2149,7 +2155,7 @@
       <c r="A78" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="B78" s="34"/>
+      <c r="B78" s="38"/>
       <c r="C78" s="10">
         <v>60</v>
       </c>
@@ -2162,7 +2168,7 @@
       <c r="A79" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B79" s="34"/>
+      <c r="B79" s="38"/>
       <c r="C79" s="10">
         <v>25</v>
       </c>
@@ -2175,7 +2181,7 @@
       <c r="A80" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B80" s="34"/>
+      <c r="B80" s="38"/>
       <c r="C80" s="10">
         <v>60</v>
       </c>
@@ -2188,7 +2194,7 @@
       <c r="A81" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B81" s="34"/>
+      <c r="B81" s="38"/>
       <c r="C81" s="10">
         <v>60</v>
       </c>
@@ -2201,7 +2207,7 @@
       <c r="A82" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B82" s="34"/>
+      <c r="B82" s="38"/>
       <c r="C82" s="10">
         <v>60</v>
       </c>
@@ -2214,7 +2220,7 @@
       <c r="A83" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B83" s="35"/>
+      <c r="B83" s="39"/>
       <c r="C83" s="10">
         <v>10</v>
       </c>
@@ -2227,19 +2233,21 @@
       <c r="A84" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="36" t="str">
+      <c r="B84" s="40" t="str">
         <f>INT(SUM(C74:C83)/60)&amp;"h"&amp;MOD(SUM(C74:C83),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C84" s="37"/>
-      <c r="D84" s="37"/>
-      <c r="E84" s="38"/>
+      <c r="C84" s="41"/>
+      <c r="D84" s="41"/>
+      <c r="E84" s="42"/>
     </row>
     <row r="85" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B85" s="41"/>
+      <c r="B85" s="43">
+        <v>46153</v>
+      </c>
       <c r="C85" s="5">
         <v>20</v>
       </c>
@@ -2252,7 +2260,7 @@
       <c r="A86" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="B86" s="34"/>
+      <c r="B86" s="38"/>
       <c r="C86" s="8">
         <v>40</v>
       </c>
@@ -2265,7 +2273,7 @@
       <c r="A87" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B87" s="34"/>
+      <c r="B87" s="38"/>
       <c r="C87" s="8">
         <v>60</v>
       </c>
@@ -2278,7 +2286,7 @@
       <c r="A88" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B88" s="34"/>
+      <c r="B88" s="38"/>
       <c r="C88" s="8">
         <v>60</v>
       </c>
@@ -2291,7 +2299,7 @@
       <c r="A89" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B89" s="34"/>
+      <c r="B89" s="38"/>
       <c r="C89" s="10">
         <v>10</v>
       </c>
@@ -2300,96 +2308,137 @@
       </c>
       <c r="E89" s="10"/>
     </row>
-    <row r="90" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="10"/>
-      <c r="B90" s="35"/>
-      <c r="C90" s="10"/>
-      <c r="D90" s="11"/>
+    <row r="90" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B90" s="38"/>
+      <c r="C90" s="10">
+        <v>60</v>
+      </c>
+      <c r="D90" s="11" t="s">
+        <v>124</v>
+      </c>
       <c r="E90" s="10"/>
     </row>
-    <row r="91" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="12" t="s">
+    <row r="91" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A91" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B91" s="38"/>
+      <c r="C91" s="10">
+        <v>60</v>
+      </c>
+      <c r="D91" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="E91" s="10"/>
+    </row>
+    <row r="92" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B92" s="39"/>
+      <c r="C92" s="10">
+        <v>10</v>
+      </c>
+      <c r="D92" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E92" s="10"/>
+    </row>
+    <row r="93" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B91" s="36" t="str">
-        <f>INT(SUM(C85:C90)/60)&amp;"h"&amp;MOD(SUM(C85:C90),60)</f>
-        <v>3h10</v>
-      </c>
-      <c r="C91" s="37"/>
-      <c r="D91" s="37"/>
-      <c r="E91" s="38"/>
-    </row>
-    <row r="92" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="13"/>
-      <c r="B92" s="41"/>
-      <c r="C92" s="13"/>
-      <c r="D92" s="14"/>
-      <c r="E92" s="13"/>
-    </row>
-    <row r="93" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="8"/>
-      <c r="B93" s="34"/>
-      <c r="C93" s="8"/>
-      <c r="D93" s="9"/>
-      <c r="E93" s="8"/>
+      <c r="B93" s="40" t="str">
+        <f>INT(SUM(C85:C92)/60)&amp;"h"&amp;MOD(SUM(C85:C92),60)</f>
+        <v>5h20</v>
+      </c>
+      <c r="C93" s="41"/>
+      <c r="D93" s="41"/>
+      <c r="E93" s="42"/>
     </row>
     <row r="94" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="8"/>
-      <c r="B94" s="34"/>
-      <c r="C94" s="8"/>
-      <c r="D94" s="9"/>
-      <c r="E94" s="8"/>
+      <c r="A94" s="13"/>
+      <c r="B94" s="37"/>
+      <c r="C94" s="13"/>
+      <c r="D94" s="14"/>
+      <c r="E94" s="13"/>
     </row>
     <row r="95" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="8"/>
-      <c r="B95" s="34"/>
+      <c r="B95" s="38"/>
       <c r="C95" s="8"/>
       <c r="D95" s="9"/>
       <c r="E95" s="8"/>
     </row>
-    <row r="96" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="8"/>
-      <c r="B96" s="35"/>
+      <c r="B96" s="38"/>
       <c r="C96" s="8"/>
       <c r="D96" s="9"/>
       <c r="E96" s="8"/>
     </row>
-    <row r="97" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="12" t="s">
+    <row r="97" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="8"/>
+      <c r="B97" s="38"/>
+      <c r="C97" s="8"/>
+      <c r="D97" s="9"/>
+      <c r="E97" s="8"/>
+    </row>
+    <row r="98" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="8"/>
+      <c r="B98" s="39"/>
+      <c r="C98" s="8"/>
+      <c r="D98" s="9"/>
+      <c r="E98" s="8"/>
+    </row>
+    <row r="99" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B97" s="36"/>
-      <c r="C97" s="37"/>
-      <c r="D97" s="37"/>
-      <c r="E97" s="38"/>
-    </row>
-    <row r="98" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="39" t="s">
+      <c r="B99" s="40"/>
+      <c r="C99" s="41"/>
+      <c r="D99" s="41"/>
+      <c r="E99" s="42"/>
+    </row>
+    <row r="100" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="B98" s="40"/>
-      <c r="C98" s="15">
-        <f>MROUND(SUM(C6:C97) /60,0.2)</f>
-        <v>48.800000000000004</v>
-      </c>
-      <c r="D98" s="16"/>
-      <c r="E98" s="17"/>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" s="18" t="s">
+      <c r="B100" s="45"/>
+      <c r="C100" s="15">
+        <f>MROUND(SUM(C6:C99) /60,0.2)</f>
+        <v>51</v>
+      </c>
+      <c r="D100" s="16"/>
+      <c r="E100" s="17"/>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A101" s="18"/>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B55:B66"/>
+    <mergeCell ref="B99:E99"/>
+    <mergeCell ref="A100:B100"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="B74:B83"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="B85:B92"/>
+    <mergeCell ref="B93:E93"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B92:B96"/>
+    <mergeCell ref="B94:B98"/>
     <mergeCell ref="B67:E67"/>
     <mergeCell ref="B6:B17"/>
     <mergeCell ref="B18:E18"/>
@@ -2401,21 +2450,12 @@
     <mergeCell ref="B45:E45"/>
     <mergeCell ref="B46:B53"/>
     <mergeCell ref="B54:E54"/>
-    <mergeCell ref="B55:B66"/>
-    <mergeCell ref="B97:E97"/>
-    <mergeCell ref="A98:B98"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B74:B83"/>
-    <mergeCell ref="B84:E84"/>
-    <mergeCell ref="B85:B90"/>
-    <mergeCell ref="B91:E91"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C90 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C92:C96 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C92 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C94:C98 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B90 B92:B96" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B92 B94:B98" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -2620,6 +2660,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -2781,12 +2827,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
@@ -2796,6 +2836,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2811,13 +2860,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor, fix(global): correct an error in privacy policy, update  project repport, fix change status bug
</commit_message>
<xml_diff>
--- a/Doc/m-planification-jnltrav_heures_2023.xlsx
+++ b/Doc/m-planification-jnltrav_heures_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D853128-8E5C-41C4-B925-ACE7E7217720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE6FDBA-3837-4A75-9573-6C57461749E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$100</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$104</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="133">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -431,6 +431,27 @@
   </si>
   <si>
     <t>J'ai commencé la partie 2 du rapport j'ai notament fais la partie de l'installation du projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai continué mon rapport j'ai notament commencé la partie documentation utilisateur et j'ai résumé le mandat </t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai commencé l'analyse critique mais j'ai un doute car dans ma conclusion je  parle déjà des points forts et faible de mon application  ducoup je ne sais pas si je fais un chapitre à part ou j'intègre ca dans la conclusion </t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai continué l'analyse critique sur l'api mail vs smtp maintant je vais vais expliquer la configuration DNS </t>
+  </si>
+  <si>
+    <t>J'ai continué la partie configuration DNS si je prends autant de temps c'est parce que en parallèle que j'ecris j'essaie de me renseigner les plus possible pour évité de dire des choses fausses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai terminé la partie analyse </t>
+  </si>
+  <si>
+    <t>J'ai principalement fait de la remise en forme  mais j'ai aussi continué le résumé</t>
+  </si>
+  <si>
+    <t>16h10</t>
   </si>
 </sst>
 </file>
@@ -670,7 +691,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -794,7 +815,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -816,10 +837,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1144,7 +1161,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G103"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -1233,7 +1250,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="43">
+      <c r="B6" s="37">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1405,7 +1422,7 @@
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="43">
+      <c r="B19" s="37">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1537,7 +1554,7 @@
       <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="43">
+      <c r="B29" s="37">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1606,7 +1623,7 @@
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="43">
+      <c r="B35" s="37">
         <v>46143</v>
       </c>
       <c r="C35" s="5">
@@ -1750,7 +1767,7 @@
       <c r="A46" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B46" s="43">
+      <c r="B46" s="37">
         <v>46146</v>
       </c>
       <c r="C46" s="13">
@@ -1862,7 +1879,7 @@
       <c r="A55" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B55" s="43">
+      <c r="B55" s="37">
         <v>46148</v>
       </c>
       <c r="C55" s="5">
@@ -2028,7 +2045,7 @@
       <c r="A68" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B68" s="43">
+      <c r="B68" s="37">
         <v>46149</v>
       </c>
       <c r="C68" s="5">
@@ -2101,7 +2118,7 @@
       <c r="A74" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B74" s="43">
+      <c r="B74" s="37">
         <v>46150</v>
       </c>
       <c r="C74" s="5">
@@ -2245,7 +2262,7 @@
       <c r="A85" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B85" s="43">
+      <c r="B85" s="37">
         <v>46153</v>
       </c>
       <c r="C85" s="5">
@@ -2359,75 +2376,164 @@
       <c r="D93" s="41"/>
       <c r="E93" s="42"/>
     </row>
-    <row r="94" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="13"/>
-      <c r="B94" s="37"/>
-      <c r="C94" s="13"/>
-      <c r="D94" s="14"/>
+    <row r="94" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A94" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B94" s="37">
+        <v>46155</v>
+      </c>
+      <c r="C94" s="13">
+        <v>60</v>
+      </c>
+      <c r="D94" s="14" t="s">
+        <v>126</v>
+      </c>
       <c r="E94" s="13"/>
     </row>
     <row r="95" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="8"/>
+      <c r="A95" s="8" t="s">
+        <v>38</v>
+      </c>
       <c r="B95" s="38"/>
-      <c r="C95" s="8"/>
-      <c r="D95" s="9"/>
+      <c r="C95" s="8">
+        <v>35</v>
+      </c>
+      <c r="D95" s="9" t="s">
+        <v>113</v>
+      </c>
       <c r="E95" s="8"/>
     </row>
-    <row r="96" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="8"/>
+    <row r="96" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A96" s="8" t="s">
+        <v>38</v>
+      </c>
       <c r="B96" s="38"/>
-      <c r="C96" s="8"/>
-      <c r="D96" s="9"/>
+      <c r="C96" s="8">
+        <v>60</v>
+      </c>
+      <c r="D96" s="9" t="s">
+        <v>127</v>
+      </c>
       <c r="E96" s="8"/>
     </row>
-    <row r="97" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="8"/>
+    <row r="97" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A97" s="8" t="s">
+        <v>38</v>
+      </c>
       <c r="B97" s="38"/>
-      <c r="C97" s="8"/>
-      <c r="D97" s="9"/>
+      <c r="C97" s="8">
+        <v>60</v>
+      </c>
+      <c r="D97" s="9" t="s">
+        <v>128</v>
+      </c>
       <c r="E97" s="8"/>
     </row>
-    <row r="98" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="8"/>
-      <c r="B98" s="39"/>
-      <c r="C98" s="8"/>
-      <c r="D98" s="9"/>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B98" s="38"/>
+      <c r="C98" s="8">
+        <v>25</v>
+      </c>
+      <c r="D98" s="9" t="s">
+        <v>113</v>
+      </c>
       <c r="E98" s="8"/>
     </row>
-    <row r="99" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="12" t="s">
+    <row r="99" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A99" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B99" s="38"/>
+      <c r="C99" s="8">
+        <v>60</v>
+      </c>
+      <c r="D99" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="E99" s="8"/>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B100" s="38"/>
+      <c r="C100" s="8">
+        <v>45</v>
+      </c>
+      <c r="D100" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E100" s="8"/>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B101" s="38"/>
+      <c r="C101" s="8">
+        <v>60</v>
+      </c>
+      <c r="D101" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="E101" s="8" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B102" s="39"/>
+      <c r="C102" s="8">
+        <v>25</v>
+      </c>
+      <c r="D102" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E102" s="8"/>
+    </row>
+    <row r="103" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B99" s="40"/>
-      <c r="C99" s="41"/>
-      <c r="D99" s="41"/>
-      <c r="E99" s="42"/>
-    </row>
-    <row r="100" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="44" t="s">
+      <c r="B103" s="40" t="str">
+        <f>INT(SUM(C94:C102)/60)&amp;"h"&amp;MOD(SUM(C94:C102),60)</f>
+        <v>7h10</v>
+      </c>
+      <c r="C103" s="41"/>
+      <c r="D103" s="41"/>
+      <c r="E103" s="42"/>
+    </row>
+    <row r="104" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="B100" s="45"/>
-      <c r="C100" s="15">
-        <f>MROUND(SUM(C6:C99) /60,0.2)</f>
-        <v>51</v>
-      </c>
-      <c r="D100" s="16"/>
-      <c r="E100" s="17"/>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="18" t="s">
+      <c r="B104" s="44"/>
+      <c r="C104" s="15">
+        <f>MROUND(SUM(C6:C103) /60,0.2)</f>
+        <v>58.2</v>
+      </c>
+      <c r="D104" s="16"/>
+      <c r="E104" s="17"/>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="18"/>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="25">
     <mergeCell ref="B55:B66"/>
-    <mergeCell ref="B99:E99"/>
-    <mergeCell ref="A100:B100"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="A104:B104"/>
     <mergeCell ref="B68:B72"/>
     <mergeCell ref="B73:E73"/>
     <mergeCell ref="B74:B83"/>
@@ -2438,7 +2544,7 @@
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B94:B98"/>
+    <mergeCell ref="B94:B102"/>
     <mergeCell ref="B67:E67"/>
     <mergeCell ref="B6:B17"/>
     <mergeCell ref="B18:E18"/>
@@ -2452,10 +2558,10 @@
     <mergeCell ref="B54:E54"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C92 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C94:C98 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C92 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C94:C102 C19:C27" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B92 B94:B98" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B92 B94:B102" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -2464,7 +2570,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="32" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="30" orientation="portrait" r:id="rId2"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -2475,164 +2581,165 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E348320A-3DEF-4FFB-92B3-3073BCAD0028}">
-  <dimension ref="C5:I33"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5703125" customWidth="1"/>
     <col min="9" max="9" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
         <v>21</v>
       </c>
-      <c r="E5" t="s">
+      <c r="C1" t="s">
         <v>22</v>
       </c>
-      <c r="F5" t="s">
+      <c r="D1" t="s">
         <v>23</v>
       </c>
-      <c r="G5" t="s">
+      <c r="E1" t="s">
         <v>24</v>
       </c>
-      <c r="H5" t="s">
+      <c r="F1" t="s">
         <v>25</v>
       </c>
-      <c r="I5" t="s">
+      <c r="G1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C6" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>27</v>
       </c>
+      <c r="B2" s="26">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C2" s="26">
+        <v>0.47569444444444442</v>
+      </c>
+      <c r="D2" s="26">
+        <v>0.51388888888888884</v>
+      </c>
+      <c r="E2" s="26">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="F2" s="26">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="G2" s="26">
+        <v>0.22222222222222221</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="26">
+        <v>0</v>
+      </c>
+      <c r="C3" s="26">
+        <v>0</v>
+      </c>
+      <c r="D3" s="26">
+        <v>0</v>
+      </c>
+      <c r="E3" s="26">
+        <v>0</v>
+      </c>
+      <c r="F3" s="26">
+        <v>0</v>
+      </c>
+      <c r="G3" s="26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="26">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C4" s="26">
+        <v>0.51041666666666663</v>
+      </c>
+      <c r="D4" s="26">
+        <v>0.54861111111111116</v>
+      </c>
+      <c r="E4" s="26">
+        <v>0.69097222222222221</v>
+      </c>
+      <c r="F4" s="26">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="G4" s="26">
+        <v>0.2986111111111111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="26">
+        <v>0</v>
+      </c>
+      <c r="C5" s="26">
+        <v>0</v>
+      </c>
+      <c r="D5" s="26">
+        <v>0.54861111111111116</v>
+      </c>
+      <c r="E5" s="26">
+        <v>0.69097222222222221</v>
+      </c>
+      <c r="F5" s="26">
+        <v>1.0416666666666666E-2</v>
+      </c>
+      <c r="G5" s="26">
+        <f>E5-D5-F5</f>
+        <v>0.13194444444444439</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="26">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C6" s="26">
+        <v>0.51041666666666663</v>
+      </c>
       <c r="D6" s="26">
-        <v>0.33333333333333331</v>
+        <v>0.54861111111111116</v>
       </c>
       <c r="E6" s="26">
-        <v>0.47569444444444442</v>
+        <v>0.69097222222222221</v>
       </c>
       <c r="F6" s="26">
-        <v>0.51388888888888884</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="G6" s="26">
-        <v>0.61458333333333337</v>
-      </c>
-      <c r="H6" s="26">
-        <v>2.0833333333333332E-2</v>
-      </c>
-      <c r="I6" s="26">
-        <v>0.22222222222222221</v>
-      </c>
-    </row>
-    <row r="7" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="26">
-        <v>0</v>
-      </c>
-      <c r="E7" s="26">
-        <v>0</v>
-      </c>
-      <c r="F7" s="26">
-        <v>0</v>
-      </c>
-      <c r="G7" s="26">
-        <v>0</v>
-      </c>
-      <c r="H7" s="26">
-        <v>0</v>
-      </c>
-      <c r="I7" s="26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C8" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="26">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="E8" s="26">
-        <v>0.51041666666666663</v>
-      </c>
-      <c r="F8" s="26">
-        <v>0.54861111111111116</v>
+        <v>0.2986111111111111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F8" t="s">
+        <v>32</v>
       </c>
       <c r="G8" s="26">
-        <v>0.69097222222222221</v>
-      </c>
-      <c r="H8" s="26">
-        <v>2.0833333333333332E-2</v>
-      </c>
-      <c r="I8" s="26">
-        <v>0.2986111111111111</v>
-      </c>
-    </row>
-    <row r="9" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C9" t="s">
-        <v>30</v>
-      </c>
-      <c r="D9" s="26">
-        <v>0</v>
-      </c>
-      <c r="E9" s="26">
-        <v>0</v>
-      </c>
-      <c r="F9" s="26">
-        <v>0.54861111111111116</v>
-      </c>
-      <c r="G9" s="26">
-        <v>0.69097222222222221</v>
-      </c>
-      <c r="H9" s="26">
-        <v>1.0416666666666666E-2</v>
-      </c>
-      <c r="I9" s="26">
-        <f>G9-F9-H9</f>
-        <v>0.13194444444444439</v>
-      </c>
-    </row>
-    <row r="10" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C10" t="s">
-        <v>31</v>
-      </c>
-      <c r="D10" s="26">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="E10" s="26">
-        <v>0.51041666666666663</v>
-      </c>
-      <c r="F10" s="26">
-        <v>0.54861111111111116</v>
-      </c>
-      <c r="G10" s="26">
-        <v>0.69097222222222221</v>
-      </c>
-      <c r="H10" s="26">
-        <v>2.0833333333333332E-2</v>
-      </c>
-      <c r="I10" s="26">
-        <v>0.2986111111111111</v>
-      </c>
-    </row>
-    <row r="12" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="H12" t="s">
-        <v>32</v>
-      </c>
-      <c r="I12" s="26">
         <v>0.95138888888888884</v>
       </c>
     </row>
-    <row r="15" spans="3:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E15" s="26">
-        <f>E6-D6-(H6/2)</f>
-        <v>0.13194444444444445</v>
-      </c>
-    </row>
-    <row r="16" spans="3:9" x14ac:dyDescent="0.25">
+        <f>C6-B6-(F6/2)</f>
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E16" s="26"/>
     </row>
     <row r="19" spans="5:5" x14ac:dyDescent="0.25">

</xml_diff>